<commit_message>
Recoleccion de predicciones corriendo collect_predictions.py tras centrelizacion de data
</commit_message>
<xml_diff>
--- a/data/england/p6_deployment/data_preparation/df_constructed.xlsx
+++ b/data/england/p6_deployment/data_preparation/df_constructed.xlsx
@@ -525,94 +525,94 @@
       </c>
       <c r="T1" s="1" t="inlineStr">
         <is>
+          <t>dif_mean_last_match_goal_attempts</t>
+        </is>
+      </c>
+      <c r="U1" s="1" t="inlineStr">
+        <is>
+          <t>dif_mean_last_match_goal_attempts_against</t>
+        </is>
+      </c>
+      <c r="V1" s="1" t="inlineStr">
+        <is>
+          <t>dif_mean_last_match_interceptions</t>
+        </is>
+      </c>
+      <c r="W1" s="1" t="inlineStr">
+        <is>
+          <t>dif_mean_last_match_interceptions_against</t>
+        </is>
+      </c>
+      <c r="X1" s="1" t="inlineStr">
+        <is>
+          <t>dif_mean_last_match_points</t>
+        </is>
+      </c>
+      <c r="Y1" s="1" t="inlineStr">
+        <is>
+          <t>dif_mean_last_match_points_against</t>
+        </is>
+      </c>
+      <c r="Z1" s="1" t="inlineStr">
+        <is>
+          <t>dif_mean_last_match_fouls</t>
+        </is>
+      </c>
+      <c r="AA1" s="1" t="inlineStr">
+        <is>
+          <t>dif_mean_last_match_fouls_against</t>
+        </is>
+      </c>
+      <c r="AB1" s="1" t="inlineStr">
+        <is>
+          <t>dif_mean_last_match_shots_on_goal</t>
+        </is>
+      </c>
+      <c r="AC1" s="1" t="inlineStr">
+        <is>
+          <t>dif_mean_last_match_shots_on_goal_against</t>
+        </is>
+      </c>
+      <c r="AD1" s="1" t="inlineStr">
+        <is>
+          <t>dif_mean_last_match_n_matches_last_days</t>
+        </is>
+      </c>
+      <c r="AE1" s="1" t="inlineStr">
+        <is>
+          <t>dif_mean_last_match_n_matches_last_days_against</t>
+        </is>
+      </c>
+      <c r="AF1" s="1" t="inlineStr">
+        <is>
           <t>dif_mean_last_match_goals</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="AG1" s="1" t="inlineStr">
         <is>
           <t>dif_mean_last_match_goals_against</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="AH1" s="1" t="inlineStr">
         <is>
           <t>dif_mean_last_match_ball_possession</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="AI1" s="1" t="inlineStr">
         <is>
           <t>dif_mean_last_match_ball_possession_against</t>
         </is>
       </c>
-      <c r="X1" s="1" t="inlineStr">
-        <is>
-          <t>dif_mean_last_match_fouls</t>
-        </is>
-      </c>
-      <c r="Y1" s="1" t="inlineStr">
-        <is>
-          <t>dif_mean_last_match_fouls_against</t>
-        </is>
-      </c>
-      <c r="Z1" s="1" t="inlineStr">
-        <is>
-          <t>dif_mean_last_match_goal_attempts</t>
-        </is>
-      </c>
-      <c r="AA1" s="1" t="inlineStr">
-        <is>
-          <t>dif_mean_last_match_goal_attempts_against</t>
-        </is>
-      </c>
-      <c r="AB1" s="1" t="inlineStr">
-        <is>
-          <t>dif_mean_last_match_n_matches_last_days</t>
-        </is>
-      </c>
-      <c r="AC1" s="1" t="inlineStr">
-        <is>
-          <t>dif_mean_last_match_n_matches_last_days_against</t>
-        </is>
-      </c>
-      <c r="AD1" s="1" t="inlineStr">
+      <c r="AJ1" s="1" t="inlineStr">
         <is>
           <t>dif_mean_last_match_expected_goals_(xg)</t>
         </is>
       </c>
-      <c r="AE1" s="1" t="inlineStr">
+      <c r="AK1" s="1" t="inlineStr">
         <is>
           <t>dif_mean_last_match_expected_goals_(xg)_against</t>
         </is>
       </c>
-      <c r="AF1" s="1" t="inlineStr">
-        <is>
-          <t>dif_mean_last_match_interceptions</t>
-        </is>
-      </c>
-      <c r="AG1" s="1" t="inlineStr">
-        <is>
-          <t>dif_mean_last_match_interceptions_against</t>
-        </is>
-      </c>
-      <c r="AH1" s="1" t="inlineStr">
-        <is>
-          <t>dif_mean_last_match_shots_on_goal</t>
-        </is>
-      </c>
-      <c r="AI1" s="1" t="inlineStr">
-        <is>
-          <t>dif_mean_last_match_shots_on_goal_against</t>
-        </is>
-      </c>
-      <c r="AJ1" s="1" t="inlineStr">
-        <is>
-          <t>dif_mean_last_match_points</t>
-        </is>
-      </c>
-      <c r="AK1" s="1" t="inlineStr">
-        <is>
-          <t>dif_mean_last_match_points_against</t>
-        </is>
-      </c>
       <c r="AL1" s="1" t="inlineStr">
         <is>
           <t>mean_last_match_mean_rat_player_start_home_against</t>
@@ -625,97 +625,97 @@
       </c>
       <c r="AN1" s="1" t="inlineStr">
         <is>
+          <t>dif_n_player_miss</t>
+        </is>
+      </c>
+      <c r="AO1" s="1" t="inlineStr">
+        <is>
+          <t>dif_mean_val_player_start</t>
+        </is>
+      </c>
+      <c r="AP1" s="1" t="inlineStr">
+        <is>
+          <t>dif_sum_rat_player_miss</t>
+        </is>
+      </c>
+      <c r="AQ1" s="1" t="inlineStr">
+        <is>
+          <t>dif_mean_age_player_sub</t>
+        </is>
+      </c>
+      <c r="AR1" s="1" t="inlineStr">
+        <is>
+          <t>dif_mean_int_rep_player_miss</t>
+        </is>
+      </c>
+      <c r="AS1" s="1" t="inlineStr">
+        <is>
+          <t>dif_mean_age_player_start</t>
+        </is>
+      </c>
+      <c r="AT1" s="1" t="inlineStr">
+        <is>
+          <t>dif_mean_rat_player_sub</t>
+        </is>
+      </c>
+      <c r="AU1" s="1" t="inlineStr">
+        <is>
+          <t>dif_mean_pot_player_start</t>
+        </is>
+      </c>
+      <c r="AV1" s="1" t="inlineStr">
+        <is>
+          <t>dif_mean_hei_player_sub</t>
+        </is>
+      </c>
+      <c r="AW1" s="1" t="inlineStr">
+        <is>
+          <t>dif_mean_val_player_sub</t>
+        </is>
+      </c>
+      <c r="AX1" s="1" t="inlineStr">
+        <is>
+          <t>dif_mean_pot_player_sub</t>
+        </is>
+      </c>
+      <c r="AY1" s="1" t="inlineStr">
+        <is>
           <t>dif_mean_rat_player_start</t>
         </is>
       </c>
-      <c r="AO1" s="1" t="inlineStr">
-        <is>
-          <t>dif_n_player_miss</t>
-        </is>
-      </c>
-      <c r="AP1" s="1" t="inlineStr">
-        <is>
-          <t>dif_mean_hei_player_sub</t>
-        </is>
-      </c>
-      <c r="AQ1" s="1" t="inlineStr">
-        <is>
-          <t>dif_mean_pot_player_sub</t>
-        </is>
-      </c>
-      <c r="AR1" s="1" t="inlineStr">
-        <is>
-          <t>dif_mean_val_player_sub</t>
-        </is>
-      </c>
-      <c r="AS1" s="1" t="inlineStr">
-        <is>
-          <t>dif_mean_val_player_start</t>
-        </is>
-      </c>
-      <c r="AT1" s="1" t="inlineStr">
+      <c r="AZ1" s="1" t="inlineStr">
+        <is>
+          <t>dif_sum_pot_player_miss</t>
+        </is>
+      </c>
+      <c r="BA1" s="1" t="inlineStr">
+        <is>
+          <t>dif_sum_val_player_miss</t>
+        </is>
+      </c>
+      <c r="BB1" s="1" t="inlineStr">
+        <is>
+          <t>dif_mean_hei_player_start</t>
+        </is>
+      </c>
+      <c r="BC1" s="1" t="inlineStr">
+        <is>
+          <t>dif_mean_age_player_miss</t>
+        </is>
+      </c>
+      <c r="BD1" s="1" t="inlineStr">
         <is>
           <t>dif_mean_int_rep_player_sub</t>
         </is>
       </c>
-      <c r="AU1" s="1" t="inlineStr">
+      <c r="BE1" s="1" t="inlineStr">
         <is>
           <t>dif_mean_int_rep_player_start</t>
         </is>
       </c>
-      <c r="AV1" s="1" t="inlineStr">
-        <is>
-          <t>dif_sum_pot_player_miss</t>
-        </is>
-      </c>
-      <c r="AW1" s="1" t="inlineStr">
-        <is>
-          <t>dif_mean_int_rep_player_miss</t>
-        </is>
-      </c>
-      <c r="AX1" s="1" t="inlineStr">
-        <is>
-          <t>dif_mean_hei_player_start</t>
-        </is>
-      </c>
-      <c r="AY1" s="1" t="inlineStr">
-        <is>
-          <t>dif_mean_age_player_start</t>
-        </is>
-      </c>
-      <c r="AZ1" s="1" t="inlineStr">
-        <is>
-          <t>dif_mean_age_player_miss</t>
-        </is>
-      </c>
-      <c r="BA1" s="1" t="inlineStr">
-        <is>
-          <t>dif_mean_pot_player_start</t>
-        </is>
-      </c>
-      <c r="BB1" s="1" t="inlineStr">
-        <is>
-          <t>dif_sum_rat_player_miss</t>
-        </is>
-      </c>
-      <c r="BC1" s="1" t="inlineStr">
+      <c r="BF1" s="1" t="inlineStr">
         <is>
           <t>dif_mean_hei_player_miss</t>
-        </is>
-      </c>
-      <c r="BD1" s="1" t="inlineStr">
-        <is>
-          <t>dif_sum_val_player_miss</t>
-        </is>
-      </c>
-      <c r="BE1" s="1" t="inlineStr">
-        <is>
-          <t>dif_mean_rat_player_sub</t>
-        </is>
-      </c>
-      <c r="BF1" s="1" t="inlineStr">
-        <is>
-          <t>dif_mean_age_player_sub</t>
         </is>
       </c>
       <c r="BG1" s="1" t="inlineStr">
@@ -803,54 +803,54 @@
         <v>0</v>
       </c>
       <c r="T2" t="n">
+        <v>-0.5</v>
+      </c>
+      <c r="U2" t="n">
+        <v>-7.666666666666666</v>
+      </c>
+      <c r="V2" t="inlineStr"/>
+      <c r="W2" t="inlineStr"/>
+      <c r="X2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="Y2" t="n">
+        <v>-0.5</v>
+      </c>
+      <c r="Z2" t="n">
+        <v>0.1666666666666661</v>
+      </c>
+      <c r="AA2" t="n">
+        <v>-5.333333333333334</v>
+      </c>
+      <c r="AB2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AC2" t="n">
+        <v>-5.333333333333333</v>
+      </c>
+      <c r="AD2" t="n">
+        <v>0.333333333333333</v>
+      </c>
+      <c r="AE2" t="n">
+        <v>-1.666666666666667</v>
+      </c>
+      <c r="AF2" t="n">
         <v>0.8333333333333333</v>
       </c>
-      <c r="U2" t="n">
+      <c r="AG2" t="n">
         <v>-1</v>
       </c>
-      <c r="V2" t="n">
+      <c r="AH2" t="n">
         <v>-10.5</v>
       </c>
-      <c r="W2" t="n">
+      <c r="AI2" t="n">
         <v>10.5</v>
       </c>
-      <c r="X2" t="n">
-        <v>0.1666666666666661</v>
-      </c>
-      <c r="Y2" t="n">
-        <v>-5.333333333333334</v>
-      </c>
-      <c r="Z2" t="n">
-        <v>-0.5</v>
-      </c>
-      <c r="AA2" t="n">
-        <v>-7.666666666666666</v>
-      </c>
-      <c r="AB2" t="n">
-        <v>0.333333333333333</v>
-      </c>
-      <c r="AC2" t="n">
-        <v>-1.666666666666667</v>
-      </c>
-      <c r="AD2" t="n">
+      <c r="AJ2" t="n">
         <v>-0.7333333333333329</v>
       </c>
-      <c r="AE2" t="n">
+      <c r="AK2" t="n">
         <v>-0.8333333333333335</v>
-      </c>
-      <c r="AF2" t="inlineStr"/>
-      <c r="AG2" t="inlineStr"/>
-      <c r="AH2" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="AI2" t="n">
-        <v>-5.333333333333333</v>
-      </c>
-      <c r="AJ2" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="AK2" t="n">
-        <v>-0.5</v>
       </c>
       <c r="AL2" t="n">
         <v>71.22727272727272</v>
@@ -858,49 +858,49 @@
       <c r="AM2" t="n">
         <v>77.21818181818182</v>
       </c>
-      <c r="AN2" t="n">
+      <c r="AN2" t="inlineStr"/>
+      <c r="AO2" t="n">
+        <v>-29846130.95238096</v>
+      </c>
+      <c r="AP2" t="inlineStr"/>
+      <c r="AQ2" t="n">
+        <v>1.697725122744469</v>
+      </c>
+      <c r="AR2" t="inlineStr"/>
+      <c r="AS2" t="n">
+        <v>1.610714285714284</v>
+      </c>
+      <c r="AT2" t="n">
+        <v>-4.617364768874054</v>
+      </c>
+      <c r="AU2" t="n">
+        <v>-6.928968253968279</v>
+      </c>
+      <c r="AV2" t="n">
+        <v>-0.6529583972743467</v>
+      </c>
+      <c r="AW2" t="n">
+        <v>-20828499.91459402</v>
+      </c>
+      <c r="AX2" t="n">
+        <v>-5.53524554758107</v>
+      </c>
+      <c r="AY2" t="n">
         <v>-5.786111111111126</v>
       </c>
-      <c r="AO2" t="inlineStr"/>
-      <c r="AP2" t="n">
-        <v>-0.6529583972743467</v>
-      </c>
-      <c r="AQ2" t="n">
-        <v>-5.53524554758107</v>
-      </c>
-      <c r="AR2" t="n">
-        <v>-20828499.91459402</v>
-      </c>
-      <c r="AS2" t="n">
-        <v>-29846130.95238096</v>
-      </c>
-      <c r="AT2" t="n">
+      <c r="AZ2" t="inlineStr"/>
+      <c r="BA2" t="inlineStr"/>
+      <c r="BB2" t="n">
+        <v>-2.036111111111097</v>
+      </c>
+      <c r="BC2" t="inlineStr"/>
+      <c r="BD2" t="n">
         <v>-0.2652031356801094</v>
       </c>
-      <c r="AU2" t="n">
+      <c r="BE2" t="n">
         <v>-0.6529761904761904</v>
       </c>
-      <c r="AV2" t="inlineStr"/>
-      <c r="AW2" t="inlineStr"/>
-      <c r="AX2" t="n">
-        <v>-2.036111111111097</v>
-      </c>
-      <c r="AY2" t="n">
-        <v>1.610714285714284</v>
-      </c>
-      <c r="AZ2" t="inlineStr"/>
-      <c r="BA2" t="n">
-        <v>-6.928968253968279</v>
-      </c>
-      <c r="BB2" t="inlineStr"/>
-      <c r="BC2" t="inlineStr"/>
-      <c r="BD2" t="inlineStr"/>
-      <c r="BE2" t="n">
-        <v>-4.617364768874054</v>
-      </c>
-      <c r="BF2" t="n">
-        <v>1.697725122744469</v>
-      </c>
+      <c r="BF2" t="inlineStr"/>
       <c r="BG2" t="n">
         <v>0</v>
       </c>
@@ -984,54 +984,54 @@
         <v>0</v>
       </c>
       <c r="T3" t="n">
-        <v>0</v>
+        <v>6.75</v>
       </c>
       <c r="U3" t="n">
+        <v>10</v>
+      </c>
+      <c r="V3" t="inlineStr"/>
+      <c r="W3" t="inlineStr"/>
+      <c r="X3" t="n">
+        <v>0.3999999999999999</v>
+      </c>
+      <c r="Y3" t="n">
+        <v>-0.2</v>
+      </c>
+      <c r="Z3" t="n">
+        <v>3.166666666666666</v>
+      </c>
+      <c r="AA3" t="n">
+        <v>1.416666666666666</v>
+      </c>
+      <c r="AB3" t="n">
+        <v>2.083333333333334</v>
+      </c>
+      <c r="AC3" t="n">
+        <v>0.5833333333333335</v>
+      </c>
+      <c r="AD3" t="n">
+        <v>2.666666666666667</v>
+      </c>
+      <c r="AE3" t="n">
+        <v>0.666666666666667</v>
+      </c>
+      <c r="AF3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG3" t="n">
         <v>0.3333333333333333</v>
       </c>
-      <c r="V3" t="n">
+      <c r="AH3" t="n">
         <v>-4.333333333333336</v>
       </c>
-      <c r="W3" t="n">
+      <c r="AI3" t="n">
         <v>4.333333333333336</v>
       </c>
-      <c r="X3" t="n">
-        <v>3.166666666666666</v>
-      </c>
-      <c r="Y3" t="n">
-        <v>1.416666666666666</v>
-      </c>
-      <c r="Z3" t="n">
-        <v>6.75</v>
-      </c>
-      <c r="AA3" t="n">
-        <v>10</v>
-      </c>
-      <c r="AB3" t="n">
-        <v>2.666666666666667</v>
-      </c>
-      <c r="AC3" t="n">
-        <v>0.666666666666667</v>
-      </c>
-      <c r="AD3" t="n">
+      <c r="AJ3" t="n">
         <v>0.5366666666666666</v>
       </c>
-      <c r="AE3" t="n">
+      <c r="AK3" t="n">
         <v>0.8383333333333336</v>
-      </c>
-      <c r="AF3" t="inlineStr"/>
-      <c r="AG3" t="inlineStr"/>
-      <c r="AH3" t="n">
-        <v>2.083333333333334</v>
-      </c>
-      <c r="AI3" t="n">
-        <v>0.5833333333333335</v>
-      </c>
-      <c r="AJ3" t="n">
-        <v>0.3999999999999999</v>
-      </c>
-      <c r="AK3" t="n">
-        <v>-0.2</v>
       </c>
       <c r="AL3" t="n">
         <v>78.76801346801348</v>
@@ -1039,49 +1039,49 @@
       <c r="AM3" t="n">
         <v>77.85375573921029</v>
       </c>
-      <c r="AN3" t="n">
+      <c r="AN3" t="inlineStr"/>
+      <c r="AO3" t="n">
+        <v>-52528383.83838384</v>
+      </c>
+      <c r="AP3" t="inlineStr"/>
+      <c r="AQ3" t="n">
+        <v>-1.702080137329435</v>
+      </c>
+      <c r="AR3" t="inlineStr"/>
+      <c r="AS3" t="n">
+        <v>-3.228484848484843</v>
+      </c>
+      <c r="AT3" t="n">
+        <v>-7.193227926985998</v>
+      </c>
+      <c r="AU3" t="n">
+        <v>-4.290404040404042</v>
+      </c>
+      <c r="AV3" t="n">
+        <v>4.663911373155372</v>
+      </c>
+      <c r="AW3" t="n">
+        <v>-30861818.17709465</v>
+      </c>
+      <c r="AX3" t="n">
+        <v>-3.922110422454423</v>
+      </c>
+      <c r="AY3" t="n">
         <v>-7.368484848484854</v>
       </c>
-      <c r="AO3" t="inlineStr"/>
-      <c r="AP3" t="n">
-        <v>4.663911373155372</v>
-      </c>
-      <c r="AQ3" t="n">
-        <v>-3.922110422454423</v>
-      </c>
-      <c r="AR3" t="n">
-        <v>-30861818.17709465</v>
-      </c>
-      <c r="AS3" t="n">
-        <v>-52528383.83838384</v>
-      </c>
-      <c r="AT3" t="n">
+      <c r="AZ3" t="inlineStr"/>
+      <c r="BA3" t="inlineStr"/>
+      <c r="BB3" t="n">
+        <v>0.7455555555555406</v>
+      </c>
+      <c r="BC3" t="inlineStr"/>
+      <c r="BD3" t="n">
         <v>-0.6644494615050729</v>
       </c>
-      <c r="AU3" t="n">
+      <c r="BE3" t="n">
         <v>-1.394848484848485</v>
       </c>
-      <c r="AV3" t="inlineStr"/>
-      <c r="AW3" t="inlineStr"/>
-      <c r="AX3" t="n">
-        <v>0.7455555555555406</v>
-      </c>
-      <c r="AY3" t="n">
-        <v>-3.228484848484843</v>
-      </c>
-      <c r="AZ3" t="inlineStr"/>
-      <c r="BA3" t="n">
-        <v>-4.290404040404042</v>
-      </c>
-      <c r="BB3" t="inlineStr"/>
-      <c r="BC3" t="inlineStr"/>
-      <c r="BD3" t="inlineStr"/>
-      <c r="BE3" t="n">
-        <v>-7.193227926985998</v>
-      </c>
-      <c r="BF3" t="n">
-        <v>-1.702080137329435</v>
-      </c>
+      <c r="BF3" t="inlineStr"/>
       <c r="BG3" t="n">
         <v>0</v>
       </c>
@@ -1165,54 +1165,54 @@
         <v>0</v>
       </c>
       <c r="T4" t="n">
+        <v>-5</v>
+      </c>
+      <c r="U4" t="n">
+        <v>2</v>
+      </c>
+      <c r="V4" t="inlineStr"/>
+      <c r="W4" t="inlineStr"/>
+      <c r="X4" t="n">
+        <v>-1.5</v>
+      </c>
+      <c r="Y4" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="Z4" t="n">
+        <v>-4.5</v>
+      </c>
+      <c r="AA4" t="n">
+        <v>-3.5</v>
+      </c>
+      <c r="AB4" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AC4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE4" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF4" t="n">
         <v>-1</v>
       </c>
-      <c r="U4" t="n">
+      <c r="AG4" t="n">
         <v>1</v>
       </c>
-      <c r="V4" t="n">
+      <c r="AH4" t="n">
         <v>12</v>
       </c>
-      <c r="W4" t="n">
+      <c r="AI4" t="n">
         <v>-12</v>
       </c>
-      <c r="X4" t="n">
-        <v>-4.5</v>
-      </c>
-      <c r="Y4" t="n">
-        <v>-3.5</v>
-      </c>
-      <c r="Z4" t="n">
-        <v>-5</v>
-      </c>
-      <c r="AA4" t="n">
-        <v>2</v>
-      </c>
-      <c r="AB4" t="n">
-        <v>0</v>
-      </c>
-      <c r="AC4" t="n">
-        <v>1</v>
-      </c>
-      <c r="AD4" t="n">
+      <c r="AJ4" t="n">
         <v>-0.8949999999999998</v>
       </c>
-      <c r="AE4" t="n">
+      <c r="AK4" t="n">
         <v>1.085</v>
-      </c>
-      <c r="AF4" t="inlineStr"/>
-      <c r="AG4" t="inlineStr"/>
-      <c r="AH4" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="AI4" t="n">
-        <v>0</v>
-      </c>
-      <c r="AJ4" t="n">
-        <v>-1.5</v>
-      </c>
-      <c r="AK4" t="n">
-        <v>1.5</v>
       </c>
       <c r="AL4" t="n">
         <v>77.95454545454545</v>
@@ -1220,49 +1220,49 @@
       <c r="AM4" t="n">
         <v>76.54545454545455</v>
       </c>
-      <c r="AN4" t="n">
+      <c r="AN4" t="inlineStr"/>
+      <c r="AO4" t="n">
+        <v>-2588798.701298706</v>
+      </c>
+      <c r="AP4" t="inlineStr"/>
+      <c r="AQ4" t="n">
+        <v>-1.6851765897053</v>
+      </c>
+      <c r="AR4" t="inlineStr"/>
+      <c r="AS4" t="n">
+        <v>0.4009740259740262</v>
+      </c>
+      <c r="AT4" t="n">
+        <v>0.4662913277439316</v>
+      </c>
+      <c r="AU4" t="n">
+        <v>-0.9415584415584277</v>
+      </c>
+      <c r="AV4" t="n">
+        <v>-3.019159858832978</v>
+      </c>
+      <c r="AW4" t="n">
+        <v>-780645.2390500437</v>
+      </c>
+      <c r="AX4" t="n">
+        <v>1.164141144634812</v>
+      </c>
+      <c r="AY4" t="n">
         <v>0.08279220779220964</v>
       </c>
-      <c r="AO4" t="inlineStr"/>
-      <c r="AP4" t="n">
-        <v>-3.019159858832978</v>
-      </c>
-      <c r="AQ4" t="n">
-        <v>1.164141144634812</v>
-      </c>
-      <c r="AR4" t="n">
-        <v>-780645.2390500437</v>
-      </c>
-      <c r="AS4" t="n">
-        <v>-2588798.701298706</v>
-      </c>
-      <c r="AT4" t="n">
+      <c r="AZ4" t="inlineStr"/>
+      <c r="BA4" t="inlineStr"/>
+      <c r="BB4" t="n">
+        <v>0.7142857142857224</v>
+      </c>
+      <c r="BC4" t="inlineStr"/>
+      <c r="BD4" t="n">
         <v>-0.07075274904011941</v>
       </c>
-      <c r="AU4" t="n">
+      <c r="BE4" t="n">
         <v>-0.2418831168831173</v>
       </c>
-      <c r="AV4" t="inlineStr"/>
-      <c r="AW4" t="inlineStr"/>
-      <c r="AX4" t="n">
-        <v>0.7142857142857224</v>
-      </c>
-      <c r="AY4" t="n">
-        <v>0.4009740259740262</v>
-      </c>
-      <c r="AZ4" t="inlineStr"/>
-      <c r="BA4" t="n">
-        <v>-0.9415584415584277</v>
-      </c>
-      <c r="BB4" t="inlineStr"/>
-      <c r="BC4" t="inlineStr"/>
-      <c r="BD4" t="inlineStr"/>
-      <c r="BE4" t="n">
-        <v>0.4662913277439316</v>
-      </c>
-      <c r="BF4" t="n">
-        <v>-1.6851765897053</v>
-      </c>
+      <c r="BF4" t="inlineStr"/>
       <c r="BG4" t="n">
         <v>0</v>
       </c>
@@ -1346,54 +1346,54 @@
         <v>0</v>
       </c>
       <c r="T5" t="n">
-        <v>2.5</v>
+        <v>12.5</v>
       </c>
       <c r="U5" t="n">
-        <v>-1.5</v>
-      </c>
-      <c r="V5" t="n">
-        <v>-4</v>
-      </c>
-      <c r="W5" t="n">
-        <v>4</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="V5" t="inlineStr"/>
+      <c r="W5" t="inlineStr"/>
       <c r="X5" t="n">
+        <v>2</v>
+      </c>
+      <c r="Y5" t="n">
+        <v>-2.5</v>
+      </c>
+      <c r="Z5" t="n">
         <v>-0.5</v>
-      </c>
-      <c r="Y5" t="n">
-        <v>1</v>
-      </c>
-      <c r="Z5" t="n">
-        <v>12.5</v>
       </c>
       <c r="AA5" t="n">
         <v>1</v>
       </c>
       <c r="AB5" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="AC5" t="n">
+        <v>-4</v>
+      </c>
+      <c r="AD5" t="n">
         <v>-1</v>
       </c>
-      <c r="AC5" t="n">
+      <c r="AE5" t="n">
         <v>-0.5</v>
       </c>
-      <c r="AD5" t="n">
+      <c r="AF5" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="AG5" t="n">
+        <v>-1.5</v>
+      </c>
+      <c r="AH5" t="n">
+        <v>-4</v>
+      </c>
+      <c r="AI5" t="n">
+        <v>4</v>
+      </c>
+      <c r="AJ5" t="n">
         <v>0.9299999999999998</v>
       </c>
-      <c r="AE5" t="n">
+      <c r="AK5" t="n">
         <v>-1.285</v>
-      </c>
-      <c r="AF5" t="inlineStr"/>
-      <c r="AG5" t="inlineStr"/>
-      <c r="AH5" t="n">
-        <v>6.5</v>
-      </c>
-      <c r="AI5" t="n">
-        <v>-4</v>
-      </c>
-      <c r="AJ5" t="n">
-        <v>2</v>
-      </c>
-      <c r="AK5" t="n">
-        <v>-2.5</v>
       </c>
       <c r="AL5" t="n">
         <v>77.62272727272727</v>
@@ -1401,49 +1401,49 @@
       <c r="AM5" t="n">
         <v>76.5</v>
       </c>
-      <c r="AN5" t="n">
+      <c r="AN5" t="inlineStr"/>
+      <c r="AO5" t="n">
+        <v>-7768311.688311685</v>
+      </c>
+      <c r="AP5" t="inlineStr"/>
+      <c r="AQ5" t="n">
+        <v>3.697361368789938</v>
+      </c>
+      <c r="AR5" t="inlineStr"/>
+      <c r="AS5" t="n">
+        <v>1.584415584415584</v>
+      </c>
+      <c r="AT5" t="n">
+        <v>-0.06373503947033043</v>
+      </c>
+      <c r="AU5" t="n">
+        <v>-1.303896103896093</v>
+      </c>
+      <c r="AV5" t="n">
+        <v>-2.482223040731469</v>
+      </c>
+      <c r="AW5" t="n">
+        <v>-4560738.276371153</v>
+      </c>
+      <c r="AX5" t="n">
+        <v>-1.855779584561105</v>
+      </c>
+      <c r="AY5" t="n">
         <v>-1.028571428571425</v>
       </c>
-      <c r="AO5" t="inlineStr"/>
-      <c r="AP5" t="n">
-        <v>-2.482223040731469</v>
-      </c>
-      <c r="AQ5" t="n">
-        <v>-1.855779584561105</v>
-      </c>
-      <c r="AR5" t="n">
-        <v>-4560738.276371153</v>
-      </c>
-      <c r="AS5" t="n">
-        <v>-7768311.688311685</v>
-      </c>
-      <c r="AT5" t="n">
+      <c r="AZ5" t="inlineStr"/>
+      <c r="BA5" t="inlineStr"/>
+      <c r="BB5" t="n">
+        <v>0.7597402597402549</v>
+      </c>
+      <c r="BC5" t="inlineStr"/>
+      <c r="BD5" t="n">
         <v>0.03935195290237292</v>
       </c>
-      <c r="AU5" t="n">
+      <c r="BE5" t="n">
         <v>-0.02467532467532463</v>
       </c>
-      <c r="AV5" t="inlineStr"/>
-      <c r="AW5" t="inlineStr"/>
-      <c r="AX5" t="n">
-        <v>0.7597402597402549</v>
-      </c>
-      <c r="AY5" t="n">
-        <v>1.584415584415584</v>
-      </c>
-      <c r="AZ5" t="inlineStr"/>
-      <c r="BA5" t="n">
-        <v>-1.303896103896093</v>
-      </c>
-      <c r="BB5" t="inlineStr"/>
-      <c r="BC5" t="inlineStr"/>
-      <c r="BD5" t="inlineStr"/>
-      <c r="BE5" t="n">
-        <v>-0.06373503947033043</v>
-      </c>
-      <c r="BF5" t="n">
-        <v>3.697361368789938</v>
-      </c>
+      <c r="BF5" t="inlineStr"/>
       <c r="BG5" t="n">
         <v>0</v>
       </c>
@@ -1527,54 +1527,54 @@
         <v>0</v>
       </c>
       <c r="T6" t="n">
+        <v>22.66666666666667</v>
+      </c>
+      <c r="U6" t="n">
+        <v>-21.66666666666667</v>
+      </c>
+      <c r="V6" t="inlineStr"/>
+      <c r="W6" t="inlineStr"/>
+      <c r="X6" t="n">
+        <v>3</v>
+      </c>
+      <c r="Y6" t="n">
+        <v>-3</v>
+      </c>
+      <c r="Z6" t="n">
+        <v>-1.5</v>
+      </c>
+      <c r="AA6" t="n">
+        <v>2.333333333333334</v>
+      </c>
+      <c r="AB6" t="n">
+        <v>6</v>
+      </c>
+      <c r="AC6" t="n">
+        <v>-11.33333333333333</v>
+      </c>
+      <c r="AD6" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AE6" t="n">
+        <v>-1.166666666666667</v>
+      </c>
+      <c r="AF6" t="n">
         <v>2.833333333333333</v>
       </c>
-      <c r="U6" t="n">
+      <c r="AG6" t="n">
         <v>-3.166666666666667</v>
       </c>
-      <c r="V6" t="n">
+      <c r="AH6" t="n">
         <v>18.33333333333334</v>
       </c>
-      <c r="W6" t="n">
+      <c r="AI6" t="n">
         <v>-18.33333333333334</v>
       </c>
-      <c r="X6" t="n">
-        <v>-1.5</v>
-      </c>
-      <c r="Y6" t="n">
-        <v>2.333333333333334</v>
-      </c>
-      <c r="Z6" t="n">
-        <v>22.66666666666667</v>
-      </c>
-      <c r="AA6" t="n">
-        <v>-21.66666666666667</v>
-      </c>
-      <c r="AB6" t="n">
-        <v>-1</v>
-      </c>
-      <c r="AC6" t="n">
-        <v>-1.166666666666667</v>
-      </c>
-      <c r="AD6" t="n">
+      <c r="AJ6" t="n">
         <v>2.831666666666667</v>
       </c>
-      <c r="AE6" t="n">
+      <c r="AK6" t="n">
         <v>-2.891666666666667</v>
-      </c>
-      <c r="AF6" t="inlineStr"/>
-      <c r="AG6" t="inlineStr"/>
-      <c r="AH6" t="n">
-        <v>6</v>
-      </c>
-      <c r="AI6" t="n">
-        <v>-11.33333333333333</v>
-      </c>
-      <c r="AJ6" t="n">
-        <v>3</v>
-      </c>
-      <c r="AK6" t="n">
-        <v>-3</v>
       </c>
       <c r="AL6" t="n">
         <v>75.97205387205388</v>
@@ -1582,49 +1582,49 @@
       <c r="AM6" t="n">
         <v>84.92727272727274</v>
       </c>
-      <c r="AN6" t="n">
+      <c r="AN6" t="inlineStr"/>
+      <c r="AO6" t="n">
+        <v>47881727.43055556</v>
+      </c>
+      <c r="AP6" t="inlineStr"/>
+      <c r="AQ6" t="n">
+        <v>0.3440181335692181</v>
+      </c>
+      <c r="AR6" t="inlineStr"/>
+      <c r="AS6" t="n">
+        <v>-1.880208333333332</v>
+      </c>
+      <c r="AT6" t="n">
+        <v>9.096245041078632</v>
+      </c>
+      <c r="AU6" t="n">
+        <v>6.868055555555557</v>
+      </c>
+      <c r="AV6" t="n">
+        <v>-1.492309818664296</v>
+      </c>
+      <c r="AW6" t="n">
+        <v>28947364.23277445</v>
+      </c>
+      <c r="AX6" t="n">
+        <v>5.901018756784993</v>
+      </c>
+      <c r="AY6" t="n">
         <v>7.060763888888886</v>
       </c>
-      <c r="AO6" t="inlineStr"/>
-      <c r="AP6" t="n">
-        <v>-1.492309818664296</v>
-      </c>
-      <c r="AQ6" t="n">
-        <v>5.901018756784993</v>
-      </c>
-      <c r="AR6" t="n">
-        <v>28947364.23277445</v>
-      </c>
-      <c r="AS6" t="n">
-        <v>47881727.43055556</v>
-      </c>
-      <c r="AT6" t="n">
+      <c r="AZ6" t="inlineStr"/>
+      <c r="BA6" t="inlineStr"/>
+      <c r="BB6" t="n">
+        <v>0.07986111111111427</v>
+      </c>
+      <c r="BC6" t="inlineStr"/>
+      <c r="BD6" t="n">
         <v>0.4727499731950198</v>
       </c>
-      <c r="AU6" t="n">
+      <c r="BE6" t="n">
         <v>0.8263888888888886</v>
       </c>
-      <c r="AV6" t="inlineStr"/>
-      <c r="AW6" t="inlineStr"/>
-      <c r="AX6" t="n">
-        <v>0.07986111111111427</v>
-      </c>
-      <c r="AY6" t="n">
-        <v>-1.880208333333332</v>
-      </c>
-      <c r="AZ6" t="inlineStr"/>
-      <c r="BA6" t="n">
-        <v>6.868055555555557</v>
-      </c>
-      <c r="BB6" t="inlineStr"/>
-      <c r="BC6" t="inlineStr"/>
-      <c r="BD6" t="inlineStr"/>
-      <c r="BE6" t="n">
-        <v>9.096245041078632</v>
-      </c>
-      <c r="BF6" t="n">
-        <v>0.3440181335692181</v>
-      </c>
+      <c r="BF6" t="inlineStr"/>
       <c r="BG6" t="n">
         <v>0</v>
       </c>
@@ -1708,54 +1708,54 @@
         <v>0</v>
       </c>
       <c r="T7" t="n">
+        <v>0</v>
+      </c>
+      <c r="U7" t="n">
+        <v>-3</v>
+      </c>
+      <c r="V7" t="inlineStr"/>
+      <c r="W7" t="inlineStr"/>
+      <c r="X7" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="Y7" t="n">
+        <v>-2</v>
+      </c>
+      <c r="Z7" t="n">
+        <v>-3.75</v>
+      </c>
+      <c r="AA7" t="n">
+        <v>-0.25</v>
+      </c>
+      <c r="AB7" t="n">
+        <v>1.75</v>
+      </c>
+      <c r="AC7" t="n">
+        <v>-2.75</v>
+      </c>
+      <c r="AD7" t="n">
+        <v>-0.25</v>
+      </c>
+      <c r="AE7" t="n">
+        <v>-0.5</v>
+      </c>
+      <c r="AF7" t="n">
         <v>1</v>
       </c>
-      <c r="U7" t="n">
+      <c r="AG7" t="n">
         <v>-2</v>
       </c>
-      <c r="V7" t="n">
+      <c r="AH7" t="n">
         <v>-14.75</v>
       </c>
-      <c r="W7" t="n">
+      <c r="AI7" t="n">
         <v>14.75</v>
       </c>
-      <c r="X7" t="n">
-        <v>-3.75</v>
-      </c>
-      <c r="Y7" t="n">
-        <v>-0.25</v>
-      </c>
-      <c r="Z7" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA7" t="n">
-        <v>-3</v>
-      </c>
-      <c r="AB7" t="n">
-        <v>-0.25</v>
-      </c>
-      <c r="AC7" t="n">
-        <v>-0.5</v>
-      </c>
-      <c r="AD7" t="n">
+      <c r="AJ7" t="n">
         <v>-0.24</v>
       </c>
-      <c r="AE7" t="n">
+      <c r="AK7" t="n">
         <v>-1.1925</v>
-      </c>
-      <c r="AF7" t="inlineStr"/>
-      <c r="AG7" t="inlineStr"/>
-      <c r="AH7" t="n">
-        <v>1.75</v>
-      </c>
-      <c r="AI7" t="n">
-        <v>-2.75</v>
-      </c>
-      <c r="AJ7" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="AK7" t="n">
-        <v>-2</v>
       </c>
       <c r="AL7" t="n">
         <v>77.02146464646464</v>
@@ -1763,49 +1763,49 @@
       <c r="AM7" t="n">
         <v>75.80000000000001</v>
       </c>
-      <c r="AN7" t="n">
+      <c r="AN7" t="inlineStr"/>
+      <c r="AO7" t="n">
+        <v>1775953.282828284</v>
+      </c>
+      <c r="AP7" t="inlineStr"/>
+      <c r="AQ7" t="n">
+        <v>1.618717119284788</v>
+      </c>
+      <c r="AR7" t="inlineStr"/>
+      <c r="AS7" t="n">
+        <v>1.663816738816742</v>
+      </c>
+      <c r="AT7" t="n">
+        <v>-0.2109521425847163</v>
+      </c>
+      <c r="AU7" t="n">
+        <v>-0.9375901875902031</v>
+      </c>
+      <c r="AV7" t="n">
+        <v>8.326102350265018</v>
+      </c>
+      <c r="AW7" t="n">
+        <v>-1432068.723799587</v>
+      </c>
+      <c r="AX7" t="n">
+        <v>-3.315135535049265</v>
+      </c>
+      <c r="AY7" t="n">
         <v>1.171753246753255</v>
       </c>
-      <c r="AO7" t="inlineStr"/>
-      <c r="AP7" t="n">
-        <v>8.326102350265018</v>
-      </c>
-      <c r="AQ7" t="n">
-        <v>-3.315135535049265</v>
-      </c>
-      <c r="AR7" t="n">
-        <v>-1432068.723799587</v>
-      </c>
-      <c r="AS7" t="n">
-        <v>1775953.282828284</v>
-      </c>
-      <c r="AT7" t="n">
+      <c r="AZ7" t="inlineStr"/>
+      <c r="BA7" t="inlineStr"/>
+      <c r="BB7" t="n">
+        <v>1.620490620490642</v>
+      </c>
+      <c r="BC7" t="inlineStr"/>
+      <c r="BD7" t="n">
         <v>-0.06534905438147809</v>
       </c>
-      <c r="AU7" t="n">
+      <c r="BE7" t="n">
         <v>0.2233766233766232</v>
       </c>
-      <c r="AV7" t="inlineStr"/>
-      <c r="AW7" t="inlineStr"/>
-      <c r="AX7" t="n">
-        <v>1.620490620490642</v>
-      </c>
-      <c r="AY7" t="n">
-        <v>1.663816738816742</v>
-      </c>
-      <c r="AZ7" t="inlineStr"/>
-      <c r="BA7" t="n">
-        <v>-0.9375901875902031</v>
-      </c>
-      <c r="BB7" t="inlineStr"/>
-      <c r="BC7" t="inlineStr"/>
-      <c r="BD7" t="inlineStr"/>
-      <c r="BE7" t="n">
-        <v>-0.2109521425847163</v>
-      </c>
-      <c r="BF7" t="n">
-        <v>1.618717119284788</v>
-      </c>
+      <c r="BF7" t="inlineStr"/>
       <c r="BG7" t="n">
         <v>0</v>
       </c>
@@ -1889,54 +1889,54 @@
         <v>0</v>
       </c>
       <c r="T8" t="n">
+        <v>7.199999999999999</v>
+      </c>
+      <c r="U8" t="n">
+        <v>1.800000000000001</v>
+      </c>
+      <c r="V8" t="inlineStr"/>
+      <c r="W8" t="inlineStr"/>
+      <c r="X8" t="n">
+        <v>0.6000000000000001</v>
+      </c>
+      <c r="Y8" t="n">
+        <v>-0.8999999999999999</v>
+      </c>
+      <c r="Z8" t="n">
+        <v>-1.800000000000001</v>
+      </c>
+      <c r="AA8" t="n">
+        <v>-2.199999999999999</v>
+      </c>
+      <c r="AB8" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="AC8" t="n">
+        <v>0.2999999999999998</v>
+      </c>
+      <c r="AD8" t="n">
+        <v>-2.8</v>
+      </c>
+      <c r="AE8" t="n">
+        <v>-0.2000000000000002</v>
+      </c>
+      <c r="AF8" t="n">
         <v>2.2</v>
       </c>
-      <c r="U8" t="n">
+      <c r="AG8" t="n">
         <v>-0.6000000000000001</v>
       </c>
-      <c r="V8" t="n">
+      <c r="AH8" t="n">
         <v>2.5</v>
       </c>
-      <c r="W8" t="n">
+      <c r="AI8" t="n">
         <v>-2.5</v>
       </c>
-      <c r="X8" t="n">
-        <v>-1.800000000000001</v>
-      </c>
-      <c r="Y8" t="n">
-        <v>-2.199999999999999</v>
-      </c>
-      <c r="Z8" t="n">
-        <v>7.199999999999999</v>
-      </c>
-      <c r="AA8" t="n">
-        <v>1.800000000000001</v>
-      </c>
-      <c r="AB8" t="n">
-        <v>-2.8</v>
-      </c>
-      <c r="AC8" t="n">
-        <v>-0.2000000000000002</v>
-      </c>
-      <c r="AD8" t="n">
+      <c r="AJ8" t="n">
         <v>1.316</v>
       </c>
-      <c r="AE8" t="n">
+      <c r="AK8" t="n">
         <v>0.3799999999999999</v>
-      </c>
-      <c r="AF8" t="inlineStr"/>
-      <c r="AG8" t="inlineStr"/>
-      <c r="AH8" t="n">
-        <v>3.4</v>
-      </c>
-      <c r="AI8" t="n">
-        <v>0.2999999999999998</v>
-      </c>
-      <c r="AJ8" t="n">
-        <v>0.6000000000000001</v>
-      </c>
-      <c r="AK8" t="n">
-        <v>-0.8999999999999999</v>
       </c>
       <c r="AL8" t="n">
         <v>73.29545454545455</v>
@@ -1944,49 +1944,49 @@
       <c r="AM8" t="n">
         <v>72.99111111111111</v>
       </c>
-      <c r="AN8" t="n">
+      <c r="AN8" t="inlineStr"/>
+      <c r="AO8" t="n">
+        <v>14692283.05785124</v>
+      </c>
+      <c r="AP8" t="inlineStr"/>
+      <c r="AQ8" t="n">
+        <v>1.409744653790366</v>
+      </c>
+      <c r="AR8" t="inlineStr"/>
+      <c r="AS8" t="n">
+        <v>0.7660123966942081</v>
+      </c>
+      <c r="AT8" t="n">
+        <v>3.202640962511481</v>
+      </c>
+      <c r="AU8" t="n">
+        <v>4.699896694214871</v>
+      </c>
+      <c r="AV8" t="n">
+        <v>2.517704458265484</v>
+      </c>
+      <c r="AW8" t="n">
+        <v>10053627.24598238</v>
+      </c>
+      <c r="AX8" t="n">
+        <v>2.96223784474266</v>
+      </c>
+      <c r="AY8" t="n">
         <v>4.902169421487613</v>
       </c>
-      <c r="AO8" t="inlineStr"/>
-      <c r="AP8" t="n">
-        <v>2.517704458265484</v>
-      </c>
-      <c r="AQ8" t="n">
-        <v>2.96223784474266</v>
-      </c>
-      <c r="AR8" t="n">
-        <v>10053627.24598238</v>
-      </c>
-      <c r="AS8" t="n">
-        <v>14692283.05785124</v>
-      </c>
-      <c r="AT8" t="n">
+      <c r="AZ8" t="inlineStr"/>
+      <c r="BA8" t="inlineStr"/>
+      <c r="BB8" t="n">
+        <v>5.375206611570235</v>
+      </c>
+      <c r="BC8" t="inlineStr"/>
+      <c r="BD8" t="n">
         <v>0.4238095238095236</v>
       </c>
-      <c r="AU8" t="n">
+      <c r="BE8" t="n">
         <v>0.5102272727272728</v>
       </c>
-      <c r="AV8" t="inlineStr"/>
-      <c r="AW8" t="inlineStr"/>
-      <c r="AX8" t="n">
-        <v>5.375206611570235</v>
-      </c>
-      <c r="AY8" t="n">
-        <v>0.7660123966942081</v>
-      </c>
-      <c r="AZ8" t="inlineStr"/>
-      <c r="BA8" t="n">
-        <v>4.699896694214871</v>
-      </c>
-      <c r="BB8" t="inlineStr"/>
-      <c r="BC8" t="inlineStr"/>
-      <c r="BD8" t="inlineStr"/>
-      <c r="BE8" t="n">
-        <v>3.202640962511481</v>
-      </c>
-      <c r="BF8" t="n">
-        <v>1.409744653790366</v>
-      </c>
+      <c r="BF8" t="inlineStr"/>
       <c r="BG8" t="n">
         <v>0</v>
       </c>
@@ -2070,54 +2070,54 @@
         <v>0</v>
       </c>
       <c r="T9" t="n">
+        <v>1</v>
+      </c>
+      <c r="U9" t="n">
+        <v>-6</v>
+      </c>
+      <c r="V9" t="inlineStr"/>
+      <c r="W9" t="inlineStr"/>
+      <c r="X9" t="n">
+        <v>-0.75</v>
+      </c>
+      <c r="Y9" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="Z9" t="n">
+        <v>-2</v>
+      </c>
+      <c r="AA9" t="n">
+        <v>-2.75</v>
+      </c>
+      <c r="AB9" t="n">
+        <v>-1.75</v>
+      </c>
+      <c r="AC9" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AD9" t="n">
+        <v>-0.25</v>
+      </c>
+      <c r="AE9" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF9" t="n">
         <v>0.25</v>
       </c>
-      <c r="U9" t="n">
+      <c r="AG9" t="n">
         <v>0.5</v>
       </c>
-      <c r="V9" t="n">
+      <c r="AH9" t="n">
         <v>-8</v>
       </c>
-      <c r="W9" t="n">
+      <c r="AI9" t="n">
         <v>8</v>
       </c>
-      <c r="X9" t="n">
-        <v>-2</v>
-      </c>
-      <c r="Y9" t="n">
-        <v>-2.75</v>
-      </c>
-      <c r="Z9" t="n">
-        <v>1</v>
-      </c>
-      <c r="AA9" t="n">
-        <v>-6</v>
-      </c>
-      <c r="AB9" t="n">
-        <v>-0.25</v>
-      </c>
-      <c r="AC9" t="n">
-        <v>1</v>
-      </c>
-      <c r="AD9" t="n">
+      <c r="AJ9" t="n">
         <v>-0.0349999999999997</v>
       </c>
-      <c r="AE9" t="n">
+      <c r="AK9" t="n">
         <v>-0.4700000000000002</v>
-      </c>
-      <c r="AF9" t="inlineStr"/>
-      <c r="AG9" t="inlineStr"/>
-      <c r="AH9" t="n">
-        <v>-1.75</v>
-      </c>
-      <c r="AI9" t="n">
-        <v>-1</v>
-      </c>
-      <c r="AJ9" t="n">
-        <v>-0.75</v>
-      </c>
-      <c r="AK9" t="n">
-        <v>0.75</v>
       </c>
       <c r="AL9" t="n">
         <v>81.76666666666667</v>
@@ -2125,49 +2125,49 @@
       <c r="AM9" t="n">
         <v>80.13415404040404</v>
       </c>
-      <c r="AN9" t="n">
+      <c r="AN9" t="inlineStr"/>
+      <c r="AO9" t="n">
+        <v>-112321.4285714291</v>
+      </c>
+      <c r="AP9" t="inlineStr"/>
+      <c r="AQ9" t="n">
+        <v>0.9000830395087078</v>
+      </c>
+      <c r="AR9" t="inlineStr"/>
+      <c r="AS9" t="n">
+        <v>0.9857142857142875</v>
+      </c>
+      <c r="AT9" t="n">
+        <v>0.9510967786844304</v>
+      </c>
+      <c r="AU9" t="n">
+        <v>-0.2910714285714278</v>
+      </c>
+      <c r="AV9" t="n">
+        <v>2.362852243863756</v>
+      </c>
+      <c r="AW9" t="n">
+        <v>-238945.7190112025</v>
+      </c>
+      <c r="AX9" t="n">
+        <v>0.3619543532862792</v>
+      </c>
+      <c r="AY9" t="n">
         <v>-0.03749999999999432</v>
       </c>
-      <c r="AO9" t="inlineStr"/>
-      <c r="AP9" t="n">
-        <v>2.362852243863756</v>
-      </c>
-      <c r="AQ9" t="n">
-        <v>0.3619543532862792</v>
-      </c>
-      <c r="AR9" t="n">
-        <v>-238945.7190112025</v>
-      </c>
-      <c r="AS9" t="n">
-        <v>-112321.4285714291</v>
-      </c>
-      <c r="AT9" t="n">
+      <c r="AZ9" t="inlineStr"/>
+      <c r="BA9" t="inlineStr"/>
+      <c r="BB9" t="n">
+        <v>3.742857142857105</v>
+      </c>
+      <c r="BC9" t="inlineStr"/>
+      <c r="BD9" t="n">
         <v>0.1161873589842288</v>
       </c>
-      <c r="AU9" t="n">
+      <c r="BE9" t="n">
         <v>0.1089285714285715</v>
       </c>
-      <c r="AV9" t="inlineStr"/>
-      <c r="AW9" t="inlineStr"/>
-      <c r="AX9" t="n">
-        <v>3.742857142857105</v>
-      </c>
-      <c r="AY9" t="n">
-        <v>0.9857142857142875</v>
-      </c>
-      <c r="AZ9" t="inlineStr"/>
-      <c r="BA9" t="n">
-        <v>-0.2910714285714278</v>
-      </c>
-      <c r="BB9" t="inlineStr"/>
-      <c r="BC9" t="inlineStr"/>
-      <c r="BD9" t="inlineStr"/>
-      <c r="BE9" t="n">
-        <v>0.9510967786844304</v>
-      </c>
-      <c r="BF9" t="n">
-        <v>0.9000830395087078</v>
-      </c>
+      <c r="BF9" t="inlineStr"/>
       <c r="BG9" t="n">
         <v>0</v>
       </c>
@@ -2247,102 +2247,102 @@
         <v>0</v>
       </c>
       <c r="T10" t="n">
-        <v>0</v>
+        <v>4.25</v>
       </c>
       <c r="U10" t="n">
+        <v>-9.5</v>
+      </c>
+      <c r="V10" t="inlineStr"/>
+      <c r="W10" t="inlineStr"/>
+      <c r="X10" t="n">
+        <v>1.75</v>
+      </c>
+      <c r="Y10" t="n">
+        <v>-1.25</v>
+      </c>
+      <c r="Z10" t="n">
+        <v>-3.25</v>
+      </c>
+      <c r="AA10" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="AB10" t="n">
+        <v>-2.25</v>
+      </c>
+      <c r="AC10" t="n">
+        <v>-4</v>
+      </c>
+      <c r="AD10" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="AE10" t="n">
+        <v>1.75</v>
+      </c>
+      <c r="AF10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG10" t="n">
         <v>-2</v>
       </c>
-      <c r="V10" t="n">
+      <c r="AH10" t="n">
         <v>-4</v>
       </c>
-      <c r="W10" t="n">
+      <c r="AI10" t="n">
         <v>4</v>
       </c>
-      <c r="X10" t="n">
-        <v>-3.25</v>
-      </c>
-      <c r="Y10" t="n">
-        <v>4.5</v>
-      </c>
-      <c r="Z10" t="n">
-        <v>4.25</v>
-      </c>
-      <c r="AA10" t="n">
-        <v>-9.5</v>
-      </c>
-      <c r="AB10" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="AC10" t="n">
-        <v>1.75</v>
-      </c>
-      <c r="AD10" t="n">
+      <c r="AJ10" t="n">
         <v>-0.1925000000000001</v>
       </c>
-      <c r="AE10" t="n">
+      <c r="AK10" t="n">
         <v>-1.3675</v>
-      </c>
-      <c r="AF10" t="inlineStr"/>
-      <c r="AG10" t="inlineStr"/>
-      <c r="AH10" t="n">
-        <v>-2.25</v>
-      </c>
-      <c r="AI10" t="n">
-        <v>-4</v>
-      </c>
-      <c r="AJ10" t="n">
-        <v>1.75</v>
-      </c>
-      <c r="AK10" t="n">
-        <v>-1.25</v>
       </c>
       <c r="AL10" t="inlineStr"/>
       <c r="AM10" t="n">
         <v>78.65909090909091</v>
       </c>
-      <c r="AN10" t="n">
+      <c r="AN10" t="inlineStr"/>
+      <c r="AO10" t="n">
+        <v>-45110909.09090909</v>
+      </c>
+      <c r="AP10" t="inlineStr"/>
+      <c r="AQ10" t="n">
+        <v>1.938006096158269</v>
+      </c>
+      <c r="AR10" t="inlineStr"/>
+      <c r="AS10" t="n">
+        <v>0.4595959595959549</v>
+      </c>
+      <c r="AT10" t="n">
+        <v>-10.60447435012652</v>
+      </c>
+      <c r="AU10" t="n">
+        <v>-11.28787878787877</v>
+      </c>
+      <c r="AV10" t="n">
+        <v>-0.06185875316307943</v>
+      </c>
+      <c r="AW10" t="n">
+        <v>-32647976.76558546</v>
+      </c>
+      <c r="AX10" t="n">
+        <v>-11.21757821486082</v>
+      </c>
+      <c r="AY10" t="n">
         <v>-12.20606060606062</v>
       </c>
-      <c r="AO10" t="inlineStr"/>
-      <c r="AP10" t="n">
-        <v>-0.06185875316307943</v>
-      </c>
-      <c r="AQ10" t="n">
-        <v>-11.21757821486082</v>
-      </c>
-      <c r="AR10" t="n">
-        <v>-32647976.76558546</v>
-      </c>
-      <c r="AS10" t="n">
-        <v>-45110909.09090909</v>
-      </c>
-      <c r="AT10" t="n">
+      <c r="AZ10" t="inlineStr"/>
+      <c r="BA10" t="inlineStr"/>
+      <c r="BB10" t="n">
+        <v>-0.6909090909090878</v>
+      </c>
+      <c r="BC10" t="inlineStr"/>
+      <c r="BD10" t="n">
         <v>-0.8513400046008743</v>
       </c>
-      <c r="AU10" t="n">
+      <c r="BE10" t="n">
         <v>-1.65050505050505</v>
       </c>
-      <c r="AV10" t="inlineStr"/>
-      <c r="AW10" t="inlineStr"/>
-      <c r="AX10" t="n">
-        <v>-0.6909090909090878</v>
-      </c>
-      <c r="AY10" t="n">
-        <v>0.4595959595959549</v>
-      </c>
-      <c r="AZ10" t="inlineStr"/>
-      <c r="BA10" t="n">
-        <v>-11.28787878787877</v>
-      </c>
-      <c r="BB10" t="inlineStr"/>
-      <c r="BC10" t="inlineStr"/>
-      <c r="BD10" t="inlineStr"/>
-      <c r="BE10" t="n">
-        <v>-10.60447435012652</v>
-      </c>
-      <c r="BF10" t="n">
-        <v>1.938006096158269</v>
-      </c>
+      <c r="BF10" t="inlineStr"/>
       <c r="BG10" t="n">
         <v>0</v>
       </c>
@@ -2426,54 +2426,54 @@
         <v>0</v>
       </c>
       <c r="T11" t="n">
-        <v>0</v>
+        <v>5.25</v>
       </c>
       <c r="U11" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="V11" t="inlineStr"/>
+      <c r="W11" t="inlineStr"/>
+      <c r="X11" t="n">
+        <v>-0.3999999999999999</v>
+      </c>
+      <c r="Y11" t="n">
         <v>0.5</v>
       </c>
-      <c r="V11" t="n">
-        <v>0</v>
-      </c>
-      <c r="W11" t="n">
-        <v>0</v>
-      </c>
-      <c r="X11" t="n">
+      <c r="Z11" t="n">
         <v>-4.25</v>
       </c>
-      <c r="Y11" t="n">
+      <c r="AA11" t="n">
         <v>-0.75</v>
       </c>
-      <c r="Z11" t="n">
-        <v>5.25</v>
-      </c>
-      <c r="AA11" t="n">
-        <v>3.5</v>
-      </c>
       <c r="AB11" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="AC11" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="AD11" t="n">
         <v>1</v>
       </c>
-      <c r="AC11" t="n">
+      <c r="AE11" t="n">
         <v>-0.25</v>
       </c>
-      <c r="AD11" t="n">
+      <c r="AF11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG11" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AH11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ11" t="n">
         <v>0.8125</v>
       </c>
-      <c r="AE11" t="n">
+      <c r="AK11" t="n">
         <v>-0.08499999999999996</v>
-      </c>
-      <c r="AF11" t="inlineStr"/>
-      <c r="AG11" t="inlineStr"/>
-      <c r="AH11" t="n">
-        <v>2.75</v>
-      </c>
-      <c r="AI11" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="AJ11" t="n">
-        <v>-0.3999999999999999</v>
-      </c>
-      <c r="AK11" t="n">
-        <v>0.5</v>
       </c>
       <c r="AL11" t="n">
         <v>78.01627272727274</v>
@@ -2481,49 +2481,49 @@
       <c r="AM11" t="n">
         <v>74.54545454545453</v>
       </c>
-      <c r="AN11" t="n">
+      <c r="AN11" t="inlineStr"/>
+      <c r="AO11" t="n">
+        <v>17019983.60225633</v>
+      </c>
+      <c r="AP11" t="inlineStr"/>
+      <c r="AQ11" t="n">
+        <v>-3.654831907610326</v>
+      </c>
+      <c r="AR11" t="inlineStr"/>
+      <c r="AS11" t="n">
+        <v>-2.333989243080151</v>
+      </c>
+      <c r="AT11" t="n">
+        <v>0.02235611336402599</v>
+      </c>
+      <c r="AU11" t="n">
+        <v>5.466745375836283</v>
+      </c>
+      <c r="AV11" t="n">
+        <v>2.544944017851492</v>
+      </c>
+      <c r="AW11" t="n">
+        <v>10984469.04336654</v>
+      </c>
+      <c r="AX11" t="n">
+        <v>5.024274162893079</v>
+      </c>
+      <c r="AY11" t="n">
         <v>2.722746950019683</v>
       </c>
-      <c r="AO11" t="inlineStr"/>
-      <c r="AP11" t="n">
-        <v>2.544944017851492</v>
-      </c>
-      <c r="AQ11" t="n">
-        <v>5.024274162893079</v>
-      </c>
-      <c r="AR11" t="n">
-        <v>10984469.04336654</v>
-      </c>
-      <c r="AS11" t="n">
-        <v>17019983.60225633</v>
-      </c>
-      <c r="AT11" t="n">
+      <c r="AZ11" t="inlineStr"/>
+      <c r="BA11" t="inlineStr"/>
+      <c r="BB11" t="n">
+        <v>0.7954742227468898</v>
+      </c>
+      <c r="BC11" t="inlineStr"/>
+      <c r="BD11" t="n">
         <v>0.5276486675638035</v>
       </c>
-      <c r="AU11" t="n">
+      <c r="BE11" t="n">
         <v>0.6762691853600942</v>
       </c>
-      <c r="AV11" t="inlineStr"/>
-      <c r="AW11" t="inlineStr"/>
-      <c r="AX11" t="n">
-        <v>0.7954742227468898</v>
-      </c>
-      <c r="AY11" t="n">
-        <v>-2.333989243080151</v>
-      </c>
-      <c r="AZ11" t="inlineStr"/>
-      <c r="BA11" t="n">
-        <v>5.466745375836283</v>
-      </c>
-      <c r="BB11" t="inlineStr"/>
-      <c r="BC11" t="inlineStr"/>
-      <c r="BD11" t="inlineStr"/>
-      <c r="BE11" t="n">
-        <v>0.02235611336402599</v>
-      </c>
-      <c r="BF11" t="n">
-        <v>-3.654831907610326</v>
-      </c>
+      <c r="BF11" t="inlineStr"/>
       <c r="BG11" t="n">
         <v>0</v>
       </c>
@@ -2607,54 +2607,54 @@
         <v>0</v>
       </c>
       <c r="T12" t="n">
+        <v>1.666666666666666</v>
+      </c>
+      <c r="U12" t="n">
+        <v>-7.333333333333333</v>
+      </c>
+      <c r="V12" t="inlineStr"/>
+      <c r="W12" t="inlineStr"/>
+      <c r="X12" t="n">
+        <v>-2</v>
+      </c>
+      <c r="Y12" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z12" t="n">
+        <v>6.666666666666668</v>
+      </c>
+      <c r="AA12" t="n">
+        <v>7</v>
+      </c>
+      <c r="AB12" t="n">
+        <v>-1.333333333333333</v>
+      </c>
+      <c r="AC12" t="n">
+        <v>-1.333333333333333</v>
+      </c>
+      <c r="AD12" t="n">
+        <v>2.666666666666667</v>
+      </c>
+      <c r="AE12" t="n">
+        <v>4</v>
+      </c>
+      <c r="AF12" t="n">
         <v>-2.333333333333333</v>
       </c>
-      <c r="U12" t="n">
-        <v>0</v>
-      </c>
-      <c r="V12" t="n">
+      <c r="AG12" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH12" t="n">
         <v>5.666666666666664</v>
       </c>
-      <c r="W12" t="n">
+      <c r="AI12" t="n">
         <v>-5.666666666666664</v>
       </c>
-      <c r="X12" t="n">
-        <v>6.666666666666668</v>
-      </c>
-      <c r="Y12" t="n">
-        <v>7</v>
-      </c>
-      <c r="Z12" t="n">
-        <v>1.666666666666666</v>
-      </c>
-      <c r="AA12" t="n">
-        <v>-7.333333333333333</v>
-      </c>
-      <c r="AB12" t="n">
-        <v>2.666666666666667</v>
-      </c>
-      <c r="AC12" t="n">
-        <v>4</v>
-      </c>
-      <c r="AD12" t="n">
+      <c r="AJ12" t="n">
         <v>-0.3266666666666667</v>
       </c>
-      <c r="AE12" t="n">
+      <c r="AK12" t="n">
         <v>-1.066666666666667</v>
-      </c>
-      <c r="AF12" t="inlineStr"/>
-      <c r="AG12" t="inlineStr"/>
-      <c r="AH12" t="n">
-        <v>-1.333333333333333</v>
-      </c>
-      <c r="AI12" t="n">
-        <v>-1.333333333333333</v>
-      </c>
-      <c r="AJ12" t="n">
-        <v>-2</v>
-      </c>
-      <c r="AK12" t="n">
-        <v>2</v>
       </c>
       <c r="AL12" t="n">
         <v>72.98888888888888</v>
@@ -2662,49 +2662,49 @@
       <c r="AM12" t="n">
         <v>69</v>
       </c>
-      <c r="AN12" t="n">
+      <c r="AN12" t="inlineStr"/>
+      <c r="AO12" t="n">
+        <v>6137873.176206509</v>
+      </c>
+      <c r="AP12" t="inlineStr"/>
+      <c r="AQ12" t="n">
+        <v>2.571972157433972</v>
+      </c>
+      <c r="AR12" t="inlineStr"/>
+      <c r="AS12" t="n">
+        <v>-1.061503928170595</v>
+      </c>
+      <c r="AT12" t="n">
+        <v>7.331146766698879</v>
+      </c>
+      <c r="AU12" t="n">
+        <v>4.746520763187448</v>
+      </c>
+      <c r="AV12" t="n">
+        <v>0.8657106619825754</v>
+      </c>
+      <c r="AW12" t="n">
+        <v>3577584.255148304</v>
+      </c>
+      <c r="AX12" t="n">
+        <v>3.016572387689507</v>
+      </c>
+      <c r="AY12" t="n">
         <v>4.648877665544319</v>
       </c>
-      <c r="AO12" t="inlineStr"/>
-      <c r="AP12" t="n">
-        <v>0.8657106619825754</v>
-      </c>
-      <c r="AQ12" t="n">
-        <v>3.016572387689507</v>
-      </c>
-      <c r="AR12" t="n">
-        <v>3577584.255148304</v>
-      </c>
-      <c r="AS12" t="n">
-        <v>6137873.176206509</v>
-      </c>
-      <c r="AT12" t="n">
+      <c r="AZ12" t="inlineStr"/>
+      <c r="BA12" t="inlineStr"/>
+      <c r="BB12" t="n">
+        <v>2.392087542087609</v>
+      </c>
+      <c r="BC12" t="inlineStr"/>
+      <c r="BD12" t="n">
         <v>0.04603727455894635</v>
       </c>
-      <c r="AU12" t="n">
+      <c r="BE12" t="n">
         <v>0.1550505050505051</v>
       </c>
-      <c r="AV12" t="inlineStr"/>
-      <c r="AW12" t="inlineStr"/>
-      <c r="AX12" t="n">
-        <v>2.392087542087609</v>
-      </c>
-      <c r="AY12" t="n">
-        <v>-1.061503928170595</v>
-      </c>
-      <c r="AZ12" t="inlineStr"/>
-      <c r="BA12" t="n">
-        <v>4.746520763187448</v>
-      </c>
-      <c r="BB12" t="inlineStr"/>
-      <c r="BC12" t="inlineStr"/>
-      <c r="BD12" t="inlineStr"/>
-      <c r="BE12" t="n">
-        <v>7.331146766698879</v>
-      </c>
-      <c r="BF12" t="n">
-        <v>2.571972157433972</v>
-      </c>
+      <c r="BF12" t="inlineStr"/>
       <c r="BG12" t="n">
         <v>0</v>
       </c>
@@ -2788,54 +2788,54 @@
         <v>0</v>
       </c>
       <c r="T13" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="U13" t="n">
+        <v>8</v>
+      </c>
+      <c r="V13" t="inlineStr"/>
+      <c r="W13" t="inlineStr"/>
+      <c r="X13" t="n">
+        <v>-2</v>
+      </c>
+      <c r="Y13" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z13" t="n">
+        <v>-2.5</v>
+      </c>
+      <c r="AA13" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="AB13" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="AC13" t="n">
+        <v>8</v>
+      </c>
+      <c r="AD13" t="n">
+        <v>1</v>
+      </c>
+      <c r="AE13" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AF13" t="n">
         <v>0.5</v>
       </c>
-      <c r="U13" t="n">
+      <c r="AG13" t="n">
         <v>2.5</v>
       </c>
-      <c r="V13" t="n">
+      <c r="AH13" t="n">
         <v>21.5</v>
       </c>
-      <c r="W13" t="n">
+      <c r="AI13" t="n">
         <v>-21.5</v>
       </c>
-      <c r="X13" t="n">
-        <v>-2.5</v>
-      </c>
-      <c r="Y13" t="n">
-        <v>7.5</v>
-      </c>
-      <c r="Z13" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="AA13" t="n">
-        <v>8</v>
-      </c>
-      <c r="AB13" t="n">
-        <v>1</v>
-      </c>
-      <c r="AC13" t="n">
-        <v>-1</v>
-      </c>
-      <c r="AD13" t="n">
+      <c r="AJ13" t="n">
         <v>1.36</v>
       </c>
-      <c r="AE13" t="n">
+      <c r="AK13" t="n">
         <v>0.665</v>
-      </c>
-      <c r="AF13" t="inlineStr"/>
-      <c r="AG13" t="inlineStr"/>
-      <c r="AH13" t="n">
-        <v>3.5</v>
-      </c>
-      <c r="AI13" t="n">
-        <v>8</v>
-      </c>
-      <c r="AJ13" t="n">
-        <v>-2</v>
-      </c>
-      <c r="AK13" t="n">
-        <v>1</v>
       </c>
       <c r="AL13" t="n">
         <v>71.18181818181819</v>
@@ -2843,49 +2843,49 @@
       <c r="AM13" t="n">
         <v>69.5409090909091</v>
       </c>
-      <c r="AN13" t="n">
+      <c r="AN13" t="inlineStr"/>
+      <c r="AO13" t="n">
+        <v>1776341.991341992</v>
+      </c>
+      <c r="AP13" t="inlineStr"/>
+      <c r="AQ13" t="n">
+        <v>0.0640253202730392</v>
+      </c>
+      <c r="AR13" t="inlineStr"/>
+      <c r="AS13" t="n">
+        <v>-2.962770562770565</v>
+      </c>
+      <c r="AT13" t="n">
+        <v>4.043052003410054</v>
+      </c>
+      <c r="AU13" t="n">
+        <v>4.493073593073603</v>
+      </c>
+      <c r="AV13" t="n">
+        <v>-4.192364047068082</v>
+      </c>
+      <c r="AW13" t="n">
+        <v>1651013.664523781</v>
+      </c>
+      <c r="AX13" t="n">
+        <v>4.433221114532756</v>
+      </c>
+      <c r="AY13" t="n">
         <v>2.123376623376615</v>
       </c>
-      <c r="AO13" t="inlineStr"/>
-      <c r="AP13" t="n">
-        <v>-4.192364047068082</v>
-      </c>
-      <c r="AQ13" t="n">
-        <v>4.433221114532756</v>
-      </c>
-      <c r="AR13" t="n">
-        <v>1651013.664523781</v>
-      </c>
-      <c r="AS13" t="n">
-        <v>1776341.991341992</v>
-      </c>
-      <c r="AT13" t="n">
+      <c r="AZ13" t="inlineStr"/>
+      <c r="BA13" t="inlineStr"/>
+      <c r="BB13" t="n">
+        <v>-3.160173160173173</v>
+      </c>
+      <c r="BC13" t="inlineStr"/>
+      <c r="BD13" t="n">
         <v>0.01481295416717421</v>
       </c>
-      <c r="AU13" t="n">
+      <c r="BE13" t="n">
         <v>0.09220779220779241</v>
       </c>
-      <c r="AV13" t="inlineStr"/>
-      <c r="AW13" t="inlineStr"/>
-      <c r="AX13" t="n">
-        <v>-3.160173160173173</v>
-      </c>
-      <c r="AY13" t="n">
-        <v>-2.962770562770565</v>
-      </c>
-      <c r="AZ13" t="inlineStr"/>
-      <c r="BA13" t="n">
-        <v>4.493073593073603</v>
-      </c>
-      <c r="BB13" t="inlineStr"/>
-      <c r="BC13" t="inlineStr"/>
-      <c r="BD13" t="inlineStr"/>
-      <c r="BE13" t="n">
-        <v>4.043052003410054</v>
-      </c>
-      <c r="BF13" t="n">
-        <v>0.0640253202730392</v>
-      </c>
+      <c r="BF13" t="inlineStr"/>
       <c r="BG13" t="n">
         <v>0</v>
       </c>
@@ -3401,54 +3401,54 @@
         <v>0</v>
       </c>
       <c r="T18" t="n">
-        <v>0</v>
+        <v>-6</v>
       </c>
       <c r="U18" t="n">
+        <v>9</v>
+      </c>
+      <c r="V18" t="inlineStr"/>
+      <c r="W18" t="inlineStr"/>
+      <c r="X18" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y18" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z18" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA18" t="n">
+        <v>-4</v>
+      </c>
+      <c r="AB18" t="n">
+        <v>-5</v>
+      </c>
+      <c r="AC18" t="n">
+        <v>8</v>
+      </c>
+      <c r="AD18" t="n">
+        <v>1</v>
+      </c>
+      <c r="AE18" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF18" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG18" t="n">
         <v>2</v>
       </c>
-      <c r="V18" t="n">
+      <c r="AH18" t="n">
         <v>-21</v>
       </c>
-      <c r="W18" t="n">
+      <c r="AI18" t="n">
         <v>21</v>
       </c>
-      <c r="X18" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y18" t="n">
-        <v>-4</v>
-      </c>
-      <c r="Z18" t="n">
-        <v>-6</v>
-      </c>
-      <c r="AA18" t="n">
-        <v>9</v>
-      </c>
-      <c r="AB18" t="n">
-        <v>1</v>
-      </c>
-      <c r="AC18" t="n">
-        <v>1</v>
-      </c>
-      <c r="AD18" t="n">
+      <c r="AJ18" t="n">
         <v>-1.04</v>
       </c>
-      <c r="AE18" t="n">
+      <c r="AK18" t="n">
         <v>2.73</v>
-      </c>
-      <c r="AF18" t="inlineStr"/>
-      <c r="AG18" t="inlineStr"/>
-      <c r="AH18" t="n">
-        <v>-5</v>
-      </c>
-      <c r="AI18" t="n">
-        <v>8</v>
-      </c>
-      <c r="AJ18" t="n">
-        <v>0</v>
-      </c>
-      <c r="AK18" t="n">
-        <v>0</v>
       </c>
       <c r="AL18" t="n">
         <v>74</v>
@@ -3456,49 +3456,49 @@
       <c r="AM18" t="n">
         <v>69</v>
       </c>
-      <c r="AN18" t="n">
+      <c r="AN18" t="inlineStr"/>
+      <c r="AO18" t="n">
+        <v>-1281253.306878306</v>
+      </c>
+      <c r="AP18" t="inlineStr"/>
+      <c r="AQ18" t="n">
+        <v>1.216519796764572</v>
+      </c>
+      <c r="AR18" t="inlineStr"/>
+      <c r="AS18" t="n">
+        <v>4.621296296296293</v>
+      </c>
+      <c r="AT18" t="n">
+        <v>0.4217652273900256</v>
+      </c>
+      <c r="AU18" t="n">
+        <v>-5.914153439153438</v>
+      </c>
+      <c r="AV18" t="n">
+        <v>0.2953982603720817</v>
+      </c>
+      <c r="AW18" t="n">
+        <v>-130365.5393059938</v>
+      </c>
+      <c r="AX18" t="n">
+        <v>-0.5411850373547225</v>
+      </c>
+      <c r="AY18" t="n">
         <v>0.3376984126984013</v>
       </c>
-      <c r="AO18" t="inlineStr"/>
-      <c r="AP18" t="n">
-        <v>0.2953982603720817</v>
-      </c>
-      <c r="AQ18" t="n">
-        <v>-0.5411850373547225</v>
-      </c>
-      <c r="AR18" t="n">
-        <v>-130365.5393059938</v>
-      </c>
-      <c r="AS18" t="n">
-        <v>-1281253.306878306</v>
-      </c>
-      <c r="AT18" t="n">
-        <v>0</v>
-      </c>
-      <c r="AU18" t="n">
-        <v>0</v>
-      </c>
-      <c r="AV18" t="inlineStr"/>
-      <c r="AW18" t="inlineStr"/>
-      <c r="AX18" t="n">
+      <c r="AZ18" t="inlineStr"/>
+      <c r="BA18" t="inlineStr"/>
+      <c r="BB18" t="n">
         <v>1.906944444444434</v>
       </c>
-      <c r="AY18" t="n">
-        <v>4.621296296296293</v>
-      </c>
-      <c r="AZ18" t="inlineStr"/>
-      <c r="BA18" t="n">
-        <v>-5.914153439153438</v>
-      </c>
-      <c r="BB18" t="inlineStr"/>
       <c r="BC18" t="inlineStr"/>
-      <c r="BD18" t="inlineStr"/>
+      <c r="BD18" t="n">
+        <v>0</v>
+      </c>
       <c r="BE18" t="n">
-        <v>0.4217652273900256</v>
-      </c>
-      <c r="BF18" t="n">
-        <v>1.216519796764572</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="BF18" t="inlineStr"/>
       <c r="BG18" t="n">
         <v>0</v>
       </c>
@@ -5044,54 +5044,54 @@
         <v>0</v>
       </c>
       <c r="T33" t="n">
+        <v>7</v>
+      </c>
+      <c r="U33" t="n">
+        <v>-24</v>
+      </c>
+      <c r="V33" t="inlineStr"/>
+      <c r="W33" t="inlineStr"/>
+      <c r="X33" t="n">
         <v>2</v>
       </c>
-      <c r="U33" t="n">
-        <v>0</v>
-      </c>
-      <c r="V33" t="n">
+      <c r="Y33" t="n">
+        <v>-1</v>
+      </c>
+      <c r="Z33" t="n">
+        <v>-4</v>
+      </c>
+      <c r="AA33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB33" t="n">
+        <v>4</v>
+      </c>
+      <c r="AC33" t="n">
+        <v>-6</v>
+      </c>
+      <c r="AD33" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AE33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF33" t="n">
+        <v>2</v>
+      </c>
+      <c r="AG33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH33" t="n">
         <v>21</v>
       </c>
-      <c r="W33" t="n">
+      <c r="AI33" t="n">
         <v>-21</v>
       </c>
-      <c r="X33" t="n">
-        <v>-4</v>
-      </c>
-      <c r="Y33" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z33" t="n">
-        <v>7</v>
-      </c>
-      <c r="AA33" t="n">
-        <v>-24</v>
-      </c>
-      <c r="AB33" t="n">
-        <v>-1</v>
-      </c>
-      <c r="AC33" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD33" t="n">
+      <c r="AJ33" t="n">
         <v>1.61</v>
       </c>
-      <c r="AE33" t="n">
+      <c r="AK33" t="n">
         <v>-1.41</v>
-      </c>
-      <c r="AF33" t="inlineStr"/>
-      <c r="AG33" t="inlineStr"/>
-      <c r="AH33" t="n">
-        <v>4</v>
-      </c>
-      <c r="AI33" t="n">
-        <v>-6</v>
-      </c>
-      <c r="AJ33" t="n">
-        <v>2</v>
-      </c>
-      <c r="AK33" t="n">
-        <v>-1</v>
       </c>
       <c r="AL33" t="n">
         <v>66.2</v>
@@ -5099,49 +5099,49 @@
       <c r="AM33" t="n">
         <v>70.18181818181819</v>
       </c>
-      <c r="AN33" t="n">
+      <c r="AN33" t="inlineStr"/>
+      <c r="AO33" t="n">
+        <v>-2234641.203703703</v>
+      </c>
+      <c r="AP33" t="inlineStr"/>
+      <c r="AQ33" t="n">
+        <v>1.301905073233439</v>
+      </c>
+      <c r="AR33" t="inlineStr"/>
+      <c r="AS33" t="n">
+        <v>-0.5010416666666657</v>
+      </c>
+      <c r="AT33" t="n">
+        <v>-2.202103660443441</v>
+      </c>
+      <c r="AU33" t="n">
+        <v>-2.82534722222222</v>
+      </c>
+      <c r="AV33" t="n">
+        <v>-0.2023692810457476</v>
+      </c>
+      <c r="AW33" t="n">
+        <v>-1269591.292981506</v>
+      </c>
+      <c r="AX33" t="n">
+        <v>-2.49301163447835</v>
+      </c>
+      <c r="AY33" t="n">
         <v>-2.816666666666649</v>
       </c>
-      <c r="AO33" t="inlineStr"/>
-      <c r="AP33" t="n">
-        <v>-0.2023692810457476</v>
-      </c>
-      <c r="AQ33" t="n">
-        <v>-2.49301163447835</v>
-      </c>
-      <c r="AR33" t="n">
-        <v>-1269591.292981506</v>
-      </c>
-      <c r="AS33" t="n">
-        <v>-2234641.203703703</v>
-      </c>
-      <c r="AT33" t="n">
-        <v>0</v>
-      </c>
-      <c r="AU33" t="n">
-        <v>0</v>
-      </c>
-      <c r="AV33" t="inlineStr"/>
-      <c r="AW33" t="inlineStr"/>
-      <c r="AX33" t="n">
+      <c r="AZ33" t="inlineStr"/>
+      <c r="BA33" t="inlineStr"/>
+      <c r="BB33" t="n">
         <v>-1.420370370370335</v>
       </c>
-      <c r="AY33" t="n">
-        <v>-0.5010416666666657</v>
-      </c>
-      <c r="AZ33" t="inlineStr"/>
-      <c r="BA33" t="n">
-        <v>-2.82534722222222</v>
-      </c>
-      <c r="BB33" t="inlineStr"/>
       <c r="BC33" t="inlineStr"/>
-      <c r="BD33" t="inlineStr"/>
+      <c r="BD33" t="n">
+        <v>0</v>
+      </c>
       <c r="BE33" t="n">
-        <v>-2.202103660443441</v>
-      </c>
-      <c r="BF33" t="n">
-        <v>1.301905073233439</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="BF33" t="inlineStr"/>
       <c r="BG33" t="n">
         <v>0</v>
       </c>
@@ -6589,54 +6589,54 @@
         <v>0</v>
       </c>
       <c r="T47" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="U47" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="V47" t="inlineStr"/>
+      <c r="W47" t="inlineStr"/>
+      <c r="X47" t="n">
+        <v>-1.25</v>
+      </c>
+      <c r="Y47" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z47" t="n">
+        <v>2.25</v>
+      </c>
+      <c r="AA47" t="n">
+        <v>-2</v>
+      </c>
+      <c r="AB47" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC47" t="n">
+        <v>3.25</v>
+      </c>
+      <c r="AD47" t="n">
+        <v>1</v>
+      </c>
+      <c r="AE47" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="AF47" t="n">
         <v>-1</v>
       </c>
-      <c r="U47" t="n">
+      <c r="AG47" t="n">
         <v>1.5</v>
       </c>
-      <c r="V47" t="n">
+      <c r="AH47" t="n">
         <v>-7</v>
       </c>
-      <c r="W47" t="n">
+      <c r="AI47" t="n">
         <v>7</v>
       </c>
-      <c r="X47" t="n">
-        <v>2.25</v>
-      </c>
-      <c r="Y47" t="n">
-        <v>-2</v>
-      </c>
-      <c r="Z47" t="n">
-        <v>8.5</v>
-      </c>
-      <c r="AA47" t="n">
-        <v>6.5</v>
-      </c>
-      <c r="AB47" t="n">
-        <v>1</v>
-      </c>
-      <c r="AC47" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="AD47" t="n">
+      <c r="AJ47" t="n">
         <v>0.1174999999999999</v>
       </c>
-      <c r="AE47" t="n">
+      <c r="AK47" t="n">
         <v>0.5950000000000002</v>
-      </c>
-      <c r="AF47" t="inlineStr"/>
-      <c r="AG47" t="inlineStr"/>
-      <c r="AH47" t="n">
-        <v>2</v>
-      </c>
-      <c r="AI47" t="n">
-        <v>3.25</v>
-      </c>
-      <c r="AJ47" t="n">
-        <v>-1.25</v>
-      </c>
-      <c r="AK47" t="n">
-        <v>1</v>
       </c>
       <c r="AL47" t="n">
         <v>76.15625</v>
@@ -6644,49 +6644,49 @@
       <c r="AM47" t="n">
         <v>77.36540404040404</v>
       </c>
-      <c r="AN47" t="n">
+      <c r="AN47" t="inlineStr"/>
+      <c r="AO47" t="n">
+        <v>-43592483.9302112</v>
+      </c>
+      <c r="AP47" t="inlineStr"/>
+      <c r="AQ47" t="n">
+        <v>-0.6387726578234556</v>
+      </c>
+      <c r="AR47" t="inlineStr"/>
+      <c r="AS47" t="n">
+        <v>-1.885417814508717</v>
+      </c>
+      <c r="AT47" t="n">
+        <v>-5.74893747653573</v>
+      </c>
+      <c r="AU47" t="n">
+        <v>-3.136501377410468</v>
+      </c>
+      <c r="AV47" t="n">
+        <v>5.572761884128397</v>
+      </c>
+      <c r="AW47" t="n">
+        <v>-27821847.68622385</v>
+      </c>
+      <c r="AX47" t="n">
+        <v>-3.786451794156378</v>
+      </c>
+      <c r="AY47" t="n">
         <v>-5.649201101928398</v>
       </c>
-      <c r="AO47" t="inlineStr"/>
-      <c r="AP47" t="n">
-        <v>5.572761884128397</v>
-      </c>
-      <c r="AQ47" t="n">
-        <v>-3.786451794156378</v>
-      </c>
-      <c r="AR47" t="n">
-        <v>-27821847.68622385</v>
-      </c>
-      <c r="AS47" t="n">
-        <v>-43592483.9302112</v>
-      </c>
-      <c r="AT47" t="n">
+      <c r="AZ47" t="inlineStr"/>
+      <c r="BA47" t="inlineStr"/>
+      <c r="BB47" t="n">
+        <v>2.633526170798888</v>
+      </c>
+      <c r="BC47" t="inlineStr"/>
+      <c r="BD47" t="n">
         <v>-0.4920997390452169</v>
       </c>
-      <c r="AU47" t="n">
+      <c r="BE47" t="n">
         <v>-0.9389256198347109</v>
       </c>
-      <c r="AV47" t="inlineStr"/>
-      <c r="AW47" t="inlineStr"/>
-      <c r="AX47" t="n">
-        <v>2.633526170798888</v>
-      </c>
-      <c r="AY47" t="n">
-        <v>-1.885417814508717</v>
-      </c>
-      <c r="AZ47" t="inlineStr"/>
-      <c r="BA47" t="n">
-        <v>-3.136501377410468</v>
-      </c>
-      <c r="BB47" t="inlineStr"/>
-      <c r="BC47" t="inlineStr"/>
-      <c r="BD47" t="inlineStr"/>
-      <c r="BE47" t="n">
-        <v>-5.74893747653573</v>
-      </c>
-      <c r="BF47" t="n">
-        <v>-0.6387726578234556</v>
-      </c>
+      <c r="BF47" t="inlineStr"/>
       <c r="BG47" t="n">
         <v>1</v>
       </c>

</xml_diff>

<commit_message>
Actualizo predicciones.xlsx al usar nuevos m_to_use.
</commit_message>
<xml_diff>
--- a/data/england/p6_deployment/data_preparation/df_constructed.xlsx
+++ b/data/england/p6_deployment/data_preparation/df_constructed.xlsx
@@ -535,84 +535,84 @@
       </c>
       <c r="V1" s="1" t="inlineStr">
         <is>
+          <t>dif_mean_last_match_interceptions</t>
+        </is>
+      </c>
+      <c r="W1" s="1" t="inlineStr">
+        <is>
+          <t>dif_mean_last_match_interceptions_against</t>
+        </is>
+      </c>
+      <c r="X1" s="1" t="inlineStr">
+        <is>
+          <t>dif_mean_last_match_fouls</t>
+        </is>
+      </c>
+      <c r="Y1" s="1" t="inlineStr">
+        <is>
+          <t>dif_mean_last_match_fouls_against</t>
+        </is>
+      </c>
+      <c r="Z1" s="1" t="inlineStr">
+        <is>
           <t>dif_mean_last_match_points</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="AA1" s="1" t="inlineStr">
         <is>
           <t>dif_mean_last_match_points_against</t>
         </is>
       </c>
-      <c r="X1" s="1" t="inlineStr">
+      <c r="AB1" s="1" t="inlineStr">
+        <is>
+          <t>dif_mean_last_match_shots_on_goal</t>
+        </is>
+      </c>
+      <c r="AC1" s="1" t="inlineStr">
+        <is>
+          <t>dif_mean_last_match_shots_on_goal_against</t>
+        </is>
+      </c>
+      <c r="AD1" s="1" t="inlineStr">
+        <is>
+          <t>dif_mean_last_match_goals</t>
+        </is>
+      </c>
+      <c r="AE1" s="1" t="inlineStr">
+        <is>
+          <t>dif_mean_last_match_goals_against</t>
+        </is>
+      </c>
+      <c r="AF1" s="1" t="inlineStr">
+        <is>
+          <t>dif_mean_last_match_n_matches_last_days</t>
+        </is>
+      </c>
+      <c r="AG1" s="1" t="inlineStr">
+        <is>
+          <t>dif_mean_last_match_n_matches_last_days_against</t>
+        </is>
+      </c>
+      <c r="AH1" s="1" t="inlineStr">
         <is>
           <t>dif_mean_last_match_expected_goals_(xg)</t>
         </is>
       </c>
-      <c r="Y1" s="1" t="inlineStr">
+      <c r="AI1" s="1" t="inlineStr">
         <is>
           <t>dif_mean_last_match_expected_goals_(xg)_against</t>
         </is>
       </c>
-      <c r="Z1" s="1" t="inlineStr">
+      <c r="AJ1" s="1" t="inlineStr">
         <is>
           <t>dif_mean_last_match_goal_attempts</t>
         </is>
       </c>
-      <c r="AA1" s="1" t="inlineStr">
+      <c r="AK1" s="1" t="inlineStr">
         <is>
           <t>dif_mean_last_match_goal_attempts_against</t>
         </is>
       </c>
-      <c r="AB1" s="1" t="inlineStr">
-        <is>
-          <t>dif_mean_last_match_goals</t>
-        </is>
-      </c>
-      <c r="AC1" s="1" t="inlineStr">
-        <is>
-          <t>dif_mean_last_match_goals_against</t>
-        </is>
-      </c>
-      <c r="AD1" s="1" t="inlineStr">
-        <is>
-          <t>dif_mean_last_match_n_matches_last_days</t>
-        </is>
-      </c>
-      <c r="AE1" s="1" t="inlineStr">
-        <is>
-          <t>dif_mean_last_match_n_matches_last_days_against</t>
-        </is>
-      </c>
-      <c r="AF1" s="1" t="inlineStr">
-        <is>
-          <t>dif_mean_last_match_interceptions</t>
-        </is>
-      </c>
-      <c r="AG1" s="1" t="inlineStr">
-        <is>
-          <t>dif_mean_last_match_interceptions_against</t>
-        </is>
-      </c>
-      <c r="AH1" s="1" t="inlineStr">
-        <is>
-          <t>dif_mean_last_match_shots_on_goal</t>
-        </is>
-      </c>
-      <c r="AI1" s="1" t="inlineStr">
-        <is>
-          <t>dif_mean_last_match_shots_on_goal_against</t>
-        </is>
-      </c>
-      <c r="AJ1" s="1" t="inlineStr">
-        <is>
-          <t>dif_mean_last_match_fouls</t>
-        </is>
-      </c>
-      <c r="AK1" s="1" t="inlineStr">
-        <is>
-          <t>dif_mean_last_match_fouls_against</t>
-        </is>
-      </c>
       <c r="AL1" s="1" t="inlineStr">
         <is>
           <t>mean_last_match_mean_rat_player_start_home_against</t>
@@ -625,92 +625,92 @@
       </c>
       <c r="AN1" s="1" t="inlineStr">
         <is>
+          <t>dif_sum_rat_player_miss</t>
+        </is>
+      </c>
+      <c r="AO1" s="1" t="inlineStr">
+        <is>
+          <t>dif_mean_rat_player_sub</t>
+        </is>
+      </c>
+      <c r="AP1" s="1" t="inlineStr">
+        <is>
+          <t>dif_mean_int_rep_player_sub</t>
+        </is>
+      </c>
+      <c r="AQ1" s="1" t="inlineStr">
+        <is>
+          <t>dif_n_player_miss</t>
+        </is>
+      </c>
+      <c r="AR1" s="1" t="inlineStr">
+        <is>
+          <t>dif_mean_age_player_start</t>
+        </is>
+      </c>
+      <c r="AS1" s="1" t="inlineStr">
+        <is>
+          <t>dif_sum_val_player_miss</t>
+        </is>
+      </c>
+      <c r="AT1" s="1" t="inlineStr">
+        <is>
           <t>dif_mean_age_player_sub</t>
         </is>
       </c>
-      <c r="AO1" s="1" t="inlineStr">
+      <c r="AU1" s="1" t="inlineStr">
+        <is>
+          <t>dif_mean_pot_player_start</t>
+        </is>
+      </c>
+      <c r="AV1" s="1" t="inlineStr">
+        <is>
+          <t>dif_mean_rat_player_start</t>
+        </is>
+      </c>
+      <c r="AW1" s="1" t="inlineStr">
+        <is>
+          <t>dif_mean_pot_player_sub</t>
+        </is>
+      </c>
+      <c r="AX1" s="1" t="inlineStr">
+        <is>
+          <t>dif_mean_val_player_start</t>
+        </is>
+      </c>
+      <c r="AY1" s="1" t="inlineStr">
         <is>
           <t>dif_mean_int_rep_player_start</t>
         </is>
       </c>
-      <c r="AP1" s="1" t="inlineStr">
-        <is>
-          <t>dif_sum_val_player_miss</t>
-        </is>
-      </c>
-      <c r="AQ1" s="1" t="inlineStr">
+      <c r="AZ1" s="1" t="inlineStr">
+        <is>
+          <t>dif_mean_val_player_sub</t>
+        </is>
+      </c>
+      <c r="BA1" s="1" t="inlineStr">
+        <is>
+          <t>dif_mean_age_player_miss</t>
+        </is>
+      </c>
+      <c r="BB1" s="1" t="inlineStr">
+        <is>
+          <t>dif_mean_hei_player_start</t>
+        </is>
+      </c>
+      <c r="BC1" s="1" t="inlineStr">
+        <is>
+          <t>dif_mean_hei_player_sub</t>
+        </is>
+      </c>
+      <c r="BD1" s="1" t="inlineStr">
         <is>
           <t>dif_mean_hei_player_miss</t>
         </is>
       </c>
-      <c r="AR1" s="1" t="inlineStr">
-        <is>
-          <t>dif_mean_age_player_start</t>
-        </is>
-      </c>
-      <c r="AS1" s="1" t="inlineStr">
-        <is>
-          <t>dif_mean_hei_player_start</t>
-        </is>
-      </c>
-      <c r="AT1" s="1" t="inlineStr">
-        <is>
-          <t>dif_n_player_miss</t>
-        </is>
-      </c>
-      <c r="AU1" s="1" t="inlineStr">
+      <c r="BE1" s="1" t="inlineStr">
         <is>
           <t>dif_sum_pot_player_miss</t>
-        </is>
-      </c>
-      <c r="AV1" s="1" t="inlineStr">
-        <is>
-          <t>dif_mean_age_player_miss</t>
-        </is>
-      </c>
-      <c r="AW1" s="1" t="inlineStr">
-        <is>
-          <t>dif_mean_val_player_sub</t>
-        </is>
-      </c>
-      <c r="AX1" s="1" t="inlineStr">
-        <is>
-          <t>dif_mean_pot_player_start</t>
-        </is>
-      </c>
-      <c r="AY1" s="1" t="inlineStr">
-        <is>
-          <t>dif_mean_rat_player_start</t>
-        </is>
-      </c>
-      <c r="AZ1" s="1" t="inlineStr">
-        <is>
-          <t>dif_mean_int_rep_player_sub</t>
-        </is>
-      </c>
-      <c r="BA1" s="1" t="inlineStr">
-        <is>
-          <t>dif_mean_pot_player_sub</t>
-        </is>
-      </c>
-      <c r="BB1" s="1" t="inlineStr">
-        <is>
-          <t>dif_mean_val_player_start</t>
-        </is>
-      </c>
-      <c r="BC1" s="1" t="inlineStr">
-        <is>
-          <t>dif_sum_rat_player_miss</t>
-        </is>
-      </c>
-      <c r="BD1" s="1" t="inlineStr">
-        <is>
-          <t>dif_mean_hei_player_sub</t>
-        </is>
-      </c>
-      <c r="BE1" s="1" t="inlineStr">
-        <is>
-          <t>dif_mean_rat_player_sub</t>
         </is>
       </c>
       <c r="BF1" s="1" t="inlineStr">
@@ -808,49 +808,49 @@
       <c r="U2" t="n">
         <v>9.5</v>
       </c>
-      <c r="V2" t="n">
-        <v>0</v>
-      </c>
-      <c r="W2" t="n">
+      <c r="V2" t="inlineStr"/>
+      <c r="W2" t="inlineStr"/>
+      <c r="X2" t="n">
+        <v>-5.5</v>
+      </c>
+      <c r="Y2" t="n">
+        <v>-2.333333333333333</v>
+      </c>
+      <c r="Z2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA2" t="n">
         <v>0.5</v>
       </c>
-      <c r="X2" t="n">
+      <c r="AB2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AC2" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="AD2" t="n">
+        <v>-1.166666666666667</v>
+      </c>
+      <c r="AE2" t="n">
+        <v>-0.5</v>
+      </c>
+      <c r="AF2" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="AG2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AH2" t="n">
         <v>-0.5183333333333331</v>
       </c>
-      <c r="Y2" t="n">
+      <c r="AI2" t="n">
         <v>-0.5916666666666666</v>
       </c>
-      <c r="Z2" t="n">
+      <c r="AJ2" t="n">
         <v>-1</v>
       </c>
-      <c r="AA2" t="n">
+      <c r="AK2" t="n">
         <v>1</v>
-      </c>
-      <c r="AB2" t="n">
-        <v>-1.166666666666667</v>
-      </c>
-      <c r="AC2" t="n">
-        <v>-0.5</v>
-      </c>
-      <c r="AD2" t="n">
-        <v>0.3333333333333333</v>
-      </c>
-      <c r="AE2" t="n">
-        <v>1</v>
-      </c>
-      <c r="AF2" t="inlineStr"/>
-      <c r="AG2" t="inlineStr"/>
-      <c r="AH2" t="n">
-        <v>-1</v>
-      </c>
-      <c r="AI2" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="AJ2" t="n">
-        <v>-5.5</v>
-      </c>
-      <c r="AK2" t="n">
-        <v>-2.333333333333333</v>
       </c>
       <c r="AL2" t="n">
         <v>79.09318181818182</v>
@@ -858,48 +858,48 @@
       <c r="AM2" t="n">
         <v>76.54545454545455</v>
       </c>
-      <c r="AN2" t="n">
-        <v>0.9561994712921837</v>
-      </c>
+      <c r="AN2" t="inlineStr"/>
       <c r="AO2" t="n">
-        <v>-0.3611616161616165</v>
-      </c>
-      <c r="AP2" t="inlineStr"/>
+        <v>-4.100489453830249</v>
+      </c>
+      <c r="AP2" t="n">
+        <v>0.07133485215646318</v>
+      </c>
       <c r="AQ2" t="inlineStr"/>
       <c r="AR2" t="n">
         <v>-0.9009932659932609</v>
       </c>
-      <c r="AS2" t="n">
+      <c r="AS2" t="inlineStr"/>
+      <c r="AT2" t="n">
+        <v>0.9561994712921837</v>
+      </c>
+      <c r="AU2" t="n">
+        <v>-1.269360269360263</v>
+      </c>
+      <c r="AV2" t="n">
+        <v>-2.887962962962973</v>
+      </c>
+      <c r="AW2" t="n">
+        <v>-2.946957639428859</v>
+      </c>
+      <c r="AX2" t="n">
+        <v>-17129304.71380471</v>
+      </c>
+      <c r="AY2" t="n">
+        <v>-0.3611616161616165</v>
+      </c>
+      <c r="AZ2" t="n">
+        <v>-15032471.45984167</v>
+      </c>
+      <c r="BA2" t="inlineStr"/>
+      <c r="BB2" t="n">
         <v>1.140286195286194</v>
       </c>
-      <c r="AT2" t="inlineStr"/>
-      <c r="AU2" t="inlineStr"/>
-      <c r="AV2" t="inlineStr"/>
-      <c r="AW2" t="n">
-        <v>-15032471.45984167</v>
-      </c>
-      <c r="AX2" t="n">
-        <v>-1.269360269360263</v>
-      </c>
-      <c r="AY2" t="n">
-        <v>-2.887962962962973</v>
-      </c>
-      <c r="AZ2" t="n">
-        <v>0.07133485215646318</v>
-      </c>
-      <c r="BA2" t="n">
-        <v>-2.946957639428859</v>
-      </c>
-      <c r="BB2" t="n">
-        <v>-17129304.71380471</v>
-      </c>
-      <c r="BC2" t="inlineStr"/>
-      <c r="BD2" t="n">
+      <c r="BC2" t="n">
         <v>0.7296165115315034</v>
       </c>
-      <c r="BE2" t="n">
-        <v>-4.100489453830249</v>
-      </c>
+      <c r="BD2" t="inlineStr"/>
+      <c r="BE2" t="inlineStr"/>
       <c r="BF2" t="inlineStr"/>
       <c r="BG2" t="n">
         <v>1</v>
@@ -989,49 +989,49 @@
       <c r="U3" t="n">
         <v>29.66666666666667</v>
       </c>
-      <c r="V3" t="n">
+      <c r="V3" t="inlineStr"/>
+      <c r="W3" t="inlineStr"/>
+      <c r="X3" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y3" t="n">
+        <v>4</v>
+      </c>
+      <c r="Z3" t="n">
         <v>0.6666666666666667</v>
       </c>
-      <c r="W3" t="n">
+      <c r="AA3" t="n">
         <v>-0.8333333333333333</v>
       </c>
-      <c r="X3" t="n">
-        <v>-0.5516666666666667</v>
-      </c>
-      <c r="Y3" t="n">
-        <v>-0.5766666666666669</v>
-      </c>
-      <c r="Z3" t="n">
-        <v>-4.166666666666666</v>
-      </c>
-      <c r="AA3" t="n">
-        <v>4.333333333333334</v>
-      </c>
       <c r="AB3" t="n">
-        <v>-1</v>
+        <v>-3</v>
       </c>
       <c r="AC3" t="n">
         <v>-1.166666666666667</v>
       </c>
       <c r="AD3" t="n">
-        <v>-2.5</v>
+        <v>-1</v>
       </c>
       <c r="AE3" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF3" t="inlineStr"/>
-      <c r="AG3" t="inlineStr"/>
+        <v>-1.166666666666667</v>
+      </c>
+      <c r="AF3" t="n">
+        <v>-1.5</v>
+      </c>
+      <c r="AG3" t="n">
+        <v>-1</v>
+      </c>
       <c r="AH3" t="n">
-        <v>-3</v>
+        <v>-0.5516666666666667</v>
       </c>
       <c r="AI3" t="n">
-        <v>-1.166666666666667</v>
+        <v>-0.5766666666666669</v>
       </c>
       <c r="AJ3" t="n">
-        <v>1</v>
+        <v>-4.166666666666666</v>
       </c>
       <c r="AK3" t="n">
-        <v>4</v>
+        <v>4.333333333333334</v>
       </c>
       <c r="AL3" t="n">
         <v>74.30555555555556</v>
@@ -1039,48 +1039,48 @@
       <c r="AM3" t="n">
         <v>76.88484848484848</v>
       </c>
-      <c r="AN3" t="n">
-        <v>1.891513343109708</v>
-      </c>
+      <c r="AN3" t="inlineStr"/>
       <c r="AO3" t="n">
-        <v>-0.5641624579124578</v>
-      </c>
-      <c r="AP3" t="inlineStr"/>
+        <v>-4.246734762485531</v>
+      </c>
+      <c r="AP3" t="n">
+        <v>-0.3514529974669298</v>
+      </c>
       <c r="AQ3" t="inlineStr"/>
       <c r="AR3" t="n">
-        <v>1.434911616161614</v>
-      </c>
-      <c r="AS3" t="n">
-        <v>0.834196127946143</v>
-      </c>
-      <c r="AT3" t="inlineStr"/>
-      <c r="AU3" t="inlineStr"/>
-      <c r="AV3" t="inlineStr"/>
+        <v>1.367125803489436</v>
+      </c>
+      <c r="AS3" t="inlineStr"/>
+      <c r="AT3" t="n">
+        <v>2.042807944549427</v>
+      </c>
+      <c r="AU3" t="n">
+        <v>-4.130670339761267</v>
+      </c>
+      <c r="AV3" t="n">
+        <v>-3.651331496786028</v>
+      </c>
       <c r="AW3" t="n">
-        <v>-14486552.70163953</v>
+        <v>-3.873556384276185</v>
       </c>
       <c r="AX3" t="n">
-        <v>-4.127882996633005</v>
+        <v>-19684692.37832875</v>
       </c>
       <c r="AY3" t="n">
-        <v>-3.608627946127939</v>
+        <v>-0.5510560146923782</v>
       </c>
       <c r="AZ3" t="n">
-        <v>-0.367619793132564</v>
-      </c>
-      <c r="BA3" t="n">
-        <v>-3.959850928010752</v>
-      </c>
+        <v>-13826652.53401999</v>
+      </c>
+      <c r="BA3" t="inlineStr"/>
       <c r="BB3" t="n">
-        <v>-19809116.16161617</v>
-      </c>
-      <c r="BC3" t="inlineStr"/>
-      <c r="BD3" t="n">
-        <v>-0.4466180072507768</v>
-      </c>
-      <c r="BE3" t="n">
-        <v>-4.411779592884471</v>
-      </c>
+        <v>0.633516988062496</v>
+      </c>
+      <c r="BC3" t="n">
+        <v>-0.2640791484057843</v>
+      </c>
+      <c r="BD3" t="inlineStr"/>
+      <c r="BE3" t="inlineStr"/>
       <c r="BF3" t="inlineStr"/>
       <c r="BG3" t="n">
         <v>0</v>
@@ -1170,49 +1170,49 @@
       <c r="U4" t="n">
         <v>-14</v>
       </c>
-      <c r="V4" t="n">
+      <c r="V4" t="inlineStr"/>
+      <c r="W4" t="inlineStr"/>
+      <c r="X4" t="n">
+        <v>-3.833333333333334</v>
+      </c>
+      <c r="Y4" t="n">
+        <v>-0.1666666666666661</v>
+      </c>
+      <c r="Z4" t="n">
         <v>0.5</v>
       </c>
-      <c r="W4" t="n">
+      <c r="AA4" t="n">
         <v>-0.5</v>
       </c>
-      <c r="X4" t="n">
+      <c r="AB4" t="n">
+        <v>3.166666666666667</v>
+      </c>
+      <c r="AC4" t="n">
+        <v>-2.5</v>
+      </c>
+      <c r="AD4" t="n">
+        <v>0.3333333333333335</v>
+      </c>
+      <c r="AE4" t="n">
+        <v>-0.5</v>
+      </c>
+      <c r="AF4" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="AG4" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AH4" t="n">
         <v>-0.08666666666666689</v>
       </c>
-      <c r="Y4" t="n">
+      <c r="AI4" t="n">
         <v>0.02333333333333343</v>
       </c>
-      <c r="Z4" t="n">
+      <c r="AJ4" t="n">
         <v>3.5</v>
       </c>
-      <c r="AA4" t="n">
+      <c r="AK4" t="n">
         <v>3.833333333333334</v>
-      </c>
-      <c r="AB4" t="n">
-        <v>0.3333333333333335</v>
-      </c>
-      <c r="AC4" t="n">
-        <v>-0.5</v>
-      </c>
-      <c r="AD4" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="AE4" t="n">
-        <v>1</v>
-      </c>
-      <c r="AF4" t="inlineStr"/>
-      <c r="AG4" t="inlineStr"/>
-      <c r="AH4" t="n">
-        <v>3.166666666666667</v>
-      </c>
-      <c r="AI4" t="n">
-        <v>-2.5</v>
-      </c>
-      <c r="AJ4" t="n">
-        <v>-3.833333333333334</v>
-      </c>
-      <c r="AK4" t="n">
-        <v>-0.1666666666666661</v>
       </c>
       <c r="AL4" t="n">
         <v>79.92727272727274</v>
@@ -1220,48 +1220,48 @@
       <c r="AM4" t="n">
         <v>76.13636363636363</v>
       </c>
-      <c r="AN4" t="n">
-        <v>-3.578898649520781</v>
-      </c>
+      <c r="AN4" t="inlineStr"/>
       <c r="AO4" t="n">
-        <v>0.4234848484848477</v>
-      </c>
-      <c r="AP4" t="inlineStr"/>
+        <v>0.8923741410345514</v>
+      </c>
+      <c r="AP4" t="n">
+        <v>0.447302868339321</v>
+      </c>
       <c r="AQ4" t="inlineStr"/>
       <c r="AR4" t="n">
-        <v>-2.445021645021647</v>
-      </c>
-      <c r="AS4" t="n">
-        <v>-0.7196608946608762</v>
-      </c>
-      <c r="AT4" t="inlineStr"/>
-      <c r="AU4" t="inlineStr"/>
-      <c r="AV4" t="inlineStr"/>
+        <v>-2.317376562831107</v>
+      </c>
+      <c r="AS4" t="inlineStr"/>
+      <c r="AT4" t="n">
+        <v>-3.518690613447909</v>
+      </c>
+      <c r="AU4" t="n">
+        <v>3.320039556403202</v>
+      </c>
+      <c r="AV4" t="n">
+        <v>1.501758847213395</v>
+      </c>
       <c r="AW4" t="n">
-        <v>9117255.802554879</v>
+        <v>4.994443970670829</v>
       </c>
       <c r="AX4" t="n">
-        <v>3.408189033189046</v>
+        <v>7332867.839231472</v>
       </c>
       <c r="AY4" t="n">
-        <v>1.520562770562748</v>
+        <v>0.4229285865649497</v>
       </c>
       <c r="AZ4" t="n">
-        <v>0.4678853967278431</v>
-      </c>
-      <c r="BA4" t="n">
-        <v>5.111238717999683</v>
-      </c>
+        <v>8992198.521931197</v>
+      </c>
+      <c r="BA4" t="inlineStr"/>
       <c r="BB4" t="n">
-        <v>7717687.590187585</v>
-      </c>
-      <c r="BC4" t="inlineStr"/>
-      <c r="BD4" t="n">
-        <v>-1.020454848325983</v>
-      </c>
-      <c r="BE4" t="n">
-        <v>0.9069109447269739</v>
-      </c>
+        <v>-0.631058840149791</v>
+      </c>
+      <c r="BC4" t="n">
+        <v>-1.078183194026025</v>
+      </c>
+      <c r="BD4" t="inlineStr"/>
+      <c r="BE4" t="inlineStr"/>
       <c r="BF4" t="inlineStr"/>
       <c r="BG4" t="n">
         <v>0</v>
@@ -1351,49 +1351,49 @@
       <c r="U5" t="n">
         <v>0.1666666666666643</v>
       </c>
-      <c r="V5" t="n">
+      <c r="V5" t="inlineStr"/>
+      <c r="W5" t="inlineStr"/>
+      <c r="X5" t="n">
+        <v>4.833333333333334</v>
+      </c>
+      <c r="Y5" t="n">
+        <v>1.333333333333334</v>
+      </c>
+      <c r="Z5" t="n">
         <v>-1.5</v>
       </c>
-      <c r="W5" t="n">
+      <c r="AA5" t="n">
         <v>1.5</v>
       </c>
-      <c r="X5" t="n">
+      <c r="AB5" t="n">
+        <v>-0.833333333333333</v>
+      </c>
+      <c r="AC5" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AD5" t="n">
+        <v>-0.6666666666666665</v>
+      </c>
+      <c r="AE5" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="AF5" t="n">
+        <v>-0.3333333333333333</v>
+      </c>
+      <c r="AG5" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AH5" t="n">
         <v>-0.04666666666666663</v>
       </c>
-      <c r="Y5" t="n">
+      <c r="AI5" t="n">
         <v>0.4083333333333333</v>
       </c>
-      <c r="Z5" t="n">
+      <c r="AJ5" t="n">
         <v>7.333333333333334</v>
       </c>
-      <c r="AA5" t="n">
+      <c r="AK5" t="n">
         <v>2.5</v>
-      </c>
-      <c r="AB5" t="n">
-        <v>-0.6666666666666665</v>
-      </c>
-      <c r="AC5" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="AD5" t="n">
-        <v>-1</v>
-      </c>
-      <c r="AE5" t="n">
-        <v>-1.5</v>
-      </c>
-      <c r="AF5" t="inlineStr"/>
-      <c r="AG5" t="inlineStr"/>
-      <c r="AH5" t="n">
-        <v>-0.833333333333333</v>
-      </c>
-      <c r="AI5" t="n">
-        <v>-1</v>
-      </c>
-      <c r="AJ5" t="n">
-        <v>4.833333333333334</v>
-      </c>
-      <c r="AK5" t="n">
-        <v>1.333333333333334</v>
       </c>
       <c r="AL5" t="n">
         <v>76.21363636363637</v>
@@ -1401,48 +1401,48 @@
       <c r="AM5" t="n">
         <v>79.17508417508417</v>
       </c>
-      <c r="AN5" t="n">
-        <v>2.585834908052345</v>
-      </c>
+      <c r="AN5" t="inlineStr"/>
       <c r="AO5" t="n">
-        <v>-0.9612304866850319</v>
-      </c>
-      <c r="AP5" t="inlineStr"/>
+        <v>-6.059816536986247</v>
+      </c>
+      <c r="AP5" t="n">
+        <v>-0.526263666898005</v>
+      </c>
       <c r="AQ5" t="inlineStr"/>
       <c r="AR5" t="n">
-        <v>1.668374655647387</v>
-      </c>
-      <c r="AS5" t="n">
-        <v>1.007456382001806</v>
-      </c>
-      <c r="AT5" t="inlineStr"/>
-      <c r="AU5" t="inlineStr"/>
-      <c r="AV5" t="inlineStr"/>
+        <v>1.718787878787882</v>
+      </c>
+      <c r="AS5" t="inlineStr"/>
+      <c r="AT5" t="n">
+        <v>2.35667932433126</v>
+      </c>
+      <c r="AU5" t="n">
+        <v>-6.89434343434344</v>
+      </c>
+      <c r="AV5" t="n">
+        <v>-5.745858585858585</v>
+      </c>
       <c r="AW5" t="n">
-        <v>-34725580.90765035</v>
+        <v>-7.090902265189186</v>
       </c>
       <c r="AX5" t="n">
-        <v>-6.887860422405865</v>
+        <v>-52132212.12121212</v>
       </c>
       <c r="AY5" t="n">
-        <v>-5.735684113865929</v>
+        <v>-0.9574747474747469</v>
       </c>
       <c r="AZ5" t="n">
-        <v>-0.5270262005616082</v>
-      </c>
-      <c r="BA5" t="n">
-        <v>-7.119658062273857</v>
-      </c>
+        <v>-34450128.72443547</v>
+      </c>
+      <c r="BA5" t="inlineStr"/>
       <c r="BB5" t="n">
-        <v>-52072438.01652893</v>
-      </c>
-      <c r="BC5" t="inlineStr"/>
-      <c r="BD5" t="n">
-        <v>1.815677715707238</v>
-      </c>
-      <c r="BE5" t="n">
-        <v>-5.949425257885082</v>
-      </c>
+        <v>1.016868686868662</v>
+      </c>
+      <c r="BC5" t="n">
+        <v>1.735629535278036</v>
+      </c>
+      <c r="BD5" t="inlineStr"/>
+      <c r="BE5" t="inlineStr"/>
       <c r="BF5" t="inlineStr"/>
       <c r="BG5" t="n">
         <v>0</v>
@@ -1532,49 +1532,49 @@
       <c r="U6" t="n">
         <v>4.583333333333336</v>
       </c>
-      <c r="V6" t="n">
+      <c r="V6" t="inlineStr"/>
+      <c r="W6" t="inlineStr"/>
+      <c r="X6" t="n">
+        <v>-5.75</v>
+      </c>
+      <c r="Y6" t="n">
+        <v>-4.083333333333334</v>
+      </c>
+      <c r="Z6" t="n">
         <v>-0.4166666666666667</v>
       </c>
-      <c r="W6" t="n">
+      <c r="AA6" t="n">
         <v>0.3333333333333333</v>
       </c>
-      <c r="X6" t="n">
+      <c r="AB6" t="n">
+        <v>0.583333333333333</v>
+      </c>
+      <c r="AC6" t="n">
+        <v>3.083333333333333</v>
+      </c>
+      <c r="AD6" t="n">
+        <v>0.5833333333333333</v>
+      </c>
+      <c r="AE6" t="n">
+        <v>1.166666666666667</v>
+      </c>
+      <c r="AF6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG6" t="n">
+        <v>1</v>
+      </c>
+      <c r="AH6" t="n">
         <v>0.3358333333333333</v>
       </c>
-      <c r="Y6" t="n">
+      <c r="AI6" t="n">
         <v>1.219166666666667</v>
       </c>
-      <c r="Z6" t="n">
+      <c r="AJ6" t="n">
         <v>-3.833333333333334</v>
       </c>
-      <c r="AA6" t="n">
+      <c r="AK6" t="n">
         <v>3.666666666666666</v>
-      </c>
-      <c r="AB6" t="n">
-        <v>0.5833333333333333</v>
-      </c>
-      <c r="AC6" t="n">
-        <v>1.166666666666667</v>
-      </c>
-      <c r="AD6" t="n">
-        <v>0</v>
-      </c>
-      <c r="AE6" t="n">
-        <v>1</v>
-      </c>
-      <c r="AF6" t="inlineStr"/>
-      <c r="AG6" t="inlineStr"/>
-      <c r="AH6" t="n">
-        <v>0.583333333333333</v>
-      </c>
-      <c r="AI6" t="n">
-        <v>3.083333333333333</v>
-      </c>
-      <c r="AJ6" t="n">
-        <v>-5.75</v>
-      </c>
-      <c r="AK6" t="n">
-        <v>-4.083333333333334</v>
       </c>
       <c r="AL6" t="n">
         <v>77.56969696969696</v>
@@ -1582,48 +1582,48 @@
       <c r="AM6" t="n">
         <v>74.68888888888888</v>
       </c>
-      <c r="AN6" t="n">
-        <v>0.0278985652925634</v>
-      </c>
+      <c r="AN6" t="inlineStr"/>
       <c r="AO6" t="n">
-        <v>0.04132231404958664</v>
-      </c>
-      <c r="AP6" t="inlineStr"/>
+        <v>3.092055875814026</v>
+      </c>
+      <c r="AP6" t="n">
+        <v>0.136595052694124</v>
+      </c>
       <c r="AQ6" t="inlineStr"/>
       <c r="AR6" t="n">
-        <v>0.4973247627793072</v>
-      </c>
-      <c r="AS6" t="n">
-        <v>4.826342209978577</v>
-      </c>
-      <c r="AT6" t="inlineStr"/>
-      <c r="AU6" t="inlineStr"/>
-      <c r="AV6" t="inlineStr"/>
+        <v>0.4513314967860396</v>
+      </c>
+      <c r="AS6" t="inlineStr"/>
+      <c r="AT6" t="n">
+        <v>0.06584250439653161</v>
+      </c>
+      <c r="AU6" t="n">
+        <v>2.907529843893485</v>
+      </c>
+      <c r="AV6" t="n">
+        <v>3.521435130526044</v>
+      </c>
       <c r="AW6" t="n">
-        <v>4754117.417338846</v>
+        <v>2.202306889054753</v>
       </c>
       <c r="AX6" t="n">
-        <v>2.860055096418733</v>
+        <v>6881653.54847173</v>
       </c>
       <c r="AY6" t="n">
-        <v>3.530468319559219</v>
+        <v>0.04132231404958664</v>
       </c>
       <c r="AZ6" t="n">
-        <v>0.136595052694124</v>
-      </c>
-      <c r="BA6" t="n">
-        <v>2.199693543321217</v>
-      </c>
+        <v>4777020.232439416</v>
+      </c>
+      <c r="BA6" t="inlineStr"/>
       <c r="BB6" t="n">
-        <v>6870490.970309153</v>
-      </c>
-      <c r="BC6" t="inlineStr"/>
-      <c r="BD6" t="n">
-        <v>0.6970477622664646</v>
-      </c>
-      <c r="BE6" t="n">
-        <v>3.011981753059956</v>
-      </c>
+        <v>4.73366784730419</v>
+      </c>
+      <c r="BC6" t="n">
+        <v>0.6812337721996755</v>
+      </c>
+      <c r="BD6" t="inlineStr"/>
+      <c r="BE6" t="inlineStr"/>
       <c r="BF6" t="inlineStr"/>
       <c r="BG6" t="n">
         <v>0</v>
@@ -1713,49 +1713,49 @@
       <c r="U7" t="n">
         <v>-1.5</v>
       </c>
-      <c r="V7" t="n">
+      <c r="V7" t="inlineStr"/>
+      <c r="W7" t="inlineStr"/>
+      <c r="X7" t="n">
+        <v>2.333333333333334</v>
+      </c>
+      <c r="Y7" t="n">
+        <v>-3.166666666666666</v>
+      </c>
+      <c r="Z7" t="n">
         <v>0.5</v>
       </c>
-      <c r="W7" t="n">
+      <c r="AA7" t="n">
         <v>-1</v>
       </c>
-      <c r="X7" t="n">
+      <c r="AB7" t="n">
+        <v>3.666666666666667</v>
+      </c>
+      <c r="AC7" t="n">
+        <v>-5.666666666666666</v>
+      </c>
+      <c r="AD7" t="n">
+        <v>1.166666666666667</v>
+      </c>
+      <c r="AE7" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AF7" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AG7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH7" t="n">
         <v>0.9266666666666666</v>
       </c>
-      <c r="Y7" t="n">
+      <c r="AI7" t="n">
         <v>-1.28</v>
       </c>
-      <c r="Z7" t="n">
+      <c r="AJ7" t="n">
         <v>12</v>
       </c>
-      <c r="AA7" t="n">
+      <c r="AK7" t="n">
         <v>-11.16666666666667</v>
-      </c>
-      <c r="AB7" t="n">
-        <v>1.166666666666667</v>
-      </c>
-      <c r="AC7" t="n">
-        <v>-1</v>
-      </c>
-      <c r="AD7" t="n">
-        <v>0</v>
-      </c>
-      <c r="AE7" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="AF7" t="inlineStr"/>
-      <c r="AG7" t="inlineStr"/>
-      <c r="AH7" t="n">
-        <v>3.666666666666667</v>
-      </c>
-      <c r="AI7" t="n">
-        <v>-5.666666666666666</v>
-      </c>
-      <c r="AJ7" t="n">
-        <v>2.333333333333334</v>
-      </c>
-      <c r="AK7" t="n">
-        <v>-3.166666666666666</v>
       </c>
       <c r="AL7" t="n">
         <v>76.55555555555554</v>
@@ -1763,48 +1763,48 @@
       <c r="AM7" t="n">
         <v>84.70151515151515</v>
       </c>
-      <c r="AN7" t="n">
-        <v>0.1886910046823935</v>
-      </c>
+      <c r="AN7" t="inlineStr"/>
       <c r="AO7" t="n">
-        <v>-0.1436868686868689</v>
-      </c>
-      <c r="AP7" t="inlineStr"/>
+        <v>2.551432944454518</v>
+      </c>
+      <c r="AP7" t="n">
+        <v>0.03531281094240724</v>
+      </c>
       <c r="AQ7" t="inlineStr"/>
       <c r="AR7" t="n">
-        <v>-1.373484848484846</v>
-      </c>
-      <c r="AS7" t="n">
-        <v>2.202525252525248</v>
-      </c>
-      <c r="AT7" t="inlineStr"/>
-      <c r="AU7" t="inlineStr"/>
-      <c r="AV7" t="inlineStr"/>
+        <v>-1.40166666666666</v>
+      </c>
+      <c r="AS7" t="inlineStr"/>
+      <c r="AT7" t="n">
+        <v>0.1217762720194848</v>
+      </c>
+      <c r="AU7" t="n">
+        <v>-0.6594444444444463</v>
+      </c>
+      <c r="AV7" t="n">
+        <v>-1.708611111111111</v>
+      </c>
       <c r="AW7" t="n">
-        <v>2240428.597877445</v>
+        <v>0.7687841189391094</v>
       </c>
       <c r="AX7" t="n">
-        <v>-0.6785353535353522</v>
+        <v>-3442173.611111112</v>
       </c>
       <c r="AY7" t="n">
-        <v>-1.666792929292924</v>
+        <v>-0.1627777777777779</v>
       </c>
       <c r="AZ7" t="n">
-        <v>0.05694861168006926</v>
-      </c>
-      <c r="BA7" t="n">
-        <v>0.8169144816237264</v>
-      </c>
+        <v>1888823.633241331</v>
+      </c>
+      <c r="BA7" t="inlineStr"/>
       <c r="BB7" t="n">
-        <v>-3325173.611111112</v>
-      </c>
-      <c r="BC7" t="inlineStr"/>
-      <c r="BD7" t="n">
-        <v>4.355336533291137</v>
-      </c>
-      <c r="BE7" t="n">
-        <v>2.840177295521215</v>
-      </c>
+        <v>2.098888888888894</v>
+      </c>
+      <c r="BC7" t="n">
+        <v>4.631822247063582</v>
+      </c>
+      <c r="BD7" t="inlineStr"/>
+      <c r="BE7" t="inlineStr"/>
       <c r="BF7" t="inlineStr"/>
       <c r="BG7" t="n">
         <v>0</v>
@@ -1894,45 +1894,45 @@
       <c r="U8" t="n">
         <v>0.5</v>
       </c>
-      <c r="V8" t="n">
+      <c r="V8" t="inlineStr"/>
+      <c r="W8" t="inlineStr"/>
+      <c r="X8" t="n">
+        <v>-3</v>
+      </c>
+      <c r="Y8" t="n">
+        <v>5</v>
+      </c>
+      <c r="Z8" t="n">
         <v>0.1666666666666667</v>
       </c>
-      <c r="W8" t="n">
+      <c r="AA8" t="n">
         <v>0.1666666666666667</v>
       </c>
-      <c r="X8" t="n">
-        <v>0.08500000000000008</v>
-      </c>
-      <c r="Y8" t="n">
-        <v>-0.246666666666667</v>
-      </c>
-      <c r="Z8" t="n">
-        <v>1.833333333333334</v>
-      </c>
-      <c r="AA8" t="n">
-        <v>-0.5</v>
-      </c>
       <c r="AB8" t="n">
+        <v>-0.833333333333333</v>
+      </c>
+      <c r="AC8" t="n">
+        <v>-1.166666666666667</v>
+      </c>
+      <c r="AD8" t="n">
         <v>-0.3333333333333333</v>
       </c>
-      <c r="AC8" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD8" t="inlineStr"/>
-      <c r="AE8" t="inlineStr"/>
+      <c r="AE8" t="n">
+        <v>0</v>
+      </c>
       <c r="AF8" t="inlineStr"/>
       <c r="AG8" t="inlineStr"/>
       <c r="AH8" t="n">
-        <v>-0.833333333333333</v>
+        <v>0.08500000000000008</v>
       </c>
       <c r="AI8" t="n">
-        <v>-1.166666666666667</v>
+        <v>-0.246666666666667</v>
       </c>
       <c r="AJ8" t="n">
-        <v>-3</v>
+        <v>1.833333333333334</v>
       </c>
       <c r="AK8" t="n">
-        <v>5</v>
+        <v>-0.5</v>
       </c>
       <c r="AL8" t="n">
         <v>84</v>
@@ -1940,48 +1940,48 @@
       <c r="AM8" t="n">
         <v>77.03030303030302</v>
       </c>
-      <c r="AN8" t="n">
-        <v>-2.819158373015039</v>
-      </c>
+      <c r="AN8" t="inlineStr"/>
       <c r="AO8" t="n">
-        <v>-0.5024793388429749</v>
-      </c>
-      <c r="AP8" t="inlineStr"/>
+        <v>-5.533637670702873</v>
+      </c>
+      <c r="AP8" t="n">
+        <v>-0.2942430178043989</v>
+      </c>
       <c r="AQ8" t="inlineStr"/>
       <c r="AR8" t="n">
-        <v>-0.634297520661157</v>
-      </c>
-      <c r="AS8" t="n">
-        <v>-1.631818181818176</v>
-      </c>
-      <c r="AT8" t="inlineStr"/>
-      <c r="AU8" t="inlineStr"/>
-      <c r="AV8" t="inlineStr"/>
+        <v>-0.6651515151515142</v>
+      </c>
+      <c r="AS8" t="inlineStr"/>
+      <c r="AT8" t="n">
+        <v>-2.615349285080747</v>
+      </c>
+      <c r="AU8" t="n">
+        <v>-4.11727272727272</v>
+      </c>
+      <c r="AV8" t="n">
+        <v>-5.865656565656579</v>
+      </c>
       <c r="AW8" t="n">
-        <v>-4502556.331911132</v>
+        <v>-2.930371366816374</v>
       </c>
       <c r="AX8" t="n">
-        <v>-4.17462809917356</v>
+        <v>-9659737.373737372</v>
       </c>
       <c r="AY8" t="n">
-        <v>-5.849338842975214</v>
+        <v>-0.4981818181818181</v>
       </c>
       <c r="AZ8" t="n">
-        <v>-0.2978447829005839</v>
-      </c>
-      <c r="BA8" t="n">
-        <v>-2.837689123439546</v>
-      </c>
+        <v>-4571138.972233602</v>
+      </c>
+      <c r="BA8" t="inlineStr"/>
       <c r="BB8" t="n">
-        <v>-9694661.157024793</v>
-      </c>
-      <c r="BC8" t="inlineStr"/>
-      <c r="BD8" t="n">
-        <v>1.532534641596499</v>
-      </c>
-      <c r="BE8" t="n">
-        <v>-5.686038533271713</v>
-      </c>
+        <v>-1.536868686868672</v>
+      </c>
+      <c r="BC8" t="n">
+        <v>1.553277178679991</v>
+      </c>
+      <c r="BD8" t="inlineStr"/>
+      <c r="BE8" t="inlineStr"/>
       <c r="BF8" t="inlineStr"/>
       <c r="BG8" t="n">
         <v>0</v>
@@ -2071,45 +2071,45 @@
       <c r="U9" t="n">
         <v>-3</v>
       </c>
-      <c r="V9" t="n">
+      <c r="V9" t="inlineStr"/>
+      <c r="W9" t="inlineStr"/>
+      <c r="X9" t="n">
+        <v>-1.666666666666666</v>
+      </c>
+      <c r="Y9" t="n">
+        <v>-4.166666666666666</v>
+      </c>
+      <c r="Z9" t="n">
         <v>-0.5</v>
       </c>
-      <c r="W9" t="n">
-        <v>0</v>
-      </c>
-      <c r="X9" t="n">
-        <v>0.07166666666666655</v>
-      </c>
-      <c r="Y9" t="n">
-        <v>-0.6383333333333332</v>
-      </c>
-      <c r="Z9" t="n">
-        <v>2.166666666666666</v>
-      </c>
       <c r="AA9" t="n">
-        <v>-2.666666666666666</v>
+        <v>0</v>
       </c>
       <c r="AB9" t="n">
+        <v>3</v>
+      </c>
+      <c r="AC9" t="n">
+        <v>-2.666666666666667</v>
+      </c>
+      <c r="AD9" t="n">
         <v>-0.1666666666666666</v>
       </c>
-      <c r="AC9" t="n">
+      <c r="AE9" t="n">
         <v>-0.8333333333333335</v>
       </c>
-      <c r="AD9" t="inlineStr"/>
-      <c r="AE9" t="inlineStr"/>
       <c r="AF9" t="inlineStr"/>
       <c r="AG9" t="inlineStr"/>
       <c r="AH9" t="n">
-        <v>3</v>
+        <v>0.07166666666666655</v>
       </c>
       <c r="AI9" t="n">
-        <v>-2.666666666666667</v>
+        <v>-0.6383333333333332</v>
       </c>
       <c r="AJ9" t="n">
-        <v>-1.666666666666666</v>
+        <v>2.166666666666666</v>
       </c>
       <c r="AK9" t="n">
-        <v>-4.166666666666666</v>
+        <v>-2.666666666666666</v>
       </c>
       <c r="AL9" t="n">
         <v>75.66666666666666</v>
@@ -2117,48 +2117,48 @@
       <c r="AM9" t="n">
         <v>77.4074074074074</v>
       </c>
-      <c r="AN9" t="n">
-        <v>2.506421558606483</v>
-      </c>
+      <c r="AN9" t="inlineStr"/>
       <c r="AO9" t="n">
-        <v>-0.7395775941230489</v>
-      </c>
-      <c r="AP9" t="inlineStr"/>
+        <v>-0.4998184130111412</v>
+      </c>
+      <c r="AP9" t="n">
+        <v>-0.2347719287076873</v>
+      </c>
       <c r="AQ9" t="inlineStr"/>
       <c r="AR9" t="n">
-        <v>0.2573002754820948</v>
-      </c>
-      <c r="AS9" t="n">
-        <v>-0.04141414141420796</v>
-      </c>
-      <c r="AT9" t="inlineStr"/>
-      <c r="AU9" t="inlineStr"/>
-      <c r="AV9" t="inlineStr"/>
+        <v>0.2030303030302996</v>
+      </c>
+      <c r="AS9" t="inlineStr"/>
+      <c r="AT9" t="n">
+        <v>2.393088559187628</v>
+      </c>
+      <c r="AU9" t="n">
+        <v>-3.358989898989904</v>
+      </c>
+      <c r="AV9" t="n">
+        <v>-3.829494949494944</v>
+      </c>
       <c r="AW9" t="n">
-        <v>-7851854.423149318</v>
+        <v>-3.030618206612814</v>
       </c>
       <c r="AX9" t="n">
-        <v>-3.508172635445362</v>
+        <v>-15873040.4040404</v>
       </c>
       <c r="AY9" t="n">
-        <v>-3.926813590449953</v>
+        <v>-0.7135353535353537</v>
       </c>
       <c r="AZ9" t="n">
-        <v>-0.1998773603723192</v>
-      </c>
-      <c r="BA9" t="n">
-        <v>-3.064254834921854</v>
-      </c>
+        <v>-8154796.076644374</v>
+      </c>
+      <c r="BA9" t="inlineStr"/>
       <c r="BB9" t="n">
-        <v>-16440945.82185491</v>
-      </c>
-      <c r="BC9" t="inlineStr"/>
-      <c r="BD9" t="n">
-        <v>-2.391073777759544</v>
-      </c>
-      <c r="BE9" t="n">
-        <v>-0.409208156379421</v>
-      </c>
+        <v>-0.1355555555555839</v>
+      </c>
+      <c r="BC9" t="n">
+        <v>-2.341361279759127</v>
+      </c>
+      <c r="BD9" t="inlineStr"/>
+      <c r="BE9" t="inlineStr"/>
       <c r="BF9" t="inlineStr"/>
       <c r="BG9" t="n">
         <v>0</v>
@@ -2248,49 +2248,49 @@
       <c r="U10" t="n">
         <v>-4.666666666666664</v>
       </c>
-      <c r="V10" t="n">
+      <c r="V10" t="inlineStr"/>
+      <c r="W10" t="inlineStr"/>
+      <c r="X10" t="n">
+        <v>-3</v>
+      </c>
+      <c r="Y10" t="n">
+        <v>-3.5</v>
+      </c>
+      <c r="Z10" t="n">
         <v>1.166666666666667</v>
       </c>
-      <c r="W10" t="n">
+      <c r="AA10" t="n">
         <v>-0.8333333333333335</v>
       </c>
-      <c r="X10" t="n">
+      <c r="AB10" t="n">
+        <v>-0.5</v>
+      </c>
+      <c r="AC10" t="n">
+        <v>-4.666666666666667</v>
+      </c>
+      <c r="AD10" t="n">
+        <v>-0.1666666666666666</v>
+      </c>
+      <c r="AE10" t="n">
+        <v>-0.5</v>
+      </c>
+      <c r="AF10" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AG10" t="n">
+        <v>-3</v>
+      </c>
+      <c r="AH10" t="n">
         <v>-0.2033333333333336</v>
       </c>
-      <c r="Y10" t="n">
+      <c r="AI10" t="n">
         <v>-0.916666666666667</v>
       </c>
-      <c r="Z10" t="n">
+      <c r="AJ10" t="n">
         <v>-2.666666666666666</v>
       </c>
-      <c r="AA10" t="n">
+      <c r="AK10" t="n">
         <v>-6.5</v>
-      </c>
-      <c r="AB10" t="n">
-        <v>-0.1666666666666666</v>
-      </c>
-      <c r="AC10" t="n">
-        <v>-0.5</v>
-      </c>
-      <c r="AD10" t="n">
-        <v>-1</v>
-      </c>
-      <c r="AE10" t="n">
-        <v>-1.5</v>
-      </c>
-      <c r="AF10" t="inlineStr"/>
-      <c r="AG10" t="inlineStr"/>
-      <c r="AH10" t="n">
-        <v>-0.5</v>
-      </c>
-      <c r="AI10" t="n">
-        <v>-4.666666666666667</v>
-      </c>
-      <c r="AJ10" t="n">
-        <v>-3</v>
-      </c>
-      <c r="AK10" t="n">
-        <v>-3.5</v>
       </c>
       <c r="AL10" t="n">
         <v>73.04861111111111</v>
@@ -2298,48 +2298,48 @@
       <c r="AM10" t="n">
         <v>79.27129629629628</v>
       </c>
-      <c r="AN10" t="n">
-        <v>1.647532406975973</v>
-      </c>
+      <c r="AN10" t="inlineStr"/>
       <c r="AO10" t="n">
-        <v>0.4184343434343432</v>
-      </c>
-      <c r="AP10" t="inlineStr"/>
+        <v>-1.174410692051623</v>
+      </c>
+      <c r="AP10" t="n">
+        <v>0.08546477412041131</v>
+      </c>
       <c r="AQ10" t="inlineStr"/>
       <c r="AR10" t="n">
-        <v>3.041666666666668</v>
-      </c>
-      <c r="AS10" t="n">
-        <v>2.481144781144764</v>
-      </c>
-      <c r="AT10" t="inlineStr"/>
-      <c r="AU10" t="inlineStr"/>
-      <c r="AV10" t="inlineStr"/>
+        <v>3.155371900826445</v>
+      </c>
+      <c r="AS10" t="inlineStr"/>
+      <c r="AT10" t="n">
+        <v>1.44680302983237</v>
+      </c>
+      <c r="AU10" t="n">
+        <v>-0.1507805325987164</v>
+      </c>
+      <c r="AV10" t="n">
+        <v>1.570064279155204</v>
+      </c>
       <c r="AW10" t="n">
-        <v>-3467877.904676599</v>
+        <v>-2.46606958528757</v>
       </c>
       <c r="AX10" t="n">
-        <v>-0.1003367003366975</v>
+        <v>2349334.251606982</v>
       </c>
       <c r="AY10" t="n">
-        <v>1.558164983165</v>
+        <v>0.4341597796143246</v>
       </c>
       <c r="AZ10" t="n">
-        <v>0.1033427096103772</v>
-      </c>
-      <c r="BA10" t="n">
-        <v>-2.523989712439544</v>
-      </c>
+        <v>-3351902.158637099</v>
+      </c>
+      <c r="BA10" t="inlineStr"/>
       <c r="BB10" t="n">
-        <v>2393632.154882155</v>
-      </c>
-      <c r="BC10" t="inlineStr"/>
-      <c r="BD10" t="n">
-        <v>3.311080574080734</v>
-      </c>
-      <c r="BE10" t="n">
-        <v>-1.15154313438066</v>
-      </c>
+        <v>2.376124885215802</v>
+      </c>
+      <c r="BC10" t="n">
+        <v>3.612592949502215</v>
+      </c>
+      <c r="BD10" t="inlineStr"/>
+      <c r="BE10" t="inlineStr"/>
       <c r="BF10" t="inlineStr"/>
       <c r="BG10" t="n">
         <v>0</v>
@@ -2429,49 +2429,49 @@
       <c r="U11" t="n">
         <v>-5.833333333333336</v>
       </c>
-      <c r="V11" t="n">
+      <c r="V11" t="inlineStr"/>
+      <c r="W11" t="inlineStr"/>
+      <c r="X11" t="n">
+        <v>1.666666666666666</v>
+      </c>
+      <c r="Y11" t="n">
+        <v>3.833333333333334</v>
+      </c>
+      <c r="Z11" t="n">
         <v>1</v>
       </c>
-      <c r="W11" t="n">
+      <c r="AA11" t="n">
         <v>-0.5</v>
       </c>
-      <c r="X11" t="n">
+      <c r="AB11" t="n">
+        <v>2.166666666666667</v>
+      </c>
+      <c r="AC11" t="n">
+        <v>-1.666666666666667</v>
+      </c>
+      <c r="AD11" t="n">
+        <v>0.3333333333333335</v>
+      </c>
+      <c r="AE11" t="n">
+        <v>-0.1666666666666667</v>
+      </c>
+      <c r="AF11" t="n">
+        <v>1</v>
+      </c>
+      <c r="AG11" t="n">
+        <v>1</v>
+      </c>
+      <c r="AH11" t="n">
         <v>1.243333333333334</v>
       </c>
-      <c r="Y11" t="n">
+      <c r="AI11" t="n">
         <v>-0.8416666666666666</v>
       </c>
-      <c r="Z11" t="n">
+      <c r="AJ11" t="n">
         <v>10.16666666666667</v>
       </c>
-      <c r="AA11" t="n">
+      <c r="AK11" t="n">
         <v>-6.5</v>
-      </c>
-      <c r="AB11" t="n">
-        <v>0.3333333333333335</v>
-      </c>
-      <c r="AC11" t="n">
-        <v>-0.1666666666666667</v>
-      </c>
-      <c r="AD11" t="n">
-        <v>0</v>
-      </c>
-      <c r="AE11" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="AF11" t="inlineStr"/>
-      <c r="AG11" t="inlineStr"/>
-      <c r="AH11" t="n">
-        <v>2.166666666666667</v>
-      </c>
-      <c r="AI11" t="n">
-        <v>-1.666666666666667</v>
-      </c>
-      <c r="AJ11" t="n">
-        <v>1.666666666666666</v>
-      </c>
-      <c r="AK11" t="n">
-        <v>3.833333333333334</v>
       </c>
       <c r="AL11" t="n">
         <v>75.51363636363637</v>
@@ -2479,48 +2479,48 @@
       <c r="AM11" t="n">
         <v>76.44090909090909</v>
       </c>
-      <c r="AN11" t="n">
-        <v>1.330697831365406</v>
-      </c>
+      <c r="AN11" t="inlineStr"/>
       <c r="AO11" t="n">
-        <v>0.8335418579736757</v>
-      </c>
-      <c r="AP11" t="inlineStr"/>
+        <v>7.977066650025264</v>
+      </c>
+      <c r="AP11" t="n">
+        <v>0.4396177609799903</v>
+      </c>
       <c r="AQ11" t="inlineStr"/>
       <c r="AR11" t="n">
         <v>-1.848433195592285</v>
       </c>
-      <c r="AS11" t="n">
+      <c r="AS11" t="inlineStr"/>
+      <c r="AT11" t="n">
+        <v>1.330697831365406</v>
+      </c>
+      <c r="AU11" t="n">
+        <v>6.635158402203857</v>
+      </c>
+      <c r="AV11" t="n">
+        <v>8.002978650137749</v>
+      </c>
+      <c r="AW11" t="n">
+        <v>4.079671563601522</v>
+      </c>
+      <c r="AX11" t="n">
+        <v>50299240.70247935</v>
+      </c>
+      <c r="AY11" t="n">
+        <v>0.8335418579736757</v>
+      </c>
+      <c r="AZ11" t="n">
+        <v>28644315.15090087</v>
+      </c>
+      <c r="BA11" t="inlineStr"/>
+      <c r="BB11" t="n">
         <v>0.8175026782981263</v>
       </c>
-      <c r="AT11" t="inlineStr"/>
-      <c r="AU11" t="inlineStr"/>
-      <c r="AV11" t="inlineStr"/>
-      <c r="AW11" t="n">
-        <v>28644315.15090087</v>
-      </c>
-      <c r="AX11" t="n">
-        <v>6.635158402203857</v>
-      </c>
-      <c r="AY11" t="n">
-        <v>8.002978650137749</v>
-      </c>
-      <c r="AZ11" t="n">
-        <v>0.4396177609799903</v>
-      </c>
-      <c r="BA11" t="n">
-        <v>4.079671563601522</v>
-      </c>
-      <c r="BB11" t="n">
-        <v>50299240.70247935</v>
-      </c>
-      <c r="BC11" t="inlineStr"/>
-      <c r="BD11" t="n">
+      <c r="BC11" t="n">
         <v>1.327260581266046</v>
       </c>
-      <c r="BE11" t="n">
-        <v>7.977066650025264</v>
-      </c>
+      <c r="BD11" t="inlineStr"/>
+      <c r="BE11" t="inlineStr"/>
       <c r="BF11" t="inlineStr"/>
       <c r="BG11" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Data. Terminó de entrenar modelos de SPA y actualicé predicciones.
</commit_message>
<xml_diff>
--- a/data/england/p6_deployment/data_preparation/df_constructed.xlsx
+++ b/data/england/p6_deployment/data_preparation/df_constructed.xlsx
@@ -695,112 +695,112 @@
       </c>
       <c r="BB1" s="1" t="inlineStr">
         <is>
+          <t>dif_sum_value_player_miss</t>
+        </is>
+      </c>
+      <c r="BC1" s="1" t="inlineStr">
+        <is>
+          <t>dif_mean_value_player_sub</t>
+        </is>
+      </c>
+      <c r="BD1" s="1" t="inlineStr">
+        <is>
+          <t>dif_mean_rat_player_sub</t>
+        </is>
+      </c>
+      <c r="BE1" s="1" t="inlineStr">
+        <is>
+          <t>dif_sum_rep_player_miss</t>
+        </is>
+      </c>
+      <c r="BF1" s="1" t="inlineStr">
+        <is>
+          <t>dif_mean_pot_player_sub</t>
+        </is>
+      </c>
+      <c r="BG1" s="1" t="inlineStr">
+        <is>
           <t>dif_mean_age_player_start</t>
         </is>
       </c>
-      <c r="BC1" s="1" t="inlineStr">
+      <c r="BH1" s="1" t="inlineStr">
+        <is>
+          <t>dif_mean_age_player_miss</t>
+        </is>
+      </c>
+      <c r="BI1" s="1" t="inlineStr">
+        <is>
+          <t>dif_mean_hei_player_miss</t>
+        </is>
+      </c>
+      <c r="BJ1" s="1" t="inlineStr">
+        <is>
+          <t>dif_sum_pot_player_miss</t>
+        </is>
+      </c>
+      <c r="BK1" s="1" t="inlineStr">
+        <is>
+          <t>dif_mean_wage_player_sub</t>
+        </is>
+      </c>
+      <c r="BL1" s="1" t="inlineStr">
+        <is>
+          <t>dif_mean_rep_player_start</t>
+        </is>
+      </c>
+      <c r="BM1" s="1" t="inlineStr">
+        <is>
+          <t>dif_mean_rat_player_start</t>
+        </is>
+      </c>
+      <c r="BN1" s="1" t="inlineStr">
+        <is>
+          <t>dif_sum_wage_player_miss</t>
+        </is>
+      </c>
+      <c r="BO1" s="1" t="inlineStr">
+        <is>
+          <t>dif_mean_value_player_start</t>
+        </is>
+      </c>
+      <c r="BP1" s="1" t="inlineStr">
         <is>
           <t>dif_mean_age_player_sub</t>
         </is>
       </c>
-      <c r="BD1" s="1" t="inlineStr">
+      <c r="BQ1" s="1" t="inlineStr">
+        <is>
+          <t>dif_mean_wage_player_start</t>
+        </is>
+      </c>
+      <c r="BR1" s="1" t="inlineStr">
+        <is>
+          <t>dif_sum_rat_player_miss</t>
+        </is>
+      </c>
+      <c r="BS1" s="1" t="inlineStr">
+        <is>
+          <t>dif_mean_rep_player_sub</t>
+        </is>
+      </c>
+      <c r="BT1" s="1" t="inlineStr">
+        <is>
+          <t>dif_mean_hei_player_start</t>
+        </is>
+      </c>
+      <c r="BU1" s="1" t="inlineStr">
         <is>
           <t>dif_mean_hei_player_sub</t>
         </is>
       </c>
-      <c r="BE1" s="1" t="inlineStr">
-        <is>
-          <t>dif_sum_value_player_miss</t>
-        </is>
-      </c>
-      <c r="BF1" s="1" t="inlineStr">
-        <is>
-          <t>dif_mean_rep_player_start</t>
-        </is>
-      </c>
-      <c r="BG1" s="1" t="inlineStr">
-        <is>
-          <t>dif_mean_age_player_miss</t>
-        </is>
-      </c>
-      <c r="BH1" s="1" t="inlineStr">
-        <is>
-          <t>dif_sum_rat_player_miss</t>
-        </is>
-      </c>
-      <c r="BI1" s="1" t="inlineStr">
-        <is>
-          <t>dif_mean_rat_player_start</t>
-        </is>
-      </c>
-      <c r="BJ1" s="1" t="inlineStr">
-        <is>
-          <t>dif_mean_value_player_sub</t>
-        </is>
-      </c>
-      <c r="BK1" s="1" t="inlineStr">
-        <is>
-          <t>dif_sum_wage_player_miss</t>
-        </is>
-      </c>
-      <c r="BL1" s="1" t="inlineStr">
-        <is>
-          <t>dif_mean_pot_player_sub</t>
-        </is>
-      </c>
-      <c r="BM1" s="1" t="inlineStr">
-        <is>
-          <t>dif_mean_hei_player_miss</t>
-        </is>
-      </c>
-      <c r="BN1" s="1" t="inlineStr">
-        <is>
-          <t>dif_mean_rat_player_sub</t>
-        </is>
-      </c>
-      <c r="BO1" s="1" t="inlineStr">
+      <c r="BV1" s="1" t="inlineStr">
         <is>
           <t>dif_n_player_miss</t>
         </is>
       </c>
-      <c r="BP1" s="1" t="inlineStr">
-        <is>
-          <t>dif_sum_rep_player_miss</t>
-        </is>
-      </c>
-      <c r="BQ1" s="1" t="inlineStr">
-        <is>
-          <t>dif_mean_hei_player_start</t>
-        </is>
-      </c>
-      <c r="BR1" s="1" t="inlineStr">
-        <is>
-          <t>dif_sum_pot_player_miss</t>
-        </is>
-      </c>
-      <c r="BS1" s="1" t="inlineStr">
-        <is>
-          <t>dif_mean_wage_player_start</t>
-        </is>
-      </c>
-      <c r="BT1" s="1" t="inlineStr">
+      <c r="BW1" s="1" t="inlineStr">
         <is>
           <t>dif_mean_pot_player_start</t>
-        </is>
-      </c>
-      <c r="BU1" s="1" t="inlineStr">
-        <is>
-          <t>dif_mean_rep_player_sub</t>
-        </is>
-      </c>
-      <c r="BV1" s="1" t="inlineStr">
-        <is>
-          <t>dif_mean_wage_player_sub</t>
-        </is>
-      </c>
-      <c r="BW1" s="1" t="inlineStr">
-        <is>
-          <t>dif_mean_value_player_start</t>
         </is>
       </c>
     </row>
@@ -982,55 +982,55 @@
       <c r="BA2" t="n">
         <v>-0.08571428571428574</v>
       </c>
-      <c r="BB2" t="n">
-        <v>-1.301041666666666</v>
-      </c>
+      <c r="BB2" t="inlineStr"/>
       <c r="BC2" t="n">
-        <v>-0.5980249143971967</v>
+        <v>-3631347.746456444</v>
       </c>
       <c r="BD2" t="n">
-        <v>-4.474926839464899</v>
+        <v>-2.134526297977388</v>
       </c>
       <c r="BE2" t="inlineStr"/>
       <c r="BF2" t="n">
+        <v>-0.2859335184742804</v>
+      </c>
+      <c r="BG2" t="n">
+        <v>-1.301041666666666</v>
+      </c>
+      <c r="BH2" t="inlineStr"/>
+      <c r="BI2" t="inlineStr"/>
+      <c r="BJ2" t="inlineStr"/>
+      <c r="BK2" t="n">
+        <v>11982.3675645007</v>
+      </c>
+      <c r="BL2" t="n">
         <v>0.07171717171717074</v>
       </c>
-      <c r="BG2" t="inlineStr"/>
-      <c r="BH2" t="inlineStr"/>
-      <c r="BI2" t="n">
+      <c r="BM2" t="n">
         <v>-0.8254419191919169</v>
       </c>
-      <c r="BJ2" t="n">
-        <v>-3631347.746456444</v>
-      </c>
-      <c r="BK2" t="inlineStr"/>
-      <c r="BL2" t="n">
-        <v>-0.2859335184742804</v>
-      </c>
-      <c r="BM2" t="inlineStr"/>
-      <c r="BN2" t="n">
-        <v>-2.134526297977388</v>
-      </c>
-      <c r="BO2" t="inlineStr"/>
-      <c r="BP2" t="inlineStr"/>
+      <c r="BN2" t="inlineStr"/>
+      <c r="BO2" t="n">
+        <v>3175852.272727281</v>
+      </c>
+      <c r="BP2" t="n">
+        <v>-0.5980249143971967</v>
+      </c>
       <c r="BQ2" t="n">
-        <v>-1.835290404040393</v>
+        <v>15648.16919191915</v>
       </c>
       <c r="BR2" t="inlineStr"/>
       <c r="BS2" t="n">
-        <v>15648.16919191915</v>
+        <v>0.1588429686255779</v>
       </c>
       <c r="BT2" t="n">
+        <v>-1.835290404040393</v>
+      </c>
+      <c r="BU2" t="n">
+        <v>-4.474926839464899</v>
+      </c>
+      <c r="BV2" t="inlineStr"/>
+      <c r="BW2" t="n">
         <v>-0.3953282828282738</v>
-      </c>
-      <c r="BU2" t="n">
-        <v>0.1588429686255779</v>
-      </c>
-      <c r="BV2" t="n">
-        <v>11982.3675645007</v>
-      </c>
-      <c r="BW2" t="n">
-        <v>3175852.272727281</v>
       </c>
     </row>
     <row r="3">
@@ -1209,55 +1209,55 @@
       <c r="BA3" t="n">
         <v>0.1803921568627451</v>
       </c>
-      <c r="BB3" t="n">
-        <v>-4.335353535353534</v>
-      </c>
+      <c r="BB3" t="inlineStr"/>
       <c r="BC3" t="n">
-        <v>-3.080528610249974</v>
+        <v>8480040.86188006</v>
       </c>
       <c r="BD3" t="n">
-        <v>-1.925434962354444</v>
+        <v>1.372677504527346</v>
       </c>
       <c r="BE3" t="inlineStr"/>
       <c r="BF3" t="n">
+        <v>3.42808109145183</v>
+      </c>
+      <c r="BG3" t="n">
+        <v>-4.335353535353534</v>
+      </c>
+      <c r="BH3" t="inlineStr"/>
+      <c r="BI3" t="inlineStr"/>
+      <c r="BJ3" t="inlineStr"/>
+      <c r="BK3" t="n">
+        <v>11646.47532621607</v>
+      </c>
+      <c r="BL3" t="n">
         <v>-0.5250000000000001</v>
       </c>
-      <c r="BG3" t="inlineStr"/>
-      <c r="BH3" t="inlineStr"/>
-      <c r="BI3" t="n">
+      <c r="BM3" t="n">
         <v>0.01338383838383095</v>
       </c>
-      <c r="BJ3" t="n">
-        <v>8480040.86188006</v>
-      </c>
-      <c r="BK3" t="inlineStr"/>
-      <c r="BL3" t="n">
-        <v>3.42808109145183</v>
-      </c>
-      <c r="BM3" t="inlineStr"/>
-      <c r="BN3" t="n">
-        <v>1.372677504527346</v>
-      </c>
-      <c r="BO3" t="inlineStr"/>
-      <c r="BP3" t="inlineStr"/>
+      <c r="BN3" t="inlineStr"/>
+      <c r="BO3" t="n">
+        <v>6952266.414141417</v>
+      </c>
+      <c r="BP3" t="n">
+        <v>-3.080528610249974</v>
+      </c>
       <c r="BQ3" t="n">
-        <v>-3.036868686868672</v>
+        <v>-7696.590909090883</v>
       </c>
       <c r="BR3" t="inlineStr"/>
       <c r="BS3" t="n">
-        <v>-7696.590909090883</v>
+        <v>-0.1183566798698377</v>
       </c>
       <c r="BT3" t="n">
+        <v>-3.036868686868672</v>
+      </c>
+      <c r="BU3" t="n">
+        <v>-1.925434962354444</v>
+      </c>
+      <c r="BV3" t="inlineStr"/>
+      <c r="BW3" t="n">
         <v>2.852777777777774</v>
-      </c>
-      <c r="BU3" t="n">
-        <v>-0.1183566798698377</v>
-      </c>
-      <c r="BV3" t="n">
-        <v>11646.47532621607</v>
-      </c>
-      <c r="BW3" t="n">
-        <v>6952266.414141417</v>
       </c>
     </row>
     <row r="4">
@@ -1438,55 +1438,55 @@
       <c r="BA4" t="n">
         <v>-0.103448275862069</v>
       </c>
-      <c r="BB4" t="n">
-        <v>1.970061728395056</v>
-      </c>
+      <c r="BB4" t="inlineStr"/>
       <c r="BC4" t="n">
-        <v>1.996401525353733</v>
+        <v>-5287633.029529475</v>
       </c>
       <c r="BD4" t="n">
-        <v>-3.561333352785596</v>
+        <v>0.08684874947130083</v>
       </c>
       <c r="BE4" t="inlineStr"/>
       <c r="BF4" t="n">
+        <v>-1.821678457707876</v>
+      </c>
+      <c r="BG4" t="n">
+        <v>1.970061728395056</v>
+      </c>
+      <c r="BH4" t="inlineStr"/>
+      <c r="BI4" t="inlineStr"/>
+      <c r="BJ4" t="inlineStr"/>
+      <c r="BK4" t="n">
+        <v>-7316.916739986598</v>
+      </c>
+      <c r="BL4" t="n">
         <v>-0.2159611992945325</v>
       </c>
-      <c r="BG4" t="inlineStr"/>
-      <c r="BH4" t="inlineStr"/>
-      <c r="BI4" t="n">
+      <c r="BM4" t="n">
         <v>-0.8423280423280488</v>
       </c>
-      <c r="BJ4" t="n">
-        <v>-5287633.029529475</v>
-      </c>
-      <c r="BK4" t="inlineStr"/>
-      <c r="BL4" t="n">
-        <v>-1.821678457707876</v>
-      </c>
-      <c r="BM4" t="inlineStr"/>
-      <c r="BN4" t="n">
-        <v>0.08684874947130083</v>
-      </c>
-      <c r="BO4" t="inlineStr"/>
-      <c r="BP4" t="inlineStr"/>
+      <c r="BN4" t="inlineStr"/>
+      <c r="BO4" t="n">
+        <v>-10208349.86772487</v>
+      </c>
+      <c r="BP4" t="n">
+        <v>1.996401525353733</v>
+      </c>
       <c r="BQ4" t="n">
-        <v>-0.5857142857142605</v>
+        <v>-13915.21164021162</v>
       </c>
       <c r="BR4" t="inlineStr"/>
       <c r="BS4" t="n">
-        <v>-13915.21164021162</v>
+        <v>-0.0258574939947489</v>
       </c>
       <c r="BT4" t="n">
+        <v>-0.5857142857142605</v>
+      </c>
+      <c r="BU4" t="n">
+        <v>-3.561333352785596</v>
+      </c>
+      <c r="BV4" t="inlineStr"/>
+      <c r="BW4" t="n">
         <v>-2.779497354497352</v>
-      </c>
-      <c r="BU4" t="n">
-        <v>-0.0258574939947489</v>
-      </c>
-      <c r="BV4" t="n">
-        <v>-7316.916739986598</v>
-      </c>
-      <c r="BW4" t="n">
-        <v>-10208349.86772487</v>
       </c>
     </row>
     <row r="5">
@@ -1667,55 +1667,55 @@
       <c r="BA5" t="n">
         <v>-0.08000000000000002</v>
       </c>
-      <c r="BB5" t="n">
-        <v>0.2217372134038769</v>
-      </c>
+      <c r="BB5" t="inlineStr"/>
       <c r="BC5" t="n">
-        <v>3.172365388548311</v>
+        <v>-13924752.79709445</v>
       </c>
       <c r="BD5" t="n">
-        <v>-0.8861477560394064</v>
+        <v>-3.266978655207495</v>
       </c>
       <c r="BE5" t="inlineStr"/>
       <c r="BF5" t="n">
+        <v>-5.672645978367072</v>
+      </c>
+      <c r="BG5" t="n">
+        <v>0.2217372134038769</v>
+      </c>
+      <c r="BH5" t="inlineStr"/>
+      <c r="BI5" t="inlineStr"/>
+      <c r="BJ5" t="inlineStr"/>
+      <c r="BK5" t="n">
+        <v>-16436.24811911705</v>
+      </c>
+      <c r="BL5" t="n">
         <v>-1.291534391534391</v>
       </c>
-      <c r="BG5" t="inlineStr"/>
-      <c r="BH5" t="inlineStr"/>
-      <c r="BI5" t="n">
+      <c r="BM5" t="n">
         <v>-3.580291005291002</v>
       </c>
-      <c r="BJ5" t="n">
-        <v>-13924752.79709445</v>
-      </c>
-      <c r="BK5" t="inlineStr"/>
-      <c r="BL5" t="n">
-        <v>-5.672645978367072</v>
-      </c>
-      <c r="BM5" t="inlineStr"/>
-      <c r="BN5" t="n">
-        <v>-3.266978655207495</v>
-      </c>
-      <c r="BO5" t="inlineStr"/>
-      <c r="BP5" t="inlineStr"/>
+      <c r="BN5" t="inlineStr"/>
+      <c r="BO5" t="n">
+        <v>-20015661.37566138</v>
+      </c>
+      <c r="BP5" t="n">
+        <v>3.172365388548311</v>
+      </c>
       <c r="BQ5" t="n">
-        <v>-1.655291005290991</v>
+        <v>-39090.34391534394</v>
       </c>
       <c r="BR5" t="inlineStr"/>
       <c r="BS5" t="n">
-        <v>-39090.34391534394</v>
+        <v>-0.8222234557954373</v>
       </c>
       <c r="BT5" t="n">
+        <v>-1.655291005290991</v>
+      </c>
+      <c r="BU5" t="n">
+        <v>-0.8861477560394064</v>
+      </c>
+      <c r="BV5" t="inlineStr"/>
+      <c r="BW5" t="n">
         <v>-3.817283950617295</v>
-      </c>
-      <c r="BU5" t="n">
-        <v>-0.8222234557954373</v>
-      </c>
-      <c r="BV5" t="n">
-        <v>-16436.24811911705</v>
-      </c>
-      <c r="BW5" t="n">
-        <v>-20015661.37566138</v>
       </c>
     </row>
     <row r="6">
@@ -1896,55 +1896,55 @@
       <c r="BA6" t="n">
         <v>0.2426108374384237</v>
       </c>
-      <c r="BB6" t="n">
-        <v>0.8967171717171674</v>
-      </c>
+      <c r="BB6" t="inlineStr"/>
       <c r="BC6" t="n">
-        <v>0.2377233960034459</v>
+        <v>-886326.9966984792</v>
       </c>
       <c r="BD6" t="n">
-        <v>0.04241022310071685</v>
+        <v>-0.3998625900480022</v>
       </c>
       <c r="BE6" t="inlineStr"/>
       <c r="BF6" t="n">
+        <v>-0.3836045632400982</v>
+      </c>
+      <c r="BG6" t="n">
+        <v>0.8967171717171674</v>
+      </c>
+      <c r="BH6" t="inlineStr"/>
+      <c r="BI6" t="inlineStr"/>
+      <c r="BJ6" t="inlineStr"/>
+      <c r="BK6" t="n">
+        <v>-21133.82785633424</v>
+      </c>
+      <c r="BL6" t="n">
         <v>0.05972222222222223</v>
       </c>
-      <c r="BG6" t="inlineStr"/>
-      <c r="BH6" t="inlineStr"/>
-      <c r="BI6" t="n">
+      <c r="BM6" t="n">
         <v>-0.1147727272727366</v>
       </c>
-      <c r="BJ6" t="n">
-        <v>-886326.9966984792</v>
-      </c>
-      <c r="BK6" t="inlineStr"/>
-      <c r="BL6" t="n">
-        <v>-0.3836045632400982</v>
-      </c>
-      <c r="BM6" t="inlineStr"/>
-      <c r="BN6" t="n">
-        <v>-0.3998625900480022</v>
-      </c>
-      <c r="BO6" t="inlineStr"/>
-      <c r="BP6" t="inlineStr"/>
+      <c r="BN6" t="inlineStr"/>
+      <c r="BO6" t="n">
+        <v>67967.17171717249</v>
+      </c>
+      <c r="BP6" t="n">
+        <v>0.2377233960034459</v>
+      </c>
       <c r="BQ6" t="n">
-        <v>-1.497727272727246</v>
+        <v>-19943.18181818182</v>
       </c>
       <c r="BR6" t="inlineStr"/>
       <c r="BS6" t="n">
-        <v>-19943.18181818182</v>
+        <v>-0.01288691298282063</v>
       </c>
       <c r="BT6" t="n">
+        <v>-1.497727272727246</v>
+      </c>
+      <c r="BU6" t="n">
+        <v>0.04241022310071685</v>
+      </c>
+      <c r="BV6" t="inlineStr"/>
+      <c r="BW6" t="n">
         <v>0.3419191919191746</v>
-      </c>
-      <c r="BU6" t="n">
-        <v>-0.01288691298282063</v>
-      </c>
-      <c r="BV6" t="n">
-        <v>-21133.82785633424</v>
-      </c>
-      <c r="BW6" t="n">
-        <v>67967.17171717249</v>
       </c>
     </row>
     <row r="7">
@@ -2127,55 +2127,55 @@
       <c r="BA7" t="n">
         <v>0.207843137254902</v>
       </c>
-      <c r="BB7" t="n">
-        <v>0.03854166666667425</v>
-      </c>
+      <c r="BB7" t="inlineStr"/>
       <c r="BC7" t="n">
-        <v>0.2460457700815013</v>
+        <v>35804129.59060227</v>
       </c>
       <c r="BD7" t="n">
-        <v>-1.049348124510971</v>
+        <v>9.101539734202262</v>
       </c>
       <c r="BE7" t="inlineStr"/>
       <c r="BF7" t="n">
+        <v>7.222887114724699</v>
+      </c>
+      <c r="BG7" t="n">
+        <v>0.03854166666667425</v>
+      </c>
+      <c r="BH7" t="inlineStr"/>
+      <c r="BI7" t="inlineStr"/>
+      <c r="BJ7" t="inlineStr"/>
+      <c r="BK7" t="n">
+        <v>98349.89435098114</v>
+      </c>
+      <c r="BL7" t="n">
         <v>2.009690656565657</v>
       </c>
-      <c r="BG7" t="inlineStr"/>
-      <c r="BH7" t="inlineStr"/>
-      <c r="BI7" t="n">
+      <c r="BM7" t="n">
         <v>10.67414772727273</v>
       </c>
-      <c r="BJ7" t="n">
-        <v>35804129.59060227</v>
-      </c>
-      <c r="BK7" t="inlineStr"/>
-      <c r="BL7" t="n">
-        <v>7.222887114724699</v>
-      </c>
-      <c r="BM7" t="inlineStr"/>
-      <c r="BN7" t="n">
-        <v>9.101539734202262</v>
-      </c>
-      <c r="BO7" t="inlineStr"/>
-      <c r="BP7" t="inlineStr"/>
+      <c r="BN7" t="inlineStr"/>
+      <c r="BO7" t="n">
+        <v>52571476.48358586</v>
+      </c>
+      <c r="BP7" t="n">
+        <v>0.2460457700815013</v>
+      </c>
       <c r="BQ7" t="n">
-        <v>-1.230271464646506</v>
+        <v>137232.0075757576</v>
       </c>
       <c r="BR7" t="inlineStr"/>
       <c r="BS7" t="n">
-        <v>137232.0075757576</v>
+        <v>1.424771625063485</v>
       </c>
       <c r="BT7" t="n">
+        <v>-1.230271464646506</v>
+      </c>
+      <c r="BU7" t="n">
+        <v>-1.049348124510971</v>
+      </c>
+      <c r="BV7" t="inlineStr"/>
+      <c r="BW7" t="n">
         <v>9.348358585858591</v>
-      </c>
-      <c r="BU7" t="n">
-        <v>1.424771625063485</v>
-      </c>
-      <c r="BV7" t="n">
-        <v>98349.89435098114</v>
-      </c>
-      <c r="BW7" t="n">
-        <v>52571476.48358586</v>
       </c>
     </row>
     <row r="8">
@@ -2356,55 +2356,55 @@
       <c r="BA8" t="n">
         <v>0.1184615384615385</v>
       </c>
-      <c r="BB8" t="n">
-        <v>0.5215909090909108</v>
-      </c>
+      <c r="BB8" t="inlineStr"/>
       <c r="BC8" t="n">
-        <v>-0.5951404901465409</v>
+        <v>8484345.249946849</v>
       </c>
       <c r="BD8" t="n">
-        <v>1.741896787969409</v>
+        <v>1.501648431935351</v>
       </c>
       <c r="BE8" t="inlineStr"/>
       <c r="BF8" t="n">
+        <v>2.302561765206036</v>
+      </c>
+      <c r="BG8" t="n">
+        <v>0.5215909090909108</v>
+      </c>
+      <c r="BH8" t="inlineStr"/>
+      <c r="BI8" t="inlineStr"/>
+      <c r="BJ8" t="inlineStr"/>
+      <c r="BK8" t="n">
+        <v>35146.45672060344</v>
+      </c>
+      <c r="BL8" t="n">
         <v>1.134375</v>
       </c>
-      <c r="BG8" t="inlineStr"/>
-      <c r="BH8" t="inlineStr"/>
-      <c r="BI8" t="n">
+      <c r="BM8" t="n">
         <v>3.298200757575756</v>
       </c>
-      <c r="BJ8" t="n">
-        <v>8484345.249946849</v>
-      </c>
-      <c r="BK8" t="inlineStr"/>
-      <c r="BL8" t="n">
-        <v>2.302561765206036</v>
-      </c>
-      <c r="BM8" t="inlineStr"/>
-      <c r="BN8" t="n">
-        <v>1.501648431935351</v>
-      </c>
-      <c r="BO8" t="inlineStr"/>
-      <c r="BP8" t="inlineStr"/>
+      <c r="BN8" t="inlineStr"/>
+      <c r="BO8" t="n">
+        <v>14494977.9040404</v>
+      </c>
+      <c r="BP8" t="n">
+        <v>-0.5951404901465409</v>
+      </c>
       <c r="BQ8" t="n">
-        <v>2.80495580808082</v>
+        <v>54298.1691919192</v>
       </c>
       <c r="BR8" t="inlineStr"/>
       <c r="BS8" t="n">
-        <v>54298.1691919192</v>
+        <v>0.436614441690621</v>
       </c>
       <c r="BT8" t="n">
+        <v>2.80495580808082</v>
+      </c>
+      <c r="BU8" t="n">
+        <v>1.741896787969409</v>
+      </c>
+      <c r="BV8" t="inlineStr"/>
+      <c r="BW8" t="n">
         <v>2.749368686868678</v>
-      </c>
-      <c r="BU8" t="n">
-        <v>0.436614441690621</v>
-      </c>
-      <c r="BV8" t="n">
-        <v>35146.45672060344</v>
-      </c>
-      <c r="BW8" t="n">
-        <v>14494977.9040404</v>
       </c>
     </row>
     <row r="9">
@@ -2585,55 +2585,55 @@
       <c r="BA9" t="n">
         <v>0.1481481481481481</v>
       </c>
-      <c r="BB9" t="n">
-        <v>-0.7299262465929139</v>
-      </c>
+      <c r="BB9" t="inlineStr"/>
       <c r="BC9" t="n">
-        <v>-4.427089826176179</v>
+        <v>-684206.1642206907</v>
       </c>
       <c r="BD9" t="n">
-        <v>-0.4583955896267753</v>
+        <v>-2.659498215030027</v>
       </c>
       <c r="BE9" t="inlineStr"/>
       <c r="BF9" t="n">
+        <v>2.399412692790548</v>
+      </c>
+      <c r="BG9" t="n">
+        <v>-0.7299262465929139</v>
+      </c>
+      <c r="BH9" t="inlineStr"/>
+      <c r="BI9" t="inlineStr"/>
+      <c r="BJ9" t="inlineStr"/>
+      <c r="BK9" t="n">
+        <v>96.88048623976647</v>
+      </c>
+      <c r="BL9" t="n">
         <v>0.09098925765592436</v>
       </c>
-      <c r="BG9" t="inlineStr"/>
-      <c r="BH9" t="inlineStr"/>
-      <c r="BI9" t="n">
+      <c r="BM9" t="n">
         <v>-1.107050665383994</v>
       </c>
-      <c r="BJ9" t="n">
-        <v>-684206.1642206907</v>
-      </c>
-      <c r="BK9" t="inlineStr"/>
-      <c r="BL9" t="n">
-        <v>2.399412692790548</v>
-      </c>
-      <c r="BM9" t="inlineStr"/>
-      <c r="BN9" t="n">
-        <v>-2.659498215030027</v>
-      </c>
-      <c r="BO9" t="inlineStr"/>
-      <c r="BP9" t="inlineStr"/>
+      <c r="BN9" t="inlineStr"/>
+      <c r="BO9" t="n">
+        <v>-1186740.820907485</v>
+      </c>
+      <c r="BP9" t="n">
+        <v>-4.427089826176179</v>
+      </c>
       <c r="BQ9" t="n">
-        <v>0.7776895943562749</v>
+        <v>10373.68125701458</v>
       </c>
       <c r="BR9" t="inlineStr"/>
       <c r="BS9" t="n">
-        <v>10373.68125701458</v>
+        <v>-0.1042685620118655</v>
       </c>
       <c r="BT9" t="n">
+        <v>0.7776895943562749</v>
+      </c>
+      <c r="BU9" t="n">
+        <v>-0.4583955896267753</v>
+      </c>
+      <c r="BV9" t="inlineStr"/>
+      <c r="BW9" t="n">
         <v>0.2592111592111621</v>
-      </c>
-      <c r="BU9" t="n">
-        <v>-0.1042685620118655</v>
-      </c>
-      <c r="BV9" t="n">
-        <v>96.88048623976647</v>
-      </c>
-      <c r="BW9" t="n">
-        <v>-1186740.820907485</v>
       </c>
     </row>
     <row r="10">
@@ -2814,55 +2814,55 @@
       <c r="BA10" t="n">
         <v>-0.1666666666666667</v>
       </c>
-      <c r="BB10" t="n">
-        <v>-0.1743686868686858</v>
-      </c>
+      <c r="BB10" t="inlineStr"/>
       <c r="BC10" t="n">
-        <v>-2.969934094495496</v>
+        <v>2822461.216699156</v>
       </c>
       <c r="BD10" t="n">
-        <v>0.5920043163464186</v>
+        <v>-0.1582944630093834</v>
       </c>
       <c r="BE10" t="inlineStr"/>
       <c r="BF10" t="n">
+        <v>4.296953610879044</v>
+      </c>
+      <c r="BG10" t="n">
+        <v>-0.1743686868686858</v>
+      </c>
+      <c r="BH10" t="inlineStr"/>
+      <c r="BI10" t="inlineStr"/>
+      <c r="BJ10" t="inlineStr"/>
+      <c r="BK10" t="n">
+        <v>3336.487631114825</v>
+      </c>
+      <c r="BL10" t="n">
         <v>0.1049277497194168</v>
       </c>
-      <c r="BG10" t="inlineStr"/>
-      <c r="BH10" t="inlineStr"/>
-      <c r="BI10" t="n">
+      <c r="BM10" t="n">
         <v>1.54325547138049</v>
       </c>
-      <c r="BJ10" t="n">
-        <v>2822461.216699156</v>
-      </c>
-      <c r="BK10" t="inlineStr"/>
-      <c r="BL10" t="n">
-        <v>4.296953610879044</v>
-      </c>
-      <c r="BM10" t="inlineStr"/>
-      <c r="BN10" t="n">
-        <v>-0.1582944630093834</v>
-      </c>
-      <c r="BO10" t="inlineStr"/>
-      <c r="BP10" t="inlineStr"/>
+      <c r="BN10" t="inlineStr"/>
+      <c r="BO10" t="n">
+        <v>4415765.642536476</v>
+      </c>
+      <c r="BP10" t="n">
+        <v>-2.969934094495496</v>
+      </c>
       <c r="BQ10" t="n">
-        <v>1.106684904601536</v>
+        <v>11623.15867003368</v>
       </c>
       <c r="BR10" t="inlineStr"/>
       <c r="BS10" t="n">
-        <v>11623.15867003368</v>
+        <v>0.03321266128283695</v>
       </c>
       <c r="BT10" t="n">
+        <v>1.106684904601536</v>
+      </c>
+      <c r="BU10" t="n">
+        <v>0.5920043163464186</v>
+      </c>
+      <c r="BV10" t="inlineStr"/>
+      <c r="BW10" t="n">
         <v>2.037338664421995</v>
-      </c>
-      <c r="BU10" t="n">
-        <v>0.03321266128283695</v>
-      </c>
-      <c r="BV10" t="n">
-        <v>3336.487631114825</v>
-      </c>
-      <c r="BW10" t="n">
-        <v>4415765.642536476</v>
       </c>
     </row>
     <row r="11">
@@ -3043,55 +3043,55 @@
       <c r="BA11" t="n">
         <v>0.3903448275862069</v>
       </c>
-      <c r="BB11" t="n">
-        <v>0.1518518518518484</v>
-      </c>
+      <c r="BB11" t="inlineStr"/>
       <c r="BC11" t="n">
-        <v>1.020766590018074</v>
+        <v>-3813254.489539482</v>
       </c>
       <c r="BD11" t="n">
-        <v>-3.824580906924183</v>
+        <v>-2.171178431167789</v>
       </c>
       <c r="BE11" t="inlineStr"/>
       <c r="BF11" t="n">
+        <v>-1.689904644850131</v>
+      </c>
+      <c r="BG11" t="n">
+        <v>0.1518518518518484</v>
+      </c>
+      <c r="BH11" t="inlineStr"/>
+      <c r="BI11" t="inlineStr"/>
+      <c r="BJ11" t="inlineStr"/>
+      <c r="BK11" t="n">
+        <v>-10611.53881264981</v>
+      </c>
+      <c r="BL11" t="n">
         <v>0.02195767195767195</v>
       </c>
-      <c r="BG11" t="inlineStr"/>
-      <c r="BH11" t="inlineStr"/>
-      <c r="BI11" t="n">
+      <c r="BM11" t="n">
         <v>-1.519532627865942</v>
       </c>
-      <c r="BJ11" t="n">
-        <v>-3813254.489539482</v>
-      </c>
-      <c r="BK11" t="inlineStr"/>
-      <c r="BL11" t="n">
-        <v>-1.689904644850131</v>
-      </c>
-      <c r="BM11" t="inlineStr"/>
-      <c r="BN11" t="n">
-        <v>-2.171178431167789</v>
-      </c>
-      <c r="BO11" t="inlineStr"/>
-      <c r="BP11" t="inlineStr"/>
+      <c r="BN11" t="inlineStr"/>
+      <c r="BO11" t="n">
+        <v>-4281528.880070546</v>
+      </c>
+      <c r="BP11" t="n">
+        <v>1.020766590018074</v>
+      </c>
       <c r="BQ11" t="n">
-        <v>-2.306790123456778</v>
+        <v>-13474.51499118166</v>
       </c>
       <c r="BR11" t="inlineStr"/>
       <c r="BS11" t="n">
-        <v>-13474.51499118166</v>
+        <v>0.05176677396104612</v>
       </c>
       <c r="BT11" t="n">
+        <v>-2.306790123456778</v>
+      </c>
+      <c r="BU11" t="n">
+        <v>-3.824580906924183</v>
+      </c>
+      <c r="BV11" t="inlineStr"/>
+      <c r="BW11" t="n">
         <v>-1.130731922398581</v>
-      </c>
-      <c r="BU11" t="n">
-        <v>0.05176677396104612</v>
-      </c>
-      <c r="BV11" t="n">
-        <v>-10611.53881264981</v>
-      </c>
-      <c r="BW11" t="n">
-        <v>-4281528.880070546</v>
       </c>
     </row>
     <row r="12">
@@ -3272,55 +3272,55 @@
       <c r="BA12" t="n">
         <v>-0.1467236467236467</v>
       </c>
-      <c r="BB12" t="n">
-        <v>0.9830246913580289</v>
-      </c>
+      <c r="BB12" t="inlineStr"/>
       <c r="BC12" t="n">
-        <v>-2.026167315787735</v>
+        <v>1123258.88149208</v>
       </c>
       <c r="BD12" t="n">
-        <v>0.3498391096204614</v>
+        <v>1.212546414653929</v>
       </c>
       <c r="BE12" t="inlineStr"/>
       <c r="BF12" t="n">
+        <v>1.745381994393526</v>
+      </c>
+      <c r="BG12" t="n">
+        <v>0.9830246913580289</v>
+      </c>
+      <c r="BH12" t="inlineStr"/>
+      <c r="BI12" t="inlineStr"/>
+      <c r="BJ12" t="inlineStr"/>
+      <c r="BK12" t="n">
+        <v>-7092.817759856909</v>
+      </c>
+      <c r="BL12" t="n">
         <v>-0.1164021164021163</v>
       </c>
-      <c r="BG12" t="inlineStr"/>
-      <c r="BH12" t="inlineStr"/>
-      <c r="BI12" t="n">
+      <c r="BM12" t="n">
         <v>-1.629232804232814</v>
       </c>
-      <c r="BJ12" t="n">
-        <v>1123258.88149208</v>
-      </c>
-      <c r="BK12" t="inlineStr"/>
-      <c r="BL12" t="n">
-        <v>1.745381994393526</v>
-      </c>
-      <c r="BM12" t="inlineStr"/>
-      <c r="BN12" t="n">
-        <v>1.212546414653929</v>
-      </c>
-      <c r="BO12" t="inlineStr"/>
-      <c r="BP12" t="inlineStr"/>
+      <c r="BN12" t="inlineStr"/>
+      <c r="BO12" t="n">
+        <v>-7753386.243386243</v>
+      </c>
+      <c r="BP12" t="n">
+        <v>-2.026167315787735</v>
+      </c>
       <c r="BQ12" t="n">
-        <v>0.631481481481444</v>
+        <v>-15546.16402116401</v>
       </c>
       <c r="BR12" t="inlineStr"/>
       <c r="BS12" t="n">
-        <v>-15546.16402116401</v>
+        <v>0.1609137687504563</v>
       </c>
       <c r="BT12" t="n">
+        <v>0.631481481481444</v>
+      </c>
+      <c r="BU12" t="n">
+        <v>0.3498391096204614</v>
+      </c>
+      <c r="BV12" t="inlineStr"/>
+      <c r="BW12" t="n">
         <v>-1.931922398589066</v>
-      </c>
-      <c r="BU12" t="n">
-        <v>0.1609137687504563</v>
-      </c>
-      <c r="BV12" t="n">
-        <v>-7092.817759856909</v>
-      </c>
-      <c r="BW12" t="n">
-        <v>-7753386.243386243</v>
       </c>
     </row>
     <row r="13">
@@ -3501,55 +3501,55 @@
       <c r="BA13" t="n">
         <v>0.2542857142857143</v>
       </c>
-      <c r="BB13" t="n">
-        <v>3.63914141414141</v>
-      </c>
+      <c r="BB13" t="inlineStr"/>
       <c r="BC13" t="n">
-        <v>1.514884621163226</v>
+        <v>5949885.115361378</v>
       </c>
       <c r="BD13" t="n">
-        <v>2.054964922091642</v>
+        <v>1.2627298481775</v>
       </c>
       <c r="BE13" t="inlineStr"/>
       <c r="BF13" t="n">
+        <v>-0.1197859507642107</v>
+      </c>
+      <c r="BG13" t="n">
+        <v>3.63914141414141</v>
+      </c>
+      <c r="BH13" t="inlineStr"/>
+      <c r="BI13" t="inlineStr"/>
+      <c r="BJ13" t="inlineStr"/>
+      <c r="BK13" t="n">
+        <v>-3590.164421771973</v>
+      </c>
+      <c r="BL13" t="n">
         <v>1.302146464646466</v>
       </c>
-      <c r="BG13" t="inlineStr"/>
-      <c r="BH13" t="inlineStr"/>
-      <c r="BI13" t="n">
+      <c r="BM13" t="n">
         <v>3.878156565656568</v>
       </c>
-      <c r="BJ13" t="n">
-        <v>5949885.115361378</v>
-      </c>
-      <c r="BK13" t="inlineStr"/>
-      <c r="BL13" t="n">
-        <v>-0.1197859507642107</v>
-      </c>
-      <c r="BM13" t="inlineStr"/>
-      <c r="BN13" t="n">
-        <v>1.2627298481775</v>
-      </c>
-      <c r="BO13" t="inlineStr"/>
-      <c r="BP13" t="inlineStr"/>
+      <c r="BN13" t="inlineStr"/>
+      <c r="BO13" t="n">
+        <v>18043813.13131313</v>
+      </c>
+      <c r="BP13" t="n">
+        <v>1.514884621163226</v>
+      </c>
       <c r="BQ13" t="n">
-        <v>0.5243686868686552</v>
+        <v>31671.59090909094</v>
       </c>
       <c r="BR13" t="inlineStr"/>
       <c r="BS13" t="n">
-        <v>31671.59090909094</v>
+        <v>0.4619302052511434</v>
       </c>
       <c r="BT13" t="n">
+        <v>0.5243686868686552</v>
+      </c>
+      <c r="BU13" t="n">
+        <v>2.054964922091642</v>
+      </c>
+      <c r="BV13" t="inlineStr"/>
+      <c r="BW13" t="n">
         <v>1.240025252525243</v>
-      </c>
-      <c r="BU13" t="n">
-        <v>0.4619302052511434</v>
-      </c>
-      <c r="BV13" t="n">
-        <v>-3590.164421771973</v>
-      </c>
-      <c r="BW13" t="n">
-        <v>18043813.13131313</v>
       </c>
     </row>
     <row r="14">
@@ -3730,55 +3730,55 @@
       <c r="BA14" t="n">
         <v>-0.1288888888888889</v>
       </c>
-      <c r="BB14" t="n">
-        <v>0.2765873015873019</v>
-      </c>
+      <c r="BB14" t="inlineStr"/>
       <c r="BC14" t="n">
-        <v>1.97873456558635</v>
+        <v>-29208527.81258821</v>
       </c>
       <c r="BD14" t="n">
-        <v>1.042361877947855</v>
+        <v>-4.008702372427862</v>
       </c>
       <c r="BE14" t="inlineStr"/>
       <c r="BF14" t="n">
+        <v>-5.266013449079111</v>
+      </c>
+      <c r="BG14" t="n">
+        <v>0.2765873015873019</v>
+      </c>
+      <c r="BH14" t="inlineStr"/>
+      <c r="BI14" t="inlineStr"/>
+      <c r="BJ14" t="inlineStr"/>
+      <c r="BK14" t="n">
+        <v>-80998.16741530169</v>
+      </c>
+      <c r="BL14" t="n">
         <v>-1.822835497835498</v>
       </c>
-      <c r="BG14" t="inlineStr"/>
-      <c r="BH14" t="inlineStr"/>
-      <c r="BI14" t="n">
+      <c r="BM14" t="n">
         <v>-7.384812409812412</v>
       </c>
-      <c r="BJ14" t="n">
-        <v>-29208527.81258821</v>
-      </c>
-      <c r="BK14" t="inlineStr"/>
-      <c r="BL14" t="n">
-        <v>-5.266013449079111</v>
-      </c>
-      <c r="BM14" t="inlineStr"/>
-      <c r="BN14" t="n">
-        <v>-4.008702372427862</v>
-      </c>
-      <c r="BO14" t="inlineStr"/>
-      <c r="BP14" t="inlineStr"/>
+      <c r="BN14" t="inlineStr"/>
+      <c r="BO14" t="n">
+        <v>-46137494.5887446</v>
+      </c>
+      <c r="BP14" t="n">
+        <v>1.97873456558635</v>
+      </c>
       <c r="BQ14" t="n">
-        <v>1.306709956709966</v>
+        <v>-129942.4242424242</v>
       </c>
       <c r="BR14" t="inlineStr"/>
       <c r="BS14" t="n">
-        <v>-129942.4242424242</v>
+        <v>-1.162400109028399</v>
       </c>
       <c r="BT14" t="n">
+        <v>1.306709956709966</v>
+      </c>
+      <c r="BU14" t="n">
+        <v>1.042361877947855</v>
+      </c>
+      <c r="BV14" t="inlineStr"/>
+      <c r="BW14" t="n">
         <v>-6.294985569985585</v>
-      </c>
-      <c r="BU14" t="n">
-        <v>-1.162400109028399</v>
-      </c>
-      <c r="BV14" t="n">
-        <v>-80998.16741530169</v>
-      </c>
-      <c r="BW14" t="n">
-        <v>-46137494.5887446</v>
       </c>
     </row>
     <row r="15">
@@ -3959,55 +3959,55 @@
       <c r="BA15" t="n">
         <v>-0.4400000000000001</v>
       </c>
-      <c r="BB15" t="n">
-        <v>-0.01701388888888289</v>
-      </c>
+      <c r="BB15" t="inlineStr"/>
       <c r="BC15" t="n">
-        <v>-0.1816396292858933</v>
+        <v>-20532666.19179343</v>
       </c>
       <c r="BD15" t="n">
-        <v>1.24357916699671</v>
+        <v>-3.445223900850493</v>
       </c>
       <c r="BE15" t="inlineStr"/>
       <c r="BF15" t="n">
+        <v>-4.364642644138314</v>
+      </c>
+      <c r="BG15" t="n">
+        <v>-0.01701388888888289</v>
+      </c>
+      <c r="BH15" t="inlineStr"/>
+      <c r="BI15" t="inlineStr"/>
+      <c r="BJ15" t="inlineStr"/>
+      <c r="BK15" t="n">
+        <v>-65235.93873934748</v>
+      </c>
+      <c r="BL15" t="n">
         <v>-2.071874999999999</v>
       </c>
-      <c r="BG15" t="inlineStr"/>
-      <c r="BH15" t="inlineStr"/>
-      <c r="BI15" t="n">
+      <c r="BM15" t="n">
         <v>-6.946875000000006</v>
       </c>
-      <c r="BJ15" t="n">
-        <v>-20532666.19179343</v>
-      </c>
-      <c r="BK15" t="inlineStr"/>
-      <c r="BL15" t="n">
-        <v>-4.364642644138314</v>
-      </c>
-      <c r="BM15" t="inlineStr"/>
-      <c r="BN15" t="n">
-        <v>-3.445223900850493</v>
-      </c>
-      <c r="BO15" t="inlineStr"/>
-      <c r="BP15" t="inlineStr"/>
+      <c r="BN15" t="inlineStr"/>
+      <c r="BO15" t="n">
+        <v>-42905173.61111112</v>
+      </c>
+      <c r="BP15" t="n">
+        <v>-0.1816396292858933</v>
+      </c>
       <c r="BQ15" t="n">
-        <v>-1.167013888888903</v>
+        <v>-97262.5</v>
       </c>
       <c r="BR15" t="inlineStr"/>
       <c r="BS15" t="n">
-        <v>-97262.5</v>
+        <v>-1.34844265566772</v>
       </c>
       <c r="BT15" t="n">
+        <v>-1.167013888888903</v>
+      </c>
+      <c r="BU15" t="n">
+        <v>1.24357916699671</v>
+      </c>
+      <c r="BV15" t="inlineStr"/>
+      <c r="BW15" t="n">
         <v>-5.993055555555557</v>
-      </c>
-      <c r="BU15" t="n">
-        <v>-1.34844265566772</v>
-      </c>
-      <c r="BV15" t="n">
-        <v>-65235.93873934748</v>
-      </c>
-      <c r="BW15" t="n">
-        <v>-42905173.61111112</v>
       </c>
     </row>
     <row r="16">
@@ -4188,55 +4188,55 @@
       <c r="BA16" t="n">
         <v>0.07999999999999999</v>
       </c>
-      <c r="BB16" t="n">
-        <v>0.7204545454545475</v>
-      </c>
+      <c r="BB16" t="inlineStr"/>
       <c r="BC16" t="n">
-        <v>3.217024878346148</v>
+        <v>14425041.38395312</v>
       </c>
       <c r="BD16" t="n">
-        <v>2.880522051656925</v>
+        <v>6.005314256081803</v>
       </c>
       <c r="BE16" t="inlineStr"/>
       <c r="BF16" t="n">
+        <v>2.391393458718028</v>
+      </c>
+      <c r="BG16" t="n">
+        <v>0.7204545454545475</v>
+      </c>
+      <c r="BH16" t="inlineStr"/>
+      <c r="BI16" t="inlineStr"/>
+      <c r="BJ16" t="inlineStr"/>
+      <c r="BK16" t="n">
+        <v>40492.08068470678</v>
+      </c>
+      <c r="BL16" t="n">
         <v>1.341045374378707</v>
       </c>
-      <c r="BG16" t="inlineStr"/>
-      <c r="BH16" t="inlineStr"/>
-      <c r="BI16" t="n">
+      <c r="BM16" t="n">
         <v>4.943843193843193</v>
       </c>
-      <c r="BJ16" t="n">
-        <v>14425041.38395312</v>
-      </c>
-      <c r="BK16" t="inlineStr"/>
-      <c r="BL16" t="n">
-        <v>2.391393458718028</v>
-      </c>
-      <c r="BM16" t="inlineStr"/>
-      <c r="BN16" t="n">
-        <v>6.005314256081803</v>
-      </c>
-      <c r="BO16" t="inlineStr"/>
-      <c r="BP16" t="inlineStr"/>
+      <c r="BN16" t="inlineStr"/>
+      <c r="BO16" t="n">
+        <v>20403810.02485169</v>
+      </c>
+      <c r="BP16" t="n">
+        <v>3.217024878346148</v>
+      </c>
       <c r="BQ16" t="n">
-        <v>-1.337826679493361</v>
+        <v>45265.71669071668</v>
       </c>
       <c r="BR16" t="inlineStr"/>
       <c r="BS16" t="n">
-        <v>45265.71669071668</v>
+        <v>0.9712415833029868</v>
       </c>
       <c r="BT16" t="n">
+        <v>-1.337826679493361</v>
+      </c>
+      <c r="BU16" t="n">
+        <v>2.880522051656925</v>
+      </c>
+      <c r="BV16" t="inlineStr"/>
+      <c r="BW16" t="n">
         <v>3.704553471220137</v>
-      </c>
-      <c r="BU16" t="n">
-        <v>0.9712415833029868</v>
-      </c>
-      <c r="BV16" t="n">
-        <v>40492.08068470678</v>
-      </c>
-      <c r="BW16" t="n">
-        <v>20403810.02485169</v>
       </c>
     </row>
     <row r="17">
@@ -4419,55 +4419,55 @@
       <c r="BA17" t="n">
         <v>0.6121794871794872</v>
       </c>
-      <c r="BB17" t="n">
-        <v>1.571773288439953</v>
-      </c>
+      <c r="BB17" t="inlineStr"/>
       <c r="BC17" t="n">
-        <v>3.540241354730181</v>
+        <v>9014180.380404595</v>
       </c>
       <c r="BD17" t="n">
-        <v>3.217460965732897</v>
+        <v>4.276960797263001</v>
       </c>
       <c r="BE17" t="inlineStr"/>
       <c r="BF17" t="n">
+        <v>-0.3816575081364988</v>
+      </c>
+      <c r="BG17" t="n">
+        <v>1.571773288439953</v>
+      </c>
+      <c r="BH17" t="inlineStr"/>
+      <c r="BI17" t="inlineStr"/>
+      <c r="BJ17" t="inlineStr"/>
+      <c r="BK17" t="n">
+        <v>35371.35706396373</v>
+      </c>
+      <c r="BL17" t="n">
         <v>0.8333613916947249</v>
       </c>
-      <c r="BG17" t="inlineStr"/>
-      <c r="BH17" t="inlineStr"/>
-      <c r="BI17" t="n">
+      <c r="BM17" t="n">
         <v>4.635297418630756</v>
       </c>
-      <c r="BJ17" t="n">
-        <v>9014180.380404595</v>
-      </c>
-      <c r="BK17" t="inlineStr"/>
-      <c r="BL17" t="n">
-        <v>-0.3816575081364988</v>
-      </c>
-      <c r="BM17" t="inlineStr"/>
-      <c r="BN17" t="n">
-        <v>4.276960797263001</v>
-      </c>
-      <c r="BO17" t="inlineStr"/>
-      <c r="BP17" t="inlineStr"/>
+      <c r="BN17" t="inlineStr"/>
+      <c r="BO17" t="n">
+        <v>14434342.7328844</v>
+      </c>
+      <c r="BP17" t="n">
+        <v>3.540241354730181</v>
+      </c>
       <c r="BQ17" t="n">
-        <v>3.384287317620647</v>
+        <v>42706.62177328842</v>
       </c>
       <c r="BR17" t="inlineStr"/>
       <c r="BS17" t="n">
-        <v>42706.62177328842</v>
+        <v>0.6235440233925897</v>
       </c>
       <c r="BT17" t="n">
+        <v>3.384287317620647</v>
+      </c>
+      <c r="BU17" t="n">
+        <v>3.217460965732897</v>
+      </c>
+      <c r="BV17" t="inlineStr"/>
+      <c r="BW17" t="n">
         <v>1.58021885521886</v>
-      </c>
-      <c r="BU17" t="n">
-        <v>0.6235440233925897</v>
-      </c>
-      <c r="BV17" t="n">
-        <v>35371.35706396373</v>
-      </c>
-      <c r="BW17" t="n">
-        <v>14434342.7328844</v>
       </c>
     </row>
     <row r="18">
@@ -4648,55 +4648,55 @@
       <c r="BA18" t="n">
         <v>-0.03703703703703703</v>
       </c>
-      <c r="BB18" t="n">
-        <v>1.165909090909089</v>
-      </c>
+      <c r="BB18" t="inlineStr"/>
       <c r="BC18" t="n">
-        <v>2.801577808156754</v>
+        <v>-10652806.00688906</v>
       </c>
       <c r="BD18" t="n">
-        <v>1.272612403937472</v>
+        <v>-1.830401942562276</v>
       </c>
       <c r="BE18" t="inlineStr"/>
       <c r="BF18" t="n">
+        <v>-3.982160148257123</v>
+      </c>
+      <c r="BG18" t="n">
+        <v>1.165909090909089</v>
+      </c>
+      <c r="BH18" t="inlineStr"/>
+      <c r="BI18" t="inlineStr"/>
+      <c r="BJ18" t="inlineStr"/>
+      <c r="BK18" t="n">
+        <v>-20473.58631640312</v>
+      </c>
+      <c r="BL18" t="n">
         <v>-0.8611111111111109</v>
       </c>
-      <c r="BG18" t="inlineStr"/>
-      <c r="BH18" t="inlineStr"/>
-      <c r="BI18" t="n">
+      <c r="BM18" t="n">
         <v>-2.971464646464639</v>
       </c>
-      <c r="BJ18" t="n">
-        <v>-10652806.00688906</v>
-      </c>
-      <c r="BK18" t="inlineStr"/>
-      <c r="BL18" t="n">
-        <v>-3.982160148257123</v>
-      </c>
-      <c r="BM18" t="inlineStr"/>
-      <c r="BN18" t="n">
-        <v>-1.830401942562276</v>
-      </c>
-      <c r="BO18" t="inlineStr"/>
-      <c r="BP18" t="inlineStr"/>
+      <c r="BN18" t="inlineStr"/>
+      <c r="BO18" t="n">
+        <v>-15010568.18181818</v>
+      </c>
+      <c r="BP18" t="n">
+        <v>2.801577808156754</v>
+      </c>
       <c r="BQ18" t="n">
-        <v>0.4613636363636431</v>
+        <v>-37233.58585858587</v>
       </c>
       <c r="BR18" t="inlineStr"/>
       <c r="BS18" t="n">
-        <v>-37233.58585858587</v>
+        <v>-0.2646361027046098</v>
       </c>
       <c r="BT18" t="n">
+        <v>0.4613636363636431</v>
+      </c>
+      <c r="BU18" t="n">
+        <v>1.272612403937472</v>
+      </c>
+      <c r="BV18" t="inlineStr"/>
+      <c r="BW18" t="n">
         <v>-3.886868686868667</v>
-      </c>
-      <c r="BU18" t="n">
-        <v>-0.2646361027046098</v>
-      </c>
-      <c r="BV18" t="n">
-        <v>-20473.58631640312</v>
-      </c>
-      <c r="BW18" t="n">
-        <v>-15010568.18181818</v>
       </c>
     </row>
     <row r="19">
@@ -4877,55 +4877,55 @@
       <c r="BA19" t="n">
         <v>0.2933333333333333</v>
       </c>
-      <c r="BB19" t="n">
-        <v>-2.467803030303028</v>
-      </c>
+      <c r="BB19" t="inlineStr"/>
       <c r="BC19" t="n">
-        <v>-0.6429093681802662</v>
+        <v>-2405181.613292682</v>
       </c>
       <c r="BD19" t="n">
-        <v>-2.4502429086794</v>
+        <v>-2.137605854614364</v>
       </c>
       <c r="BE19" t="inlineStr"/>
       <c r="BF19" t="n">
+        <v>-2.104906191303257</v>
+      </c>
+      <c r="BG19" t="n">
+        <v>-2.467803030303028</v>
+      </c>
+      <c r="BH19" t="inlineStr"/>
+      <c r="BI19" t="inlineStr"/>
+      <c r="BJ19" t="inlineStr"/>
+      <c r="BK19" t="n">
+        <v>1224.379794755179</v>
+      </c>
+      <c r="BL19" t="n">
         <v>-0.4394255050505051</v>
       </c>
-      <c r="BG19" t="inlineStr"/>
-      <c r="BH19" t="inlineStr"/>
-      <c r="BI19" t="n">
+      <c r="BM19" t="n">
         <v>-2.487405303030314</v>
       </c>
-      <c r="BJ19" t="n">
-        <v>-2405181.613292682</v>
-      </c>
-      <c r="BK19" t="inlineStr"/>
-      <c r="BL19" t="n">
-        <v>-2.104906191303257</v>
-      </c>
-      <c r="BM19" t="inlineStr"/>
-      <c r="BN19" t="n">
-        <v>-2.137605854614364</v>
-      </c>
-      <c r="BO19" t="inlineStr"/>
-      <c r="BP19" t="inlineStr"/>
+      <c r="BN19" t="inlineStr"/>
+      <c r="BO19" t="n">
+        <v>-4719655.934343435</v>
+      </c>
+      <c r="BP19" t="n">
+        <v>-0.6429093681802662</v>
+      </c>
       <c r="BQ19" t="n">
-        <v>0.3784722222222285</v>
+        <v>-3484.185606060608</v>
       </c>
       <c r="BR19" t="inlineStr"/>
       <c r="BS19" t="n">
-        <v>-3484.185606060608</v>
+        <v>-0.213902584916517</v>
       </c>
       <c r="BT19" t="n">
+        <v>0.3784722222222285</v>
+      </c>
+      <c r="BU19" t="n">
+        <v>-2.4502429086794</v>
+      </c>
+      <c r="BV19" t="inlineStr"/>
+      <c r="BW19" t="n">
         <v>-0.8496843434343333</v>
-      </c>
-      <c r="BU19" t="n">
-        <v>-0.213902584916517</v>
-      </c>
-      <c r="BV19" t="n">
-        <v>1224.379794755179</v>
-      </c>
-      <c r="BW19" t="n">
-        <v>-4719655.934343435</v>
       </c>
     </row>
     <row r="20">
@@ -5106,55 +5106,55 @@
       <c r="BA20" t="n">
         <v>-0.0438871473354232</v>
       </c>
-      <c r="BB20" t="n">
-        <v>-0.4598379629629683</v>
-      </c>
+      <c r="BB20" t="inlineStr"/>
       <c r="BC20" t="n">
-        <v>-0.9288341484032934</v>
+        <v>-1854675.709531553</v>
       </c>
       <c r="BD20" t="n">
-        <v>0.4145858618123839</v>
+        <v>-2.767859395220071</v>
       </c>
       <c r="BE20" t="inlineStr"/>
       <c r="BF20" t="n">
+        <v>-0.5539894497582765</v>
+      </c>
+      <c r="BG20" t="n">
+        <v>-0.4598379629629683</v>
+      </c>
+      <c r="BH20" t="inlineStr"/>
+      <c r="BI20" t="inlineStr"/>
+      <c r="BJ20" t="inlineStr"/>
+      <c r="BK20" t="n">
+        <v>-3936.283575099369</v>
+      </c>
+      <c r="BL20" t="n">
         <v>-0.08182870370370376</v>
       </c>
-      <c r="BG20" t="inlineStr"/>
-      <c r="BH20" t="inlineStr"/>
-      <c r="BI20" t="n">
+      <c r="BM20" t="n">
         <v>-2.224961419753086</v>
       </c>
-      <c r="BJ20" t="n">
-        <v>-1854675.709531553</v>
-      </c>
-      <c r="BK20" t="inlineStr"/>
-      <c r="BL20" t="n">
-        <v>-0.5539894497582765</v>
-      </c>
-      <c r="BM20" t="inlineStr"/>
-      <c r="BN20" t="n">
-        <v>-2.767859395220071</v>
-      </c>
-      <c r="BO20" t="inlineStr"/>
-      <c r="BP20" t="inlineStr"/>
+      <c r="BN20" t="inlineStr"/>
+      <c r="BO20" t="n">
+        <v>-1515984.760802469</v>
+      </c>
+      <c r="BP20" t="n">
+        <v>-0.9288341484032934</v>
+      </c>
       <c r="BQ20" t="n">
-        <v>1.327970679012367</v>
+        <v>3885.725308641966</v>
       </c>
       <c r="BR20" t="inlineStr"/>
       <c r="BS20" t="n">
-        <v>3885.725308641966</v>
+        <v>-0.1022361806675531</v>
       </c>
       <c r="BT20" t="n">
+        <v>1.327970679012367</v>
+      </c>
+      <c r="BU20" t="n">
+        <v>0.4145858618123839</v>
+      </c>
+      <c r="BV20" t="inlineStr"/>
+      <c r="BW20" t="n">
         <v>-1.079783950617283</v>
-      </c>
-      <c r="BU20" t="n">
-        <v>-0.1022361806675531</v>
-      </c>
-      <c r="BV20" t="n">
-        <v>-3936.283575099369</v>
-      </c>
-      <c r="BW20" t="n">
-        <v>-1515984.760802469</v>
       </c>
     </row>
     <row r="21">
@@ -5335,55 +5335,55 @@
       <c r="BA21" t="n">
         <v>0.1185897435897436</v>
       </c>
-      <c r="BB21" t="n">
-        <v>-2.672045855379185</v>
-      </c>
+      <c r="BB21" t="inlineStr"/>
       <c r="BC21" t="n">
-        <v>-4.27549750086515</v>
+        <v>6778035.877294458</v>
       </c>
       <c r="BD21" t="n">
-        <v>3.778172753172782</v>
+        <v>0.159866381802658</v>
       </c>
       <c r="BE21" t="inlineStr"/>
       <c r="BF21" t="n">
+        <v>2.840250775912537</v>
+      </c>
+      <c r="BG21" t="n">
+        <v>-2.672045855379185</v>
+      </c>
+      <c r="BH21" t="inlineStr"/>
+      <c r="BI21" t="inlineStr"/>
+      <c r="BJ21" t="inlineStr"/>
+      <c r="BK21" t="n">
+        <v>-820.8898672133946</v>
+      </c>
+      <c r="BL21" t="n">
         <v>0.4560405643738972</v>
       </c>
-      <c r="BG21" t="inlineStr"/>
-      <c r="BH21" t="inlineStr"/>
-      <c r="BI21" t="n">
+      <c r="BM21" t="n">
         <v>2.647883597883592</v>
       </c>
-      <c r="BJ21" t="n">
-        <v>6778035.877294458</v>
-      </c>
-      <c r="BK21" t="inlineStr"/>
-      <c r="BL21" t="n">
-        <v>2.840250775912537</v>
-      </c>
-      <c r="BM21" t="inlineStr"/>
-      <c r="BN21" t="n">
-        <v>0.159866381802658</v>
-      </c>
-      <c r="BO21" t="inlineStr"/>
-      <c r="BP21" t="inlineStr"/>
+      <c r="BN21" t="inlineStr"/>
+      <c r="BO21" t="n">
+        <v>19174272.48677249</v>
+      </c>
+      <c r="BP21" t="n">
+        <v>-4.27549750086515</v>
+      </c>
       <c r="BQ21" t="n">
-        <v>1.94880952380953</v>
+        <v>24883.86243386244</v>
       </c>
       <c r="BR21" t="inlineStr"/>
       <c r="BS21" t="n">
-        <v>24883.86243386244</v>
+        <v>-0.1476273136812352</v>
       </c>
       <c r="BT21" t="n">
+        <v>1.94880952380953</v>
+      </c>
+      <c r="BU21" t="n">
+        <v>3.778172753172782</v>
+      </c>
+      <c r="BV21" t="inlineStr"/>
+      <c r="BW21" t="n">
         <v>4.045370370370378</v>
-      </c>
-      <c r="BU21" t="n">
-        <v>-0.1476273136812352</v>
-      </c>
-      <c r="BV21" t="n">
-        <v>-820.8898672133946</v>
-      </c>
-      <c r="BW21" t="n">
-        <v>19174272.48677249</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
DATA. Vuelvo a obtener predicciones de proximos 15 dias por error formateo de fecha.
</commit_message>
<xml_diff>
--- a/data/england/p6_deployment/data_preparation/df_constructed.xlsx
+++ b/data/england/p6_deployment/data_preparation/df_constructed.xlsx
@@ -695,112 +695,112 @@
       </c>
       <c r="BB1" s="1" t="inlineStr">
         <is>
+          <t>dif_n_player_miss</t>
+        </is>
+      </c>
+      <c r="BC1" s="1" t="inlineStr">
+        <is>
+          <t>dif_mean_wage_player_start</t>
+        </is>
+      </c>
+      <c r="BD1" s="1" t="inlineStr">
+        <is>
+          <t>dif_mean_age_player_sub</t>
+        </is>
+      </c>
+      <c r="BE1" s="1" t="inlineStr">
+        <is>
           <t>dif_mean_age_player_start</t>
         </is>
       </c>
-      <c r="BC1" s="1" t="inlineStr">
+      <c r="BF1" s="1" t="inlineStr">
+        <is>
+          <t>dif_mean_value_player_sub</t>
+        </is>
+      </c>
+      <c r="BG1" s="1" t="inlineStr">
+        <is>
+          <t>dif_sum_pot_player_miss</t>
+        </is>
+      </c>
+      <c r="BH1" s="1" t="inlineStr">
+        <is>
+          <t>dif_mean_value_player_start</t>
+        </is>
+      </c>
+      <c r="BI1" s="1" t="inlineStr">
+        <is>
+          <t>dif_mean_rep_player_sub</t>
+        </is>
+      </c>
+      <c r="BJ1" s="1" t="inlineStr">
+        <is>
+          <t>dif_mean_hei_player_start</t>
+        </is>
+      </c>
+      <c r="BK1" s="1" t="inlineStr">
+        <is>
+          <t>dif_mean_rat_player_sub</t>
+        </is>
+      </c>
+      <c r="BL1" s="1" t="inlineStr">
+        <is>
+          <t>dif_mean_wage_player_sub</t>
+        </is>
+      </c>
+      <c r="BM1" s="1" t="inlineStr">
+        <is>
+          <t>dif_mean_rat_player_start</t>
+        </is>
+      </c>
+      <c r="BN1" s="1" t="inlineStr">
+        <is>
+          <t>dif_mean_pot_player_start</t>
+        </is>
+      </c>
+      <c r="BO1" s="1" t="inlineStr">
+        <is>
+          <t>dif_sum_rat_player_miss</t>
+        </is>
+      </c>
+      <c r="BP1" s="1" t="inlineStr">
+        <is>
+          <t>dif_sum_value_player_miss</t>
+        </is>
+      </c>
+      <c r="BQ1" s="1" t="inlineStr">
+        <is>
+          <t>dif_sum_wage_player_miss</t>
+        </is>
+      </c>
+      <c r="BR1" s="1" t="inlineStr">
+        <is>
+          <t>dif_mean_pot_player_sub</t>
+        </is>
+      </c>
+      <c r="BS1" s="1" t="inlineStr">
+        <is>
+          <t>dif_mean_age_player_miss</t>
+        </is>
+      </c>
+      <c r="BT1" s="1" t="inlineStr">
         <is>
           <t>dif_mean_rep_player_start</t>
         </is>
       </c>
-      <c r="BD1" s="1" t="inlineStr">
-        <is>
-          <t>dif_mean_age_player_sub</t>
-        </is>
-      </c>
-      <c r="BE1" s="1" t="inlineStr">
-        <is>
-          <t>dif_mean_wage_player_sub</t>
-        </is>
-      </c>
-      <c r="BF1" s="1" t="inlineStr">
-        <is>
-          <t>dif_mean_rep_player_sub</t>
-        </is>
-      </c>
-      <c r="BG1" s="1" t="inlineStr">
+      <c r="BU1" s="1" t="inlineStr">
         <is>
           <t>dif_mean_hei_player_miss</t>
         </is>
       </c>
-      <c r="BH1" s="1" t="inlineStr">
-        <is>
-          <t>dif_mean_pot_player_start</t>
-        </is>
-      </c>
-      <c r="BI1" s="1" t="inlineStr">
-        <is>
-          <t>dif_mean_wage_player_start</t>
-        </is>
-      </c>
-      <c r="BJ1" s="1" t="inlineStr">
-        <is>
-          <t>dif_sum_value_player_miss</t>
-        </is>
-      </c>
-      <c r="BK1" s="1" t="inlineStr">
-        <is>
-          <t>dif_mean_hei_player_start</t>
-        </is>
-      </c>
-      <c r="BL1" s="1" t="inlineStr">
-        <is>
-          <t>dif_n_player_miss</t>
-        </is>
-      </c>
-      <c r="BM1" s="1" t="inlineStr">
-        <is>
-          <t>dif_mean_rat_player_start</t>
-        </is>
-      </c>
-      <c r="BN1" s="1" t="inlineStr">
-        <is>
-          <t>dif_mean_rat_player_sub</t>
-        </is>
-      </c>
-      <c r="BO1" s="1" t="inlineStr">
-        <is>
-          <t>dif_sum_wage_player_miss</t>
-        </is>
-      </c>
-      <c r="BP1" s="1" t="inlineStr">
+      <c r="BV1" s="1" t="inlineStr">
+        <is>
+          <t>dif_mean_hei_player_sub</t>
+        </is>
+      </c>
+      <c r="BW1" s="1" t="inlineStr">
         <is>
           <t>dif_sum_rep_player_miss</t>
-        </is>
-      </c>
-      <c r="BQ1" s="1" t="inlineStr">
-        <is>
-          <t>dif_mean_age_player_miss</t>
-        </is>
-      </c>
-      <c r="BR1" s="1" t="inlineStr">
-        <is>
-          <t>dif_mean_pot_player_sub</t>
-        </is>
-      </c>
-      <c r="BS1" s="1" t="inlineStr">
-        <is>
-          <t>dif_sum_rat_player_miss</t>
-        </is>
-      </c>
-      <c r="BT1" s="1" t="inlineStr">
-        <is>
-          <t>dif_mean_value_player_start</t>
-        </is>
-      </c>
-      <c r="BU1" s="1" t="inlineStr">
-        <is>
-          <t>dif_sum_pot_player_miss</t>
-        </is>
-      </c>
-      <c r="BV1" s="1" t="inlineStr">
-        <is>
-          <t>dif_mean_hei_player_sub</t>
-        </is>
-      </c>
-      <c r="BW1" s="1" t="inlineStr">
-        <is>
-          <t>dif_mean_value_player_sub</t>
         </is>
       </c>
     </row>
@@ -983,70 +983,70 @@
         <v>0.04120879120879123</v>
       </c>
       <c r="BB2" t="n">
-        <v>1.977777777777781</v>
+        <v>-1.885714285714286</v>
       </c>
       <c r="BC2" t="n">
-        <v>0.2969977553310887</v>
+        <v>12651.6835016835</v>
       </c>
       <c r="BD2" t="n">
         <v>3.38421814399122</v>
       </c>
       <c r="BE2" t="n">
+        <v>1.977777777777781</v>
+      </c>
+      <c r="BF2" t="n">
+        <v>643682.7096929122</v>
+      </c>
+      <c r="BG2" t="n">
+        <v>-155.4571428571428</v>
+      </c>
+      <c r="BH2" t="n">
+        <v>363902.9180695843</v>
+      </c>
+      <c r="BI2" t="n">
+        <v>0.1910637604478183</v>
+      </c>
+      <c r="BJ2" t="n">
+        <v>0.1368125701459064</v>
+      </c>
+      <c r="BK2" t="n">
+        <v>2.948807959915897</v>
+      </c>
+      <c r="BL2" t="n">
         <v>17448.06183130934</v>
-      </c>
-      <c r="BF2" t="n">
-        <v>0.1910637604478183</v>
-      </c>
-      <c r="BG2" t="n">
-        <v>11.09047619047621</v>
-      </c>
-      <c r="BH2" t="n">
-        <v>-1.663916947250272</v>
-      </c>
-      <c r="BI2" t="n">
-        <v>12651.6835016835</v>
-      </c>
-      <c r="BJ2" t="n">
-        <v>-32414285.71428572</v>
-      </c>
-      <c r="BK2" t="n">
-        <v>0.1368125701459064</v>
-      </c>
-      <c r="BL2" t="n">
-        <v>-1.885714285714286</v>
       </c>
       <c r="BM2" t="n">
         <v>1.15286195286194</v>
       </c>
       <c r="BN2" t="n">
-        <v>2.948807959915897</v>
+        <v>-1.663916947250272</v>
       </c>
       <c r="BO2" t="n">
+        <v>-148.4571428571429</v>
+      </c>
+      <c r="BP2" t="n">
+        <v>-32414285.71428572</v>
+      </c>
+      <c r="BQ2" t="n">
         <v>-108914.2857142857</v>
-      </c>
-      <c r="BP2" t="n">
-        <v>-1.885714285714286</v>
-      </c>
-      <c r="BQ2" t="n">
-        <v>3.547619047619051</v>
       </c>
       <c r="BR2" t="n">
         <v>-1.638545740357344</v>
       </c>
       <c r="BS2" t="n">
-        <v>-148.4571428571429</v>
+        <v>3.547619047619051</v>
       </c>
       <c r="BT2" t="n">
-        <v>363902.9180695843</v>
+        <v>0.2969977553310887</v>
       </c>
       <c r="BU2" t="n">
-        <v>-155.4571428571428</v>
+        <v>11.09047619047621</v>
       </c>
       <c r="BV2" t="n">
         <v>1.649782971922576</v>
       </c>
       <c r="BW2" t="n">
-        <v>643682.7096929122</v>
+        <v>-1.885714285714286</v>
       </c>
     </row>
     <row r="3">
@@ -1228,70 +1228,70 @@
         <v>0.03846153846153846</v>
       </c>
       <c r="BB3" t="n">
-        <v>3.107936507936508</v>
+        <v>0.3333333333333335</v>
       </c>
       <c r="BC3" t="n">
-        <v>0.6515873015873015</v>
+        <v>2725.39682539682</v>
       </c>
       <c r="BD3" t="n">
         <v>2.812969258446234</v>
       </c>
       <c r="BE3" t="n">
+        <v>3.107936507936508</v>
+      </c>
+      <c r="BF3" t="n">
+        <v>-6718122.031477295</v>
+      </c>
+      <c r="BG3" t="n">
+        <v>32.90476190476193</v>
+      </c>
+      <c r="BH3" t="n">
+        <v>-1224404.761904765</v>
+      </c>
+      <c r="BI3" t="n">
+        <v>0.148175526958422</v>
+      </c>
+      <c r="BJ3" t="n">
+        <v>-0.503571428571405</v>
+      </c>
+      <c r="BK3" t="n">
+        <v>-1.096318666713401</v>
+      </c>
+      <c r="BL3" t="n">
         <v>-16829.46929715024</v>
-      </c>
-      <c r="BF3" t="n">
-        <v>0.148175526958422</v>
-      </c>
-      <c r="BG3" t="n">
-        <v>-0.6706349206349387</v>
-      </c>
-      <c r="BH3" t="n">
-        <v>-0.9416666666666487</v>
-      </c>
-      <c r="BI3" t="n">
-        <v>2725.39682539682</v>
-      </c>
-      <c r="BJ3" t="n">
-        <v>20571428.57142857</v>
-      </c>
-      <c r="BK3" t="n">
-        <v>-0.503571428571405</v>
-      </c>
-      <c r="BL3" t="n">
-        <v>0.3333333333333335</v>
       </c>
       <c r="BM3" t="n">
         <v>0.5498015873015873</v>
       </c>
       <c r="BN3" t="n">
-        <v>-1.096318666713401</v>
+        <v>-0.9416666666666487</v>
       </c>
       <c r="BO3" t="n">
+        <v>45.92857142857142</v>
+      </c>
+      <c r="BP3" t="n">
+        <v>20571428.57142857</v>
+      </c>
+      <c r="BQ3" t="n">
         <v>104309.5238095238</v>
-      </c>
-      <c r="BP3" t="n">
-        <v>2.285714285714286</v>
-      </c>
-      <c r="BQ3" t="n">
-        <v>3.178571428571431</v>
       </c>
       <c r="BR3" t="n">
         <v>-2.078729950604952</v>
       </c>
       <c r="BS3" t="n">
-        <v>45.92857142857142</v>
+        <v>3.178571428571431</v>
       </c>
       <c r="BT3" t="n">
-        <v>-1224404.761904765</v>
+        <v>0.6515873015873015</v>
       </c>
       <c r="BU3" t="n">
-        <v>32.90476190476193</v>
+        <v>-0.6706349206349387</v>
       </c>
       <c r="BV3" t="n">
         <v>2.627179098313945</v>
       </c>
       <c r="BW3" t="n">
-        <v>-6718122.031477295</v>
+        <v>2.285714285714286</v>
       </c>
     </row>
     <row r="4">
@@ -1475,70 +1475,70 @@
         <v>0.04000000000000001</v>
       </c>
       <c r="BB4" t="n">
-        <v>-0.5068542568542576</v>
+        <v>-1.142857142857143</v>
       </c>
       <c r="BC4" t="n">
-        <v>0.4936147186147184</v>
+        <v>8010.533910533908</v>
       </c>
       <c r="BD4" t="n">
         <v>0.4169434625009885</v>
       </c>
       <c r="BE4" t="n">
+        <v>-0.5068542568542576</v>
+      </c>
+      <c r="BF4" t="n">
+        <v>4805863.558809757</v>
+      </c>
+      <c r="BG4" t="n">
+        <v>-88.00000000000003</v>
+      </c>
+      <c r="BH4" t="n">
+        <v>14491747.83549784</v>
+      </c>
+      <c r="BI4" t="n">
+        <v>0.3099442692063252</v>
+      </c>
+      <c r="BJ4" t="n">
+        <v>0.3743867243867385</v>
+      </c>
+      <c r="BK4" t="n">
+        <v>1.836741160498349</v>
+      </c>
+      <c r="BL4" t="n">
         <v>-4474.686089273979</v>
-      </c>
-      <c r="BF4" t="n">
-        <v>0.3099442692063252</v>
-      </c>
-      <c r="BG4" t="n">
-        <v>-4.154761904761898</v>
-      </c>
-      <c r="BH4" t="n">
-        <v>2.632936507936506</v>
-      </c>
-      <c r="BI4" t="n">
-        <v>8010.533910533908</v>
-      </c>
-      <c r="BJ4" t="n">
-        <v>-8960714.285714276</v>
-      </c>
-      <c r="BK4" t="n">
-        <v>0.3743867243867385</v>
-      </c>
-      <c r="BL4" t="n">
-        <v>-1.142857142857143</v>
       </c>
       <c r="BM4" t="n">
         <v>2.804401154401148</v>
       </c>
       <c r="BN4" t="n">
-        <v>1.836741160498349</v>
+        <v>2.632936507936506</v>
       </c>
       <c r="BO4" t="n">
+        <v>-90.99999999999997</v>
+      </c>
+      <c r="BP4" t="n">
+        <v>-8960714.285714276</v>
+      </c>
+      <c r="BQ4" t="n">
         <v>-96428.57142857142</v>
-      </c>
-      <c r="BP4" t="n">
-        <v>-1.714285714285714</v>
-      </c>
-      <c r="BQ4" t="n">
-        <v>-2.761904761904763</v>
       </c>
       <c r="BR4" t="n">
         <v>1.339901082403856</v>
       </c>
       <c r="BS4" t="n">
-        <v>-90.99999999999997</v>
+        <v>-2.761904761904763</v>
       </c>
       <c r="BT4" t="n">
-        <v>14491747.83549784</v>
+        <v>0.4936147186147184</v>
       </c>
       <c r="BU4" t="n">
-        <v>-88.00000000000003</v>
+        <v>-4.154761904761898</v>
       </c>
       <c r="BV4" t="n">
         <v>2.641442564671365</v>
       </c>
       <c r="BW4" t="n">
-        <v>4805863.558809757</v>
+        <v>-1.714285714285714</v>
       </c>
     </row>
     <row r="5">
@@ -1720,70 +1720,70 @@
         <v>0.1456043956043956</v>
       </c>
       <c r="BB5" t="n">
-        <v>1.010069444444444</v>
+        <v>0.3142857142857145</v>
       </c>
       <c r="BC5" t="n">
-        <v>0.03948412698412729</v>
+        <v>-17216.22023809523</v>
       </c>
       <c r="BD5" t="n">
         <v>0.2731710812980168</v>
       </c>
       <c r="BE5" t="n">
+        <v>1.010069444444444</v>
+      </c>
+      <c r="BF5" t="n">
+        <v>2325138.337277139</v>
+      </c>
+      <c r="BG5" t="n">
+        <v>25.88571428571427</v>
+      </c>
+      <c r="BH5" t="n">
+        <v>-6721845.238095235</v>
+      </c>
+      <c r="BI5" t="n">
+        <v>0.4038875598086122</v>
+      </c>
+      <c r="BJ5" t="n">
+        <v>0.3457341269841265</v>
+      </c>
+      <c r="BK5" t="n">
+        <v>1.560293118665129</v>
+      </c>
+      <c r="BL5" t="n">
         <v>-3820.494287560847</v>
-      </c>
-      <c r="BF5" t="n">
-        <v>0.4038875598086122</v>
-      </c>
-      <c r="BG5" t="n">
-        <v>4.92857142857136</v>
-      </c>
-      <c r="BH5" t="n">
-        <v>-0.8827380952380963</v>
-      </c>
-      <c r="BI5" t="n">
-        <v>-17216.22023809523</v>
-      </c>
-      <c r="BJ5" t="n">
-        <v>-6585714.285714287</v>
-      </c>
-      <c r="BK5" t="n">
-        <v>0.3457341269841265</v>
-      </c>
-      <c r="BL5" t="n">
-        <v>0.3142857142857145</v>
       </c>
       <c r="BM5" t="n">
         <v>-1.862847222222229</v>
       </c>
       <c r="BN5" t="n">
-        <v>1.560293118665129</v>
+        <v>-0.8827380952380963</v>
       </c>
       <c r="BO5" t="n">
+        <v>18.80000000000001</v>
+      </c>
+      <c r="BP5" t="n">
+        <v>-6585714.285714287</v>
+      </c>
+      <c r="BQ5" t="n">
         <v>-17428.57142857142</v>
-      </c>
-      <c r="BP5" t="n">
-        <v>1.457142857142857</v>
-      </c>
-      <c r="BQ5" t="n">
-        <v>-1.676190476190474</v>
       </c>
       <c r="BR5" t="n">
         <v>1.579924025254272</v>
       </c>
       <c r="BS5" t="n">
-        <v>18.80000000000001</v>
+        <v>-1.676190476190474</v>
       </c>
       <c r="BT5" t="n">
-        <v>-6721845.238095235</v>
+        <v>0.03948412698412729</v>
       </c>
       <c r="BU5" t="n">
-        <v>25.88571428571427</v>
+        <v>4.92857142857136</v>
       </c>
       <c r="BV5" t="n">
         <v>-3.233375203705435</v>
       </c>
       <c r="BW5" t="n">
-        <v>2325138.337277139</v>
+        <v>1.457142857142857</v>
       </c>
     </row>
     <row r="6">
@@ -1965,70 +1965,70 @@
         <v>0.2487179487179487</v>
       </c>
       <c r="BB6" t="n">
-        <v>-1.983238636363637</v>
+        <v>-2.571428571428572</v>
       </c>
       <c r="BC6" t="n">
-        <v>-0.1934027777777778</v>
+        <v>-104.4823232323251</v>
       </c>
       <c r="BD6" t="n">
         <v>-0.9744944831761124</v>
       </c>
       <c r="BE6" t="n">
+        <v>-1.983238636363637</v>
+      </c>
+      <c r="BF6" t="n">
+        <v>-2123322.052837274</v>
+      </c>
+      <c r="BG6" t="n">
+        <v>-207.5714285714286</v>
+      </c>
+      <c r="BH6" t="n">
+        <v>-4218774.463383839</v>
+      </c>
+      <c r="BI6" t="n">
+        <v>-0.1208626345752248</v>
+      </c>
+      <c r="BJ6" t="n">
+        <v>-0.7081123737373503</v>
+      </c>
+      <c r="BK6" t="n">
+        <v>-2.745085104953517</v>
+      </c>
+      <c r="BL6" t="n">
         <v>372.3722041059518</v>
-      </c>
-      <c r="BF6" t="n">
-        <v>-0.1208626345752248</v>
-      </c>
-      <c r="BG6" t="n">
-        <v>-0.4690476190476147</v>
-      </c>
-      <c r="BH6" t="n">
-        <v>-1.576893939393941</v>
-      </c>
-      <c r="BI6" t="n">
-        <v>-104.4823232323251</v>
-      </c>
-      <c r="BJ6" t="n">
-        <v>-29557142.85714285</v>
-      </c>
-      <c r="BK6" t="n">
-        <v>-0.7081123737373503</v>
-      </c>
-      <c r="BL6" t="n">
-        <v>-2.571428571428572</v>
       </c>
       <c r="BM6" t="n">
         <v>-3.258617424242431</v>
       </c>
       <c r="BN6" t="n">
-        <v>-2.745085104953517</v>
+        <v>-1.576893939393941</v>
       </c>
       <c r="BO6" t="n">
+        <v>-192</v>
+      </c>
+      <c r="BP6" t="n">
+        <v>-29557142.85714285</v>
+      </c>
+      <c r="BQ6" t="n">
         <v>-128714.2857142857</v>
-      </c>
-      <c r="BP6" t="n">
-        <v>-2.571428571428571</v>
-      </c>
-      <c r="BQ6" t="n">
-        <v>-0.4119047619047613</v>
       </c>
       <c r="BR6" t="n">
         <v>-1.07711345671872</v>
       </c>
       <c r="BS6" t="n">
-        <v>-192</v>
+        <v>-0.4119047619047613</v>
       </c>
       <c r="BT6" t="n">
-        <v>-4218774.463383839</v>
+        <v>-0.1934027777777778</v>
       </c>
       <c r="BU6" t="n">
-        <v>-207.5714285714286</v>
+        <v>-0.4690476190476147</v>
       </c>
       <c r="BV6" t="n">
         <v>-2.521097779069919</v>
       </c>
       <c r="BW6" t="n">
-        <v>-2123322.052837274</v>
+        <v>-2.571428571428571</v>
       </c>
     </row>
     <row r="7">
@@ -2212,70 +2212,70 @@
         <v>0.3180076628352491</v>
       </c>
       <c r="BB7" t="n">
-        <v>1.466806958473622</v>
+        <v>-0.7333333333333334</v>
       </c>
       <c r="BC7" t="n">
-        <v>1.641849046015713</v>
+        <v>68947.75533108869</v>
       </c>
       <c r="BD7" t="n">
         <v>2.012852196561305</v>
       </c>
       <c r="BE7" t="n">
+        <v>1.466806958473622</v>
+      </c>
+      <c r="BF7" t="n">
+        <v>24181974.71513396</v>
+      </c>
+      <c r="BG7" t="n">
+        <v>-48.90000000000001</v>
+      </c>
+      <c r="BH7" t="n">
+        <v>39534111.95286195</v>
+      </c>
+      <c r="BI7" t="n">
+        <v>0.98638083379805</v>
+      </c>
+      <c r="BJ7" t="n">
+        <v>0.9636363636363683</v>
+      </c>
+      <c r="BK7" t="n">
+        <v>6.715870565426769</v>
+      </c>
+      <c r="BL7" t="n">
         <v>44446.4179684078</v>
-      </c>
-      <c r="BF7" t="n">
-        <v>0.98638083379805</v>
-      </c>
-      <c r="BG7" t="n">
-        <v>-4.558333333333337</v>
-      </c>
-      <c r="BH7" t="n">
-        <v>5.390319865319867</v>
-      </c>
-      <c r="BI7" t="n">
-        <v>68947.75533108869</v>
-      </c>
-      <c r="BJ7" t="n">
-        <v>16916666.66666666</v>
-      </c>
-      <c r="BK7" t="n">
-        <v>0.9636363636363683</v>
-      </c>
-      <c r="BL7" t="n">
-        <v>-0.7333333333333334</v>
       </c>
       <c r="BM7" t="n">
         <v>8.77608024691358</v>
       </c>
       <c r="BN7" t="n">
-        <v>6.715870565426769</v>
+        <v>5.390319865319867</v>
       </c>
       <c r="BO7" t="n">
+        <v>-51.83333333333334</v>
+      </c>
+      <c r="BP7" t="n">
+        <v>16916666.66666666</v>
+      </c>
+      <c r="BQ7" t="n">
         <v>-64666.66666666666</v>
-      </c>
-      <c r="BP7" t="n">
-        <v>-0.8999999999999999</v>
-      </c>
-      <c r="BQ7" t="n">
-        <v>-8.558333333333334</v>
       </c>
       <c r="BR7" t="n">
         <v>2.767881593903766</v>
       </c>
       <c r="BS7" t="n">
-        <v>-51.83333333333334</v>
+        <v>-8.558333333333334</v>
       </c>
       <c r="BT7" t="n">
-        <v>39534111.95286195</v>
+        <v>1.641849046015713</v>
       </c>
       <c r="BU7" t="n">
-        <v>-48.90000000000001</v>
+        <v>-4.558333333333337</v>
       </c>
       <c r="BV7" t="n">
         <v>3.097383437547421</v>
       </c>
       <c r="BW7" t="n">
-        <v>24181974.71513396</v>
+        <v>-0.8999999999999999</v>
       </c>
     </row>
     <row r="8">
@@ -2457,70 +2457,70 @@
         <v>-0.07969639468690703</v>
       </c>
       <c r="BB8" t="n">
-        <v>-1.064141414141414</v>
+        <v>0</v>
       </c>
       <c r="BC8" t="n">
-        <v>-0.2912773569023566</v>
+        <v>1055.76950056116</v>
       </c>
       <c r="BD8" t="n">
         <v>-0.3959888828825875</v>
       </c>
       <c r="BE8" t="n">
+        <v>-1.064141414141414</v>
+      </c>
+      <c r="BF8" t="n">
+        <v>-2045736.700138145</v>
+      </c>
+      <c r="BG8" t="n">
+        <v>-7.571428571428584</v>
+      </c>
+      <c r="BH8" t="n">
+        <v>-1801114.267676767</v>
+      </c>
+      <c r="BI8" t="n">
+        <v>-0.2259199878781926</v>
+      </c>
+      <c r="BJ8" t="n">
+        <v>2.544605780022437</v>
+      </c>
+      <c r="BK8" t="n">
+        <v>-1.694921638245944</v>
+      </c>
+      <c r="BL8" t="n">
         <v>-1630.222376474958</v>
-      </c>
-      <c r="BF8" t="n">
-        <v>-0.2259199878781926</v>
-      </c>
-      <c r="BG8" t="n">
-        <v>-6.623809523809541</v>
-      </c>
-      <c r="BH8" t="n">
-        <v>-0.1052960157126819</v>
-      </c>
-      <c r="BI8" t="n">
-        <v>1055.76950056116</v>
-      </c>
-      <c r="BJ8" t="n">
-        <v>-3242857.142857143</v>
-      </c>
-      <c r="BK8" t="n">
-        <v>2.544605780022437</v>
-      </c>
-      <c r="BL8" t="n">
-        <v>0</v>
       </c>
       <c r="BM8" t="n">
         <v>-1.493676346801365</v>
       </c>
       <c r="BN8" t="n">
-        <v>-1.694921638245944</v>
+        <v>-0.1052960157126819</v>
       </c>
       <c r="BO8" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP8" t="n">
+        <v>-3242857.142857143</v>
+      </c>
+      <c r="BQ8" t="n">
         <v>-10000</v>
-      </c>
-      <c r="BP8" t="n">
-        <v>0.1428571428571428</v>
-      </c>
-      <c r="BQ8" t="n">
-        <v>2.414285714285718</v>
       </c>
       <c r="BR8" t="n">
         <v>-1.733541608651265</v>
       </c>
       <c r="BS8" t="n">
-        <v>0</v>
+        <v>2.414285714285718</v>
       </c>
       <c r="BT8" t="n">
-        <v>-1801114.267676767</v>
+        <v>-0.2912773569023566</v>
       </c>
       <c r="BU8" t="n">
-        <v>-7.571428571428584</v>
+        <v>-6.623809523809541</v>
       </c>
       <c r="BV8" t="n">
         <v>0.6372100594624044</v>
       </c>
       <c r="BW8" t="n">
-        <v>-2045736.700138145</v>
+        <v>0.1428571428571428</v>
       </c>
     </row>
     <row r="9">
@@ -2702,70 +2702,70 @@
         <v>-0.1937321937321937</v>
       </c>
       <c r="BB9" t="n">
-        <v>-1.023611111111109</v>
+        <v>-0.5952380952380951</v>
       </c>
       <c r="BC9" t="n">
-        <v>-2.100662878787879</v>
+        <v>-133452.8409090909</v>
       </c>
       <c r="BD9" t="n">
         <v>-1.208464455436204</v>
       </c>
       <c r="BE9" t="n">
+        <v>-1.023611111111109</v>
+      </c>
+      <c r="BF9" t="n">
+        <v>-29531666.41735672</v>
+      </c>
+      <c r="BG9" t="n">
+        <v>-64.21428571428572</v>
+      </c>
+      <c r="BH9" t="n">
+        <v>-47347440.02525252</v>
+      </c>
+      <c r="BI9" t="n">
+        <v>-1.45571243395837</v>
+      </c>
+      <c r="BJ9" t="n">
+        <v>0.2163825757575921</v>
+      </c>
+      <c r="BK9" t="n">
+        <v>-5.087123252564425</v>
+      </c>
+      <c r="BL9" t="n">
         <v>-90233.87781057094</v>
-      </c>
-      <c r="BF9" t="n">
-        <v>-1.45571243395837</v>
-      </c>
-      <c r="BG9" t="n">
-        <v>1.309523809523824</v>
-      </c>
-      <c r="BH9" t="n">
-        <v>-6.617803030303037</v>
-      </c>
-      <c r="BI9" t="n">
-        <v>-133452.8409090909</v>
-      </c>
-      <c r="BJ9" t="n">
-        <v>-65780952.38095239</v>
-      </c>
-      <c r="BK9" t="n">
-        <v>0.2163825757575921</v>
-      </c>
-      <c r="BL9" t="n">
-        <v>-0.5952380952380951</v>
       </c>
       <c r="BM9" t="n">
         <v>-7.642897727272725</v>
       </c>
       <c r="BN9" t="n">
-        <v>-5.087123252564425</v>
+        <v>-6.617803030303037</v>
       </c>
       <c r="BO9" t="n">
+        <v>-54.02380952380952</v>
+      </c>
+      <c r="BP9" t="n">
+        <v>-65780952.38095239</v>
+      </c>
+      <c r="BQ9" t="n">
         <v>-265261.9047619047</v>
-      </c>
-      <c r="BP9" t="n">
-        <v>-1.952380952380953</v>
-      </c>
-      <c r="BQ9" t="n">
-        <v>0.3650793650793638</v>
       </c>
       <c r="BR9" t="n">
         <v>-4.44165973452931</v>
       </c>
       <c r="BS9" t="n">
-        <v>-54.02380952380952</v>
+        <v>0.3650793650793638</v>
       </c>
       <c r="BT9" t="n">
-        <v>-47347440.02525252</v>
+        <v>-2.100662878787879</v>
       </c>
       <c r="BU9" t="n">
-        <v>-64.21428571428572</v>
+        <v>1.309523809523824</v>
       </c>
       <c r="BV9" t="n">
         <v>-0.005607545511765011</v>
       </c>
       <c r="BW9" t="n">
-        <v>-29531666.41735672</v>
+        <v>-1.952380952380953</v>
       </c>
     </row>
     <row r="10">
@@ -2947,70 +2947,70 @@
         <v>-0.1111111111111111</v>
       </c>
       <c r="BB10" t="n">
-        <v>-1.368827160493822</v>
+        <v>0.75</v>
       </c>
       <c r="BC10" t="n">
-        <v>-0.9660493827160495</v>
+        <v>-29043.20987654322</v>
       </c>
       <c r="BD10" t="n">
         <v>-3.076867413632119</v>
       </c>
       <c r="BE10" t="n">
+        <v>-1.368827160493822</v>
+      </c>
+      <c r="BF10" t="n">
+        <v>-5984904.554414356</v>
+      </c>
+      <c r="BG10" t="n">
+        <v>59.5</v>
+      </c>
+      <c r="BH10" t="n">
+        <v>-8683641.975308642</v>
+      </c>
+      <c r="BI10" t="n">
+        <v>-0.8157939101566549</v>
+      </c>
+      <c r="BJ10" t="n">
+        <v>0.6712962962963047</v>
+      </c>
+      <c r="BK10" t="n">
+        <v>-1.823410104782653</v>
+      </c>
+      <c r="BL10" t="n">
         <v>-23806.53983815747</v>
-      </c>
-      <c r="BF10" t="n">
-        <v>-0.8157939101566549</v>
-      </c>
-      <c r="BG10" t="n">
-        <v>9.5</v>
-      </c>
-      <c r="BH10" t="n">
-        <v>-1.763888888888886</v>
-      </c>
-      <c r="BI10" t="n">
-        <v>-29043.20987654322</v>
-      </c>
-      <c r="BJ10" t="n">
-        <v>5000000</v>
-      </c>
-      <c r="BK10" t="n">
-        <v>0.6712962962963047</v>
-      </c>
-      <c r="BL10" t="n">
-        <v>0.75</v>
       </c>
       <c r="BM10" t="n">
         <v>-2.566358024691368</v>
       </c>
       <c r="BN10" t="n">
-        <v>-1.823410104782653</v>
+        <v>-1.763888888888886</v>
       </c>
       <c r="BO10" t="n">
+        <v>57.75</v>
+      </c>
+      <c r="BP10" t="n">
+        <v>5000000</v>
+      </c>
+      <c r="BQ10" t="n">
         <v>21750</v>
-      </c>
-      <c r="BP10" t="n">
-        <v>1.25</v>
-      </c>
-      <c r="BQ10" t="n">
-        <v>-2.5</v>
       </c>
       <c r="BR10" t="n">
         <v>-1.00902972300031</v>
       </c>
       <c r="BS10" t="n">
-        <v>57.75</v>
+        <v>-2.5</v>
       </c>
       <c r="BT10" t="n">
-        <v>-8683641.975308642</v>
+        <v>-0.9660493827160495</v>
       </c>
       <c r="BU10" t="n">
-        <v>59.5</v>
+        <v>9.5</v>
       </c>
       <c r="BV10" t="n">
         <v>2.472766884531609</v>
       </c>
       <c r="BW10" t="n">
-        <v>-5984904.554414356</v>
+        <v>1.25</v>
       </c>
     </row>
     <row r="11">
@@ -3194,70 +3194,70 @@
         <v>0.01538461538461544</v>
       </c>
       <c r="BB11" t="n">
-        <v>1.749337121212125</v>
+        <v>-0.7142857142857144</v>
       </c>
       <c r="BC11" t="n">
-        <v>-0.8051136363636364</v>
+        <v>-38441.57196969702</v>
       </c>
       <c r="BD11" t="n">
         <v>2.207396567551523</v>
       </c>
       <c r="BE11" t="n">
+        <v>1.749337121212125</v>
+      </c>
+      <c r="BF11" t="n">
+        <v>-8854322.626496501</v>
+      </c>
+      <c r="BG11" t="n">
+        <v>-62.57142857142856</v>
+      </c>
+      <c r="BH11" t="n">
+        <v>-25762383.20707072</v>
+      </c>
+      <c r="BI11" t="n">
+        <v>-0.3900921356573057</v>
+      </c>
+      <c r="BJ11" t="n">
+        <v>4.185637626262604</v>
+      </c>
+      <c r="BK11" t="n">
+        <v>0.05811118861235798</v>
+      </c>
+      <c r="BL11" t="n">
         <v>-16577.33993743084</v>
-      </c>
-      <c r="BF11" t="n">
-        <v>-0.3900921356573057</v>
-      </c>
-      <c r="BG11" t="n">
-        <v>7.042857142857116</v>
-      </c>
-      <c r="BH11" t="n">
-        <v>-3.46622474747474</v>
-      </c>
-      <c r="BI11" t="n">
-        <v>-38441.57196969702</v>
-      </c>
-      <c r="BJ11" t="n">
-        <v>-117942857.1428571</v>
-      </c>
-      <c r="BK11" t="n">
-        <v>4.185637626262604</v>
-      </c>
-      <c r="BL11" t="n">
-        <v>-0.7142857142857144</v>
       </c>
       <c r="BM11" t="n">
         <v>-2.894917929292944</v>
       </c>
       <c r="BN11" t="n">
-        <v>0.05811118861235798</v>
+        <v>-3.46622474747474</v>
       </c>
       <c r="BO11" t="n">
+        <v>-73.57142857142861</v>
+      </c>
+      <c r="BP11" t="n">
+        <v>-117942857.1428571</v>
+      </c>
+      <c r="BQ11" t="n">
         <v>-289142.8571428572</v>
-      </c>
-      <c r="BP11" t="n">
-        <v>-2.857142857142856</v>
-      </c>
-      <c r="BQ11" t="n">
-        <v>-0.764285714285716</v>
       </c>
       <c r="BR11" t="n">
         <v>-2.812586605969017</v>
       </c>
       <c r="BS11" t="n">
-        <v>-73.57142857142861</v>
+        <v>-0.764285714285716</v>
       </c>
       <c r="BT11" t="n">
-        <v>-25762383.20707072</v>
+        <v>-0.8051136363636364</v>
       </c>
       <c r="BU11" t="n">
-        <v>-62.57142857142856</v>
+        <v>7.042857142857116</v>
       </c>
       <c r="BV11" t="n">
         <v>4.039937774789422</v>
       </c>
       <c r="BW11" t="n">
-        <v>-8854322.626496501</v>
+        <v>-2.857142857142856</v>
       </c>
     </row>
     <row r="12">
@@ -3439,70 +3439,70 @@
         <v>-0.08571428571428574</v>
       </c>
       <c r="BB12" t="n">
-        <v>-1.048074494949496</v>
+        <v>3.114285714285714</v>
       </c>
       <c r="BC12" t="n">
-        <v>0.09539141414141339</v>
+        <v>15746.11742424243</v>
       </c>
       <c r="BD12" t="n">
         <v>-0.8626630722919302</v>
       </c>
       <c r="BE12" t="n">
+        <v>-1.048074494949496</v>
+      </c>
+      <c r="BF12" t="n">
+        <v>-5967351.035930127</v>
+      </c>
+      <c r="BG12" t="n">
+        <v>251.4</v>
+      </c>
+      <c r="BH12" t="n">
+        <v>1889157.196969703</v>
+      </c>
+      <c r="BI12" t="n">
+        <v>0.007938363362419931</v>
+      </c>
+      <c r="BJ12" t="n">
+        <v>-1.934122474747454</v>
+      </c>
+      <c r="BK12" t="n">
+        <v>-2.708950640082634</v>
+      </c>
+      <c r="BL12" t="n">
         <v>7477.433353974411</v>
-      </c>
-      <c r="BF12" t="n">
-        <v>0.007938363362419931</v>
-      </c>
-      <c r="BG12" t="n">
-        <v>6.623809523809541</v>
-      </c>
-      <c r="BH12" t="n">
-        <v>-0.4660984848484873</v>
-      </c>
-      <c r="BI12" t="n">
-        <v>15746.11742424243</v>
-      </c>
-      <c r="BJ12" t="n">
-        <v>141557142.8571429</v>
-      </c>
-      <c r="BK12" t="n">
-        <v>-1.934122474747454</v>
-      </c>
-      <c r="BL12" t="n">
-        <v>3.114285714285714</v>
       </c>
       <c r="BM12" t="n">
         <v>-0.8125315656565562</v>
       </c>
       <c r="BN12" t="n">
-        <v>-2.708950640082634</v>
+        <v>-0.4660984848484873</v>
       </c>
       <c r="BO12" t="n">
+        <v>255.1428571428572</v>
+      </c>
+      <c r="BP12" t="n">
+        <v>141557142.8571429</v>
+      </c>
+      <c r="BQ12" t="n">
         <v>511285.7142857143</v>
-      </c>
-      <c r="BP12" t="n">
-        <v>8.114285714285714</v>
-      </c>
-      <c r="BQ12" t="n">
-        <v>2.821428571428573</v>
       </c>
       <c r="BR12" t="n">
         <v>-0.2967887816321735</v>
       </c>
       <c r="BS12" t="n">
-        <v>255.1428571428572</v>
+        <v>2.821428571428573</v>
       </c>
       <c r="BT12" t="n">
-        <v>1889157.196969703</v>
+        <v>0.09539141414141339</v>
       </c>
       <c r="BU12" t="n">
-        <v>251.4</v>
+        <v>6.623809523809541</v>
       </c>
       <c r="BV12" t="n">
         <v>-4.101489339464905</v>
       </c>
       <c r="BW12" t="n">
-        <v>-5967351.035930127</v>
+        <v>8.114285714285714</v>
       </c>
     </row>
     <row r="13">
@@ -3684,70 +3684,70 @@
         <v>-0.103448275862069</v>
       </c>
       <c r="BB13" t="n">
-        <v>1.748853615520279</v>
+        <v>-2</v>
       </c>
       <c r="BC13" t="n">
-        <v>-0.1827601410934747</v>
+        <v>-13596.07583774249</v>
       </c>
       <c r="BD13" t="n">
         <v>1.771054303131507</v>
       </c>
       <c r="BE13" t="n">
+        <v>1.748853615520279</v>
+      </c>
+      <c r="BF13" t="n">
+        <v>-5238032.335085034</v>
+      </c>
+      <c r="BG13" t="n">
+        <v>-164.0714285714286</v>
+      </c>
+      <c r="BH13" t="n">
+        <v>-10215911.59611993</v>
+      </c>
+      <c r="BI13" t="n">
+        <v>-0.001204716216971491</v>
+      </c>
+      <c r="BJ13" t="n">
+        <v>-0.817724867724877</v>
+      </c>
+      <c r="BK13" t="n">
+        <v>-0.0937068060842563</v>
+      </c>
+      <c r="BL13" t="n">
         <v>-8854.416739986598</v>
-      </c>
-      <c r="BF13" t="n">
-        <v>-0.001204716216971491</v>
-      </c>
-      <c r="BG13" t="n">
-        <v>0.8095238095238244</v>
-      </c>
-      <c r="BH13" t="n">
-        <v>-2.64166666666668</v>
-      </c>
-      <c r="BI13" t="n">
-        <v>-13596.07583774249</v>
-      </c>
-      <c r="BJ13" t="n">
-        <v>-32071428.57142857</v>
-      </c>
-      <c r="BK13" t="n">
-        <v>-0.817724867724877</v>
-      </c>
-      <c r="BL13" t="n">
-        <v>-2</v>
       </c>
       <c r="BM13" t="n">
         <v>-0.7894620811287467</v>
       </c>
       <c r="BN13" t="n">
-        <v>-0.0937068060842563</v>
+        <v>-2.64166666666668</v>
       </c>
       <c r="BO13" t="n">
+        <v>-154.9285714285714</v>
+      </c>
+      <c r="BP13" t="n">
+        <v>-32071428.57142857</v>
+      </c>
+      <c r="BQ13" t="n">
         <v>-148642.8571428571</v>
-      </c>
-      <c r="BP13" t="n">
-        <v>-2.785714285714286</v>
-      </c>
-      <c r="BQ13" t="n">
-        <v>4.654761904761902</v>
       </c>
       <c r="BR13" t="n">
         <v>-1.74980345770787</v>
       </c>
       <c r="BS13" t="n">
-        <v>-154.9285714285714</v>
+        <v>4.654761904761902</v>
       </c>
       <c r="BT13" t="n">
-        <v>-10215911.59611993</v>
+        <v>-0.1827601410934747</v>
       </c>
       <c r="BU13" t="n">
-        <v>-164.0714285714286</v>
+        <v>0.8095238095238244</v>
       </c>
       <c r="BV13" t="n">
         <v>-2.838416686118904</v>
       </c>
       <c r="BW13" t="n">
-        <v>-5238032.335085034</v>
+        <v>-2.785714285714286</v>
       </c>
     </row>
     <row r="14">
@@ -3929,70 +3929,70 @@
         <v>-0.08000000000000002</v>
       </c>
       <c r="BB14" t="n">
-        <v>0.1907242063492056</v>
+        <v>0.2571428571428571</v>
       </c>
       <c r="BC14" t="n">
-        <v>-1.310912698412699</v>
+        <v>-39270.28769841272</v>
       </c>
       <c r="BD14" t="n">
         <v>3.059057950563371</v>
       </c>
       <c r="BE14" t="n">
+        <v>0.1907242063492056</v>
+      </c>
+      <c r="BF14" t="n">
+        <v>-14349115.34565366</v>
+      </c>
+      <c r="BG14" t="n">
+        <v>10.25714285714287</v>
+      </c>
+      <c r="BH14" t="n">
+        <v>-20064702.38095239</v>
+      </c>
+      <c r="BI14" t="n">
+        <v>-0.8484971577270339</v>
+      </c>
+      <c r="BJ14" t="n">
+        <v>-1.816369047619048</v>
+      </c>
+      <c r="BK14" t="n">
+        <v>-3.635294510700845</v>
+      </c>
+      <c r="BL14" t="n">
         <v>-17653.40441722021</v>
-      </c>
-      <c r="BF14" t="n">
-        <v>-0.8484971577270339</v>
-      </c>
-      <c r="BG14" t="n">
-        <v>2.980952380952431</v>
-      </c>
-      <c r="BH14" t="n">
-        <v>-3.78710317460316</v>
-      </c>
-      <c r="BI14" t="n">
-        <v>-39270.28769841272</v>
-      </c>
-      <c r="BJ14" t="n">
-        <v>-32071428.57142857</v>
-      </c>
-      <c r="BK14" t="n">
-        <v>-1.816369047619048</v>
-      </c>
-      <c r="BL14" t="n">
-        <v>0.2571428571428571</v>
       </c>
       <c r="BM14" t="n">
         <v>-3.5923115079365</v>
       </c>
       <c r="BN14" t="n">
-        <v>-3.635294510700845</v>
+        <v>-3.78710317460316</v>
       </c>
       <c r="BO14" t="n">
+        <v>11.62857142857141</v>
+      </c>
+      <c r="BP14" t="n">
+        <v>-32071428.57142857</v>
+      </c>
+      <c r="BQ14" t="n">
         <v>-80000</v>
-      </c>
-      <c r="BP14" t="n">
-        <v>-3.028571428571429</v>
-      </c>
-      <c r="BQ14" t="n">
-        <v>1.438095238095237</v>
       </c>
       <c r="BR14" t="n">
         <v>-5.929309448291647</v>
       </c>
       <c r="BS14" t="n">
-        <v>11.62857142857141</v>
+        <v>1.438095238095237</v>
       </c>
       <c r="BT14" t="n">
-        <v>-20064702.38095239</v>
+        <v>-1.310912698412699</v>
       </c>
       <c r="BU14" t="n">
-        <v>10.25714285714287</v>
+        <v>2.980952380952431</v>
       </c>
       <c r="BV14" t="n">
         <v>-1.030773320246993</v>
       </c>
       <c r="BW14" t="n">
-        <v>-14349115.34565366</v>
+        <v>-3.028571428571429</v>
       </c>
     </row>
     <row r="15">
@@ -4172,70 +4172,70 @@
         <v>0.1803921568627451</v>
       </c>
       <c r="BB15" t="n">
-        <v>-4.251767676767678</v>
+        <v>-1.333333333333333</v>
       </c>
       <c r="BC15" t="n">
-        <v>-0.5969696969696967</v>
+        <v>-10538.63636363634</v>
       </c>
       <c r="BD15" t="n">
         <v>-2.862983501038201</v>
       </c>
       <c r="BE15" t="n">
+        <v>-4.251767676767678</v>
+      </c>
+      <c r="BF15" t="n">
+        <v>8303158.739372946</v>
+      </c>
+      <c r="BG15" t="n">
+        <v>-117.7619047619048</v>
+      </c>
+      <c r="BH15" t="n">
+        <v>5724015.151515156</v>
+      </c>
+      <c r="BI15" t="n">
+        <v>-0.06535335603318049</v>
+      </c>
+      <c r="BJ15" t="n">
+        <v>-2.842929292929313</v>
+      </c>
+      <c r="BK15" t="n">
+        <v>1.273205757138939</v>
+      </c>
+      <c r="BL15" t="n">
         <v>10732.3786975361</v>
-      </c>
-      <c r="BF15" t="n">
-        <v>-0.06535335603318049</v>
-      </c>
-      <c r="BG15" t="n">
-        <v>-7.705555555555549</v>
-      </c>
-      <c r="BH15" t="n">
-        <v>2.525252525252512</v>
-      </c>
-      <c r="BI15" t="n">
-        <v>-10538.63636363634</v>
-      </c>
-      <c r="BJ15" t="n">
-        <v>-58614285.71428572</v>
-      </c>
-      <c r="BK15" t="n">
-        <v>-2.842929292929313</v>
-      </c>
-      <c r="BL15" t="n">
-        <v>-1.333333333333333</v>
       </c>
       <c r="BM15" t="n">
         <v>-0.3332070707070613</v>
       </c>
       <c r="BN15" t="n">
-        <v>1.273205757138939</v>
+        <v>2.525252525252512</v>
       </c>
       <c r="BO15" t="n">
+        <v>-125.0714285714286</v>
+      </c>
+      <c r="BP15" t="n">
+        <v>-58614285.71428572</v>
+      </c>
+      <c r="BQ15" t="n">
         <v>-235309.5238095238</v>
-      </c>
-      <c r="BP15" t="n">
-        <v>-5.857142857142858</v>
-      </c>
-      <c r="BQ15" t="n">
-        <v>-3.290476190476188</v>
       </c>
       <c r="BR15" t="n">
         <v>3.160892107596169</v>
       </c>
       <c r="BS15" t="n">
-        <v>-125.0714285714286</v>
+        <v>-3.290476190476188</v>
       </c>
       <c r="BT15" t="n">
-        <v>5724015.151515156</v>
+        <v>-0.5969696969696967</v>
       </c>
       <c r="BU15" t="n">
-        <v>-117.7619047619048</v>
+        <v>-7.705555555555549</v>
       </c>
       <c r="BV15" t="n">
         <v>-1.601105665108463</v>
       </c>
       <c r="BW15" t="n">
-        <v>8303158.739372946</v>
+        <v>-5.857142857142858</v>
       </c>
     </row>
     <row r="16">
@@ -4417,70 +4417,70 @@
         <v>0.2426108374384237</v>
       </c>
       <c r="BB16" t="n">
-        <v>0.8196969696969667</v>
+        <v>3.314285714285715</v>
       </c>
       <c r="BC16" t="n">
-        <v>0.03749999999999942</v>
+        <v>-20026.76767676767</v>
       </c>
       <c r="BD16" t="n">
         <v>0.5078407182946805</v>
       </c>
       <c r="BE16" t="n">
+        <v>0.8196969696969667</v>
+      </c>
+      <c r="BF16" t="n">
+        <v>-1188360.583079893</v>
+      </c>
+      <c r="BG16" t="n">
+        <v>270.7428571428571</v>
+      </c>
+      <c r="BH16" t="n">
+        <v>67133.83838383853</v>
+      </c>
+      <c r="BI16" t="n">
+        <v>0.02244780061276264</v>
+      </c>
+      <c r="BJ16" t="n">
+        <v>-1.676262626262627</v>
+      </c>
+      <c r="BK16" t="n">
+        <v>-0.4932910081141131</v>
+      </c>
+      <c r="BL16" t="n">
         <v>-22676.14823053868</v>
-      </c>
-      <c r="BF16" t="n">
-        <v>0.02244780061276264</v>
-      </c>
-      <c r="BG16" t="n">
-        <v>-2.480952380952374</v>
-      </c>
-      <c r="BH16" t="n">
-        <v>0.3866161616161463</v>
-      </c>
-      <c r="BI16" t="n">
-        <v>-20026.76767676767</v>
-      </c>
-      <c r="BJ16" t="n">
-        <v>31453571.42857143</v>
-      </c>
-      <c r="BK16" t="n">
-        <v>-1.676262626262627</v>
-      </c>
-      <c r="BL16" t="n">
-        <v>3.314285714285715</v>
       </c>
       <c r="BM16" t="n">
         <v>-0.07992424242424079</v>
       </c>
       <c r="BN16" t="n">
-        <v>-0.4932910081141131</v>
+        <v>0.3866161616161463</v>
       </c>
       <c r="BO16" t="n">
+        <v>241.4571428571428</v>
+      </c>
+      <c r="BP16" t="n">
+        <v>31453571.42857143</v>
+      </c>
+      <c r="BQ16" t="n">
         <v>97771.42857142858</v>
-      </c>
-      <c r="BP16" t="n">
-        <v>3.457142857142857</v>
-      </c>
-      <c r="BQ16" t="n">
-        <v>-4.638095238095239</v>
       </c>
       <c r="BR16" t="n">
         <v>-0.438922406963755</v>
       </c>
       <c r="BS16" t="n">
-        <v>241.4571428571428</v>
+        <v>-4.638095238095239</v>
       </c>
       <c r="BT16" t="n">
-        <v>67133.83838383853</v>
+        <v>0.03749999999999942</v>
       </c>
       <c r="BU16" t="n">
-        <v>270.7428571428571</v>
+        <v>-2.480952380952374</v>
       </c>
       <c r="BV16" t="n">
         <v>0.01627725783734491</v>
       </c>
       <c r="BW16" t="n">
-        <v>-1188360.583079893</v>
+        <v>3.457142857142857</v>
       </c>
     </row>
     <row r="17">
@@ -4662,70 +4662,70 @@
         <v>0.1184615384615385</v>
       </c>
       <c r="BB17" t="n">
-        <v>0.6616161616161591</v>
+        <v>1.452380952380952</v>
       </c>
       <c r="BC17" t="n">
-        <v>1.085006313131313</v>
+        <v>53262.18434343436</v>
       </c>
       <c r="BD17" t="n">
         <v>-0.7134440615751174</v>
       </c>
       <c r="BE17" t="n">
+        <v>0.6616161616161591</v>
+      </c>
+      <c r="BF17" t="n">
+        <v>8303020.845184945</v>
+      </c>
+      <c r="BG17" t="n">
+        <v>121.6428571428572</v>
+      </c>
+      <c r="BH17" t="n">
+        <v>13946114.26767677</v>
+      </c>
+      <c r="BI17" t="n">
+        <v>0.4455430131191924</v>
+      </c>
+      <c r="BJ17" t="n">
+        <v>2.689551767676761</v>
+      </c>
+      <c r="BK17" t="n">
+        <v>1.293315098602022</v>
+      </c>
+      <c r="BL17" t="n">
         <v>34828.00433965105</v>
-      </c>
-      <c r="BF17" t="n">
-        <v>0.4455430131191924</v>
-      </c>
-      <c r="BG17" t="n">
-        <v>10.27380952380952</v>
-      </c>
-      <c r="BH17" t="n">
-        <v>2.591666666666654</v>
-      </c>
-      <c r="BI17" t="n">
-        <v>53262.18434343436</v>
-      </c>
-      <c r="BJ17" t="n">
-        <v>47598809.52380952</v>
-      </c>
-      <c r="BK17" t="n">
-        <v>2.689551767676761</v>
-      </c>
-      <c r="BL17" t="n">
-        <v>1.452380952380952</v>
       </c>
       <c r="BM17" t="n">
         <v>3.173327020202024</v>
       </c>
       <c r="BN17" t="n">
-        <v>1.293315098602022</v>
+        <v>2.591666666666654</v>
       </c>
       <c r="BO17" t="n">
+        <v>120.7380952380952</v>
+      </c>
+      <c r="BP17" t="n">
+        <v>47598809.52380952</v>
+      </c>
+      <c r="BQ17" t="n">
         <v>225261.9047619047</v>
-      </c>
-      <c r="BP17" t="n">
-        <v>2.80952380952381</v>
-      </c>
-      <c r="BQ17" t="n">
-        <v>2.13492063492064</v>
       </c>
       <c r="BR17" t="n">
         <v>2.223692717586999</v>
       </c>
       <c r="BS17" t="n">
-        <v>120.7380952380952</v>
+        <v>2.13492063492064</v>
       </c>
       <c r="BT17" t="n">
-        <v>13946114.26767677</v>
+        <v>1.085006313131313</v>
       </c>
       <c r="BU17" t="n">
-        <v>121.6428571428572</v>
+        <v>10.27380952380952</v>
       </c>
       <c r="BV17" t="n">
         <v>2.299188454636123</v>
       </c>
       <c r="BW17" t="n">
-        <v>8303020.845184945</v>
+        <v>2.80952380952381</v>
       </c>
     </row>
     <row r="18">
@@ -4909,70 +4909,70 @@
         <v>0.207843137254902</v>
       </c>
       <c r="BB18" t="n">
-        <v>0.23715277777778</v>
+        <v>0.2857142857142856</v>
       </c>
       <c r="BC18" t="n">
-        <v>1.976357323232323</v>
+        <v>136676.452020202</v>
       </c>
       <c r="BD18" t="n">
         <v>-0.2573657965653595</v>
       </c>
       <c r="BE18" t="n">
+        <v>0.23715277777778</v>
+      </c>
+      <c r="BF18" t="n">
+        <v>35001667.75822622</v>
+      </c>
+      <c r="BG18" t="n">
+        <v>41.14285714285714</v>
+      </c>
+      <c r="BH18" t="n">
+        <v>52238837.59469697</v>
+      </c>
+      <c r="BI18" t="n">
+        <v>1.425023325070087</v>
+      </c>
+      <c r="BJ18" t="n">
+        <v>-1.070549242424278</v>
+      </c>
+      <c r="BK18" t="n">
+        <v>8.711044916746673</v>
+      </c>
+      <c r="BL18" t="n">
         <v>97738.11561591813</v>
-      </c>
-      <c r="BF18" t="n">
-        <v>1.425023325070087</v>
-      </c>
-      <c r="BG18" t="n">
-        <v>-9.892857142857167</v>
-      </c>
-      <c r="BH18" t="n">
-        <v>9.102525252525268</v>
-      </c>
-      <c r="BI18" t="n">
-        <v>136676.452020202</v>
-      </c>
-      <c r="BJ18" t="n">
-        <v>78517857.14285715</v>
-      </c>
-      <c r="BK18" t="n">
-        <v>-1.070549242424278</v>
-      </c>
-      <c r="BL18" t="n">
-        <v>0.2857142857142856</v>
       </c>
       <c r="BM18" t="n">
         <v>10.68942550505051</v>
       </c>
       <c r="BN18" t="n">
-        <v>8.711044916746673</v>
+        <v>9.102525252525268</v>
       </c>
       <c r="BO18" t="n">
+        <v>41</v>
+      </c>
+      <c r="BP18" t="n">
+        <v>78517857.14285715</v>
+      </c>
+      <c r="BQ18" t="n">
         <v>305571.4285714286</v>
-      </c>
-      <c r="BP18" t="n">
-        <v>4</v>
-      </c>
-      <c r="BQ18" t="n">
-        <v>1.273809523809522</v>
       </c>
       <c r="BR18" t="n">
         <v>7.505565202794955</v>
       </c>
       <c r="BS18" t="n">
-        <v>41</v>
+        <v>1.273809523809522</v>
       </c>
       <c r="BT18" t="n">
-        <v>52238837.59469697</v>
+        <v>1.976357323232323</v>
       </c>
       <c r="BU18" t="n">
-        <v>41.14285714285714</v>
+        <v>-9.892857142857167</v>
       </c>
       <c r="BV18" t="n">
         <v>-1.01394424915614</v>
       </c>
       <c r="BW18" t="n">
-        <v>35001667.75822622</v>
+        <v>4</v>
       </c>
     </row>
     <row r="19">
@@ -5154,70 +5154,70 @@
         <v>0.1481481481481481</v>
       </c>
       <c r="BB19" t="n">
-        <v>-1.380190796857459</v>
+        <v>-0.3809523809523809</v>
       </c>
       <c r="BC19" t="n">
-        <v>0.001747635080968424</v>
+        <v>6721.653038319702</v>
       </c>
       <c r="BD19" t="n">
         <v>-4.384094657094053</v>
       </c>
       <c r="BE19" t="n">
+        <v>-1.380190796857459</v>
+      </c>
+      <c r="BF19" t="n">
+        <v>-233880.0772641692</v>
+      </c>
+      <c r="BG19" t="n">
+        <v>-26.78571428571428</v>
+      </c>
+      <c r="BH19" t="n">
+        <v>-2272014.18951419</v>
+      </c>
+      <c r="BI19" t="n">
+        <v>-0.07492073592490867</v>
+      </c>
+      <c r="BJ19" t="n">
+        <v>0.4674603174603078</v>
+      </c>
+      <c r="BK19" t="n">
+        <v>-2.310222852711178</v>
+      </c>
+      <c r="BL19" t="n">
         <v>1152.436041795314</v>
-      </c>
-      <c r="BF19" t="n">
-        <v>-0.07492073592490867</v>
-      </c>
-      <c r="BG19" t="n">
-        <v>-12.23690476190473</v>
-      </c>
-      <c r="BH19" t="n">
-        <v>0.2481000481000422</v>
-      </c>
-      <c r="BI19" t="n">
-        <v>6721.653038319702</v>
-      </c>
-      <c r="BJ19" t="n">
-        <v>22669047.61904762</v>
-      </c>
-      <c r="BK19" t="n">
-        <v>0.4674603174603078</v>
-      </c>
-      <c r="BL19" t="n">
-        <v>-0.3809523809523809</v>
       </c>
       <c r="BM19" t="n">
         <v>-1.678479236812578</v>
       </c>
       <c r="BN19" t="n">
-        <v>-2.310222852711178</v>
+        <v>0.2481000481000422</v>
       </c>
       <c r="BO19" t="n">
+        <v>-19.16666666666666</v>
+      </c>
+      <c r="BP19" t="n">
+        <v>22669047.61904762</v>
+      </c>
+      <c r="BQ19" t="n">
         <v>67095.23809523808</v>
-      </c>
-      <c r="BP19" t="n">
-        <v>0.6428571428571428</v>
-      </c>
-      <c r="BQ19" t="n">
-        <v>7.434523809523807</v>
       </c>
       <c r="BR19" t="n">
         <v>2.651224286993454</v>
       </c>
       <c r="BS19" t="n">
-        <v>-19.16666666666666</v>
+        <v>7.434523809523807</v>
       </c>
       <c r="BT19" t="n">
-        <v>-2272014.18951419</v>
+        <v>0.001747635080968424</v>
       </c>
       <c r="BU19" t="n">
-        <v>-26.78571428571428</v>
+        <v>-12.23690476190473</v>
       </c>
       <c r="BV19" t="n">
         <v>-0.1678158794818785</v>
       </c>
       <c r="BW19" t="n">
-        <v>-233880.0772641692</v>
+        <v>0.6428571428571428</v>
       </c>
     </row>
     <row r="20">
@@ -5399,70 +5399,70 @@
         <v>-0.1666666666666667</v>
       </c>
       <c r="BB20" t="n">
-        <v>-0.258080808080809</v>
+        <v>0.4285714285714284</v>
       </c>
       <c r="BC20" t="n">
-        <v>0.09242774971941659</v>
+        <v>10395.63341750843</v>
       </c>
       <c r="BD20" t="n">
         <v>-3.096589581251607</v>
       </c>
       <c r="BE20" t="n">
+        <v>-0.258080808080809</v>
+      </c>
+      <c r="BF20" t="n">
+        <v>2739792.765546765</v>
+      </c>
+      <c r="BG20" t="n">
+        <v>54.85714285714283</v>
+      </c>
+      <c r="BH20" t="n">
+        <v>4250891.905162739</v>
+      </c>
+      <c r="BI20" t="n">
+        <v>0.02220474934613237</v>
+      </c>
+      <c r="BJ20" t="n">
+        <v>0.8587051066217555</v>
+      </c>
+      <c r="BK20" t="n">
+        <v>-0.5578257667589526</v>
+      </c>
+      <c r="BL20" t="n">
         <v>2733.653953784255</v>
-      </c>
-      <c r="BF20" t="n">
-        <v>0.02220474934613237</v>
-      </c>
-      <c r="BG20" t="n">
-        <v>-3.576190476190504</v>
-      </c>
-      <c r="BH20" t="n">
-        <v>2.013348765432099</v>
-      </c>
-      <c r="BI20" t="n">
-        <v>10395.63341750843</v>
-      </c>
-      <c r="BJ20" t="n">
-        <v>32771428.57142857</v>
-      </c>
-      <c r="BK20" t="n">
-        <v>0.8587051066217555</v>
-      </c>
-      <c r="BL20" t="n">
-        <v>0.4285714285714284</v>
       </c>
       <c r="BM20" t="n">
         <v>1.391740319865349</v>
       </c>
       <c r="BN20" t="n">
-        <v>-0.5578257667589526</v>
+        <v>2.013348765432099</v>
       </c>
       <c r="BO20" t="n">
+        <v>51.28571428571428</v>
+      </c>
+      <c r="BP20" t="n">
+        <v>32771428.57142857</v>
+      </c>
+      <c r="BQ20" t="n">
         <v>111142.8571428571</v>
-      </c>
-      <c r="BP20" t="n">
-        <v>0.2857142857142856</v>
-      </c>
-      <c r="BQ20" t="n">
-        <v>-2.340476190476195</v>
       </c>
       <c r="BR20" t="n">
         <v>4.00913541342463</v>
       </c>
       <c r="BS20" t="n">
-        <v>51.28571428571428</v>
+        <v>-2.340476190476195</v>
       </c>
       <c r="BT20" t="n">
-        <v>4250891.905162739</v>
+        <v>0.09242774971941659</v>
       </c>
       <c r="BU20" t="n">
-        <v>54.85714285714283</v>
+        <v>-3.576190476190504</v>
       </c>
       <c r="BV20" t="n">
         <v>0.9192316985273692</v>
       </c>
       <c r="BW20" t="n">
-        <v>2739792.765546765</v>
+        <v>0.2857142857142856</v>
       </c>
     </row>
     <row r="21">
@@ -5644,70 +5644,70 @@
         <v>0.3903448275862069</v>
       </c>
       <c r="BB21" t="n">
-        <v>-0.08518518518518903</v>
+        <v>1.107142857142857</v>
       </c>
       <c r="BC21" t="n">
-        <v>0.03518518518518521</v>
+        <v>-14503.08641975308</v>
       </c>
       <c r="BD21" t="n">
         <v>1.387452222604445</v>
       </c>
       <c r="BE21" t="n">
+        <v>-0.08518518518518903</v>
+      </c>
+      <c r="BF21" t="n">
+        <v>-4069485.669511469</v>
+      </c>
+      <c r="BG21" t="n">
+        <v>74.57142857142858</v>
+      </c>
+      <c r="BH21" t="n">
+        <v>-4193680.555555556</v>
+      </c>
+      <c r="BI21" t="n">
+        <v>0.03574786639802108</v>
+      </c>
+      <c r="BJ21" t="n">
+        <v>-2.08456790123455</v>
+      </c>
+      <c r="BK21" t="n">
+        <v>-2.151239413894217</v>
+      </c>
+      <c r="BL21" t="n">
         <v>-10372.27498211761</v>
-      </c>
-      <c r="BF21" t="n">
-        <v>0.03574786639802108</v>
-      </c>
-      <c r="BG21" t="n">
-        <v>-2.190476190476176</v>
-      </c>
-      <c r="BH21" t="n">
-        <v>-0.9774691358024654</v>
-      </c>
-      <c r="BI21" t="n">
-        <v>-14503.08641975308</v>
-      </c>
-      <c r="BJ21" t="n">
-        <v>-9814285.714285715</v>
-      </c>
-      <c r="BK21" t="n">
-        <v>-2.08456790123455</v>
-      </c>
-      <c r="BL21" t="n">
-        <v>1.107142857142857</v>
       </c>
       <c r="BM21" t="n">
         <v>-1.532407407407391</v>
       </c>
       <c r="BN21" t="n">
-        <v>-2.151239413894217</v>
+        <v>-0.9774691358024654</v>
       </c>
       <c r="BO21" t="n">
+        <v>66.32142857142858</v>
+      </c>
+      <c r="BP21" t="n">
+        <v>-9814285.714285715</v>
+      </c>
+      <c r="BQ21" t="n">
         <v>321.4285714285652</v>
-      </c>
-      <c r="BP21" t="n">
-        <v>-0.8928571428571428</v>
-      </c>
-      <c r="BQ21" t="n">
-        <v>-2.321428571428573</v>
       </c>
       <c r="BR21" t="n">
         <v>-2.032185515531737</v>
       </c>
       <c r="BS21" t="n">
-        <v>66.32142857142858</v>
+        <v>-2.321428571428573</v>
       </c>
       <c r="BT21" t="n">
-        <v>-4193680.555555556</v>
+        <v>0.03518518518518521</v>
       </c>
       <c r="BU21" t="n">
-        <v>74.57142857142858</v>
+        <v>-2.190476190476176</v>
       </c>
       <c r="BV21" t="n">
         <v>-3.886774534375178</v>
       </c>
       <c r="BW21" t="n">
-        <v>-4069485.669511469</v>
+        <v>-0.8928571428571428</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualizo predicciones tras cambiar m_to_use de ligas
</commit_message>
<xml_diff>
--- a/data/england/p6_deployment/data_preparation/df_constructed.xlsx
+++ b/data/england/p6_deployment/data_preparation/df_constructed.xlsx
@@ -695,112 +695,112 @@
       </c>
       <c r="BB1" s="1" t="inlineStr">
         <is>
+          <t>dif_mean_hei_player_start</t>
+        </is>
+      </c>
+      <c r="BC1" s="1" t="inlineStr">
+        <is>
+          <t>dif_mean_wage_player_sub</t>
+        </is>
+      </c>
+      <c r="BD1" s="1" t="inlineStr">
+        <is>
+          <t>dif_n_player_miss</t>
+        </is>
+      </c>
+      <c r="BE1" s="1" t="inlineStr">
+        <is>
+          <t>dif_sum_rep_player_miss</t>
+        </is>
+      </c>
+      <c r="BF1" s="1" t="inlineStr">
+        <is>
+          <t>dif_mean_pot_player_sub</t>
+        </is>
+      </c>
+      <c r="BG1" s="1" t="inlineStr">
+        <is>
+          <t>dif_mean_rep_player_start</t>
+        </is>
+      </c>
+      <c r="BH1" s="1" t="inlineStr">
+        <is>
+          <t>dif_mean_wage_player_start</t>
+        </is>
+      </c>
+      <c r="BI1" s="1" t="inlineStr">
+        <is>
+          <t>dif_mean_age_player_sub</t>
+        </is>
+      </c>
+      <c r="BJ1" s="1" t="inlineStr">
+        <is>
+          <t>dif_mean_age_player_start</t>
+        </is>
+      </c>
+      <c r="BK1" s="1" t="inlineStr">
+        <is>
+          <t>dif_mean_rep_player_sub</t>
+        </is>
+      </c>
+      <c r="BL1" s="1" t="inlineStr">
+        <is>
+          <t>dif_mean_rat_player_sub</t>
+        </is>
+      </c>
+      <c r="BM1" s="1" t="inlineStr">
+        <is>
+          <t>dif_mean_rat_player_start</t>
+        </is>
+      </c>
+      <c r="BN1" s="1" t="inlineStr">
+        <is>
           <t>dif_mean_age_player_miss</t>
         </is>
       </c>
-      <c r="BC1" s="1" t="inlineStr">
-        <is>
-          <t>dif_mean_rep_player_start</t>
-        </is>
-      </c>
-      <c r="BD1" s="1" t="inlineStr">
+      <c r="BO1" s="1" t="inlineStr">
         <is>
           <t>dif_mean_value_player_start</t>
         </is>
       </c>
-      <c r="BE1" s="1" t="inlineStr">
-        <is>
-          <t>dif_mean_age_player_start</t>
-        </is>
-      </c>
-      <c r="BF1" s="1" t="inlineStr">
+      <c r="BP1" s="1" t="inlineStr">
+        <is>
+          <t>dif_sum_value_player_miss</t>
+        </is>
+      </c>
+      <c r="BQ1" s="1" t="inlineStr">
         <is>
           <t>dif_mean_hei_player_sub</t>
         </is>
       </c>
-      <c r="BG1" s="1" t="inlineStr">
-        <is>
-          <t>dif_mean_hei_player_start</t>
-        </is>
-      </c>
-      <c r="BH1" s="1" t="inlineStr">
+      <c r="BR1" s="1" t="inlineStr">
         <is>
           <t>dif_mean_value_player_sub</t>
         </is>
       </c>
-      <c r="BI1" s="1" t="inlineStr">
+      <c r="BS1" s="1" t="inlineStr">
+        <is>
+          <t>dif_sum_pot_player_miss</t>
+        </is>
+      </c>
+      <c r="BT1" s="1" t="inlineStr">
         <is>
           <t>dif_sum_wage_player_miss</t>
         </is>
       </c>
-      <c r="BJ1" s="1" t="inlineStr">
-        <is>
-          <t>dif_mean_rat_player_sub</t>
-        </is>
-      </c>
-      <c r="BK1" s="1" t="inlineStr">
-        <is>
-          <t>dif_sum_pot_player_miss</t>
-        </is>
-      </c>
-      <c r="BL1" s="1" t="inlineStr">
+      <c r="BU1" s="1" t="inlineStr">
         <is>
           <t>dif_mean_pot_player_start</t>
         </is>
       </c>
-      <c r="BM1" s="1" t="inlineStr">
-        <is>
-          <t>dif_n_player_miss</t>
-        </is>
-      </c>
-      <c r="BN1" s="1" t="inlineStr">
+      <c r="BV1" s="1" t="inlineStr">
+        <is>
+          <t>dif_mean_hei_player_miss</t>
+        </is>
+      </c>
+      <c r="BW1" s="1" t="inlineStr">
         <is>
           <t>dif_sum_rat_player_miss</t>
-        </is>
-      </c>
-      <c r="BO1" s="1" t="inlineStr">
-        <is>
-          <t>dif_mean_rat_player_start</t>
-        </is>
-      </c>
-      <c r="BP1" s="1" t="inlineStr">
-        <is>
-          <t>dif_mean_rep_player_sub</t>
-        </is>
-      </c>
-      <c r="BQ1" s="1" t="inlineStr">
-        <is>
-          <t>dif_sum_rep_player_miss</t>
-        </is>
-      </c>
-      <c r="BR1" s="1" t="inlineStr">
-        <is>
-          <t>dif_mean_hei_player_miss</t>
-        </is>
-      </c>
-      <c r="BS1" s="1" t="inlineStr">
-        <is>
-          <t>dif_mean_wage_player_start</t>
-        </is>
-      </c>
-      <c r="BT1" s="1" t="inlineStr">
-        <is>
-          <t>dif_mean_age_player_sub</t>
-        </is>
-      </c>
-      <c r="BU1" s="1" t="inlineStr">
-        <is>
-          <t>dif_mean_pot_player_sub</t>
-        </is>
-      </c>
-      <c r="BV1" s="1" t="inlineStr">
-        <is>
-          <t>dif_sum_value_player_miss</t>
-        </is>
-      </c>
-      <c r="BW1" s="1" t="inlineStr">
-        <is>
-          <t>dif_mean_wage_player_sub</t>
         </is>
       </c>
     </row>
@@ -985,70 +985,70 @@
         <v>-0.2142857142857142</v>
       </c>
       <c r="BB2" t="n">
+        <v>1.431790123456807</v>
+      </c>
+      <c r="BC2" t="n">
+        <v>-9153.224120357991</v>
+      </c>
+      <c r="BD2" t="n">
+        <v>-2.142857142857143</v>
+      </c>
+      <c r="BE2" t="n">
+        <v>-9</v>
+      </c>
+      <c r="BF2" t="n">
+        <v>0.05066659016888764</v>
+      </c>
+      <c r="BG2" t="n">
+        <v>-1.348765432098765</v>
+      </c>
+      <c r="BH2" t="n">
+        <v>-46786.11111111112</v>
+      </c>
+      <c r="BI2" t="n">
+        <v>-0.8057148296374095</v>
+      </c>
+      <c r="BJ2" t="n">
+        <v>-2.388580246913577</v>
+      </c>
+      <c r="BK2" t="n">
+        <v>-0.4757738246582641</v>
+      </c>
+      <c r="BL2" t="n">
+        <v>1.329471713062475</v>
+      </c>
+      <c r="BM2" t="n">
+        <v>-3.201543209876533</v>
+      </c>
+      <c r="BN2" t="n">
         <v>-4.161904761904761</v>
       </c>
-      <c r="BC2" t="n">
-        <v>-1.348765432098765</v>
-      </c>
-      <c r="BD2" t="n">
+      <c r="BO2" t="n">
         <v>-17247314.81481482</v>
       </c>
-      <c r="BE2" t="n">
-        <v>-2.388580246913577</v>
-      </c>
-      <c r="BF2" t="n">
+      <c r="BP2" t="n">
+        <v>-206485714.2857143</v>
+      </c>
+      <c r="BQ2" t="n">
         <v>2.604349775221294</v>
       </c>
-      <c r="BG2" t="n">
-        <v>1.431790123456807</v>
-      </c>
-      <c r="BH2" t="n">
+      <c r="BR2" t="n">
         <v>-682388.7709318697</v>
       </c>
-      <c r="BI2" t="n">
+      <c r="BS2" t="n">
+        <v>-190.1428571428571</v>
+      </c>
+      <c r="BT2" t="n">
         <v>-551000</v>
       </c>
-      <c r="BJ2" t="n">
-        <v>1.329471713062475</v>
-      </c>
-      <c r="BK2" t="n">
-        <v>-190.1428571428571</v>
-      </c>
-      <c r="BL2" t="n">
+      <c r="BU2" t="n">
         <v>-1.063580246913588</v>
       </c>
-      <c r="BM2" t="n">
-        <v>-2.142857142857143</v>
-      </c>
-      <c r="BN2" t="n">
+      <c r="BV2" t="n">
+        <v>1.035714285714278</v>
+      </c>
+      <c r="BW2" t="n">
         <v>-208.8571428571429</v>
-      </c>
-      <c r="BO2" t="n">
-        <v>-3.201543209876533</v>
-      </c>
-      <c r="BP2" t="n">
-        <v>-0.4757738246582641</v>
-      </c>
-      <c r="BQ2" t="n">
-        <v>-9</v>
-      </c>
-      <c r="BR2" t="n">
-        <v>1.035714285714278</v>
-      </c>
-      <c r="BS2" t="n">
-        <v>-46786.11111111112</v>
-      </c>
-      <c r="BT2" t="n">
-        <v>-0.8057148296374095</v>
-      </c>
-      <c r="BU2" t="n">
-        <v>0.05066659016888764</v>
-      </c>
-      <c r="BV2" t="n">
-        <v>-206485714.2857143</v>
-      </c>
-      <c r="BW2" t="n">
-        <v>-9153.224120357991</v>
       </c>
     </row>
     <row r="3">
@@ -1232,70 +1232,70 @@
         <v>-0.1666666666666667</v>
       </c>
       <c r="BB3" t="n">
+        <v>2.526014109347443</v>
+      </c>
+      <c r="BC3" t="n">
+        <v>37452.80463907915</v>
+      </c>
+      <c r="BD3" t="n">
+        <v>-0.1428571428571428</v>
+      </c>
+      <c r="BE3" t="n">
+        <v>2.714285714285714</v>
+      </c>
+      <c r="BF3" t="n">
+        <v>5.118640745601539</v>
+      </c>
+      <c r="BG3" t="n">
+        <v>1.10978835978836</v>
+      </c>
+      <c r="BH3" t="n">
+        <v>58309.78835978836</v>
+      </c>
+      <c r="BI3" t="n">
+        <v>-0.6646493031296963</v>
+      </c>
+      <c r="BJ3" t="n">
+        <v>-0.2311728395061721</v>
+      </c>
+      <c r="BK3" t="n">
+        <v>0.5904027345203813</v>
+      </c>
+      <c r="BL3" t="n">
+        <v>3.507388989006643</v>
+      </c>
+      <c r="BM3" t="n">
+        <v>5.101984126984121</v>
+      </c>
+      <c r="BN3" t="n">
         <v>0.2452380952380935</v>
       </c>
-      <c r="BC3" t="n">
-        <v>1.10978835978836</v>
-      </c>
-      <c r="BD3" t="n">
+      <c r="BO3" t="n">
         <v>24073206.5696649</v>
       </c>
-      <c r="BE3" t="n">
-        <v>-0.2311728395061721</v>
-      </c>
-      <c r="BF3" t="n">
+      <c r="BP3" t="n">
+        <v>35814285.71428572</v>
+      </c>
+      <c r="BQ3" t="n">
         <v>2.991407067877645</v>
       </c>
-      <c r="BG3" t="n">
-        <v>2.526014109347443</v>
-      </c>
-      <c r="BH3" t="n">
+      <c r="BR3" t="n">
         <v>13602414.12159917</v>
       </c>
-      <c r="BI3" t="n">
+      <c r="BS3" t="n">
+        <v>9.714285714285694</v>
+      </c>
+      <c r="BT3" t="n">
         <v>120714.2857142857</v>
       </c>
-      <c r="BJ3" t="n">
-        <v>3.507388989006643</v>
-      </c>
-      <c r="BK3" t="n">
-        <v>9.714285714285694</v>
-      </c>
-      <c r="BL3" t="n">
+      <c r="BU3" t="n">
         <v>5.425176366843033</v>
       </c>
-      <c r="BM3" t="n">
-        <v>-0.1428571428571428</v>
-      </c>
-      <c r="BN3" t="n">
+      <c r="BV3" t="n">
+        <v>-7.857142857142861</v>
+      </c>
+      <c r="BW3" t="n">
         <v>10.71428571428572</v>
-      </c>
-      <c r="BO3" t="n">
-        <v>5.101984126984121</v>
-      </c>
-      <c r="BP3" t="n">
-        <v>0.5904027345203813</v>
-      </c>
-      <c r="BQ3" t="n">
-        <v>2.714285714285714</v>
-      </c>
-      <c r="BR3" t="n">
-        <v>-7.857142857142861</v>
-      </c>
-      <c r="BS3" t="n">
-        <v>58309.78835978836</v>
-      </c>
-      <c r="BT3" t="n">
-        <v>-0.6646493031296963</v>
-      </c>
-      <c r="BU3" t="n">
-        <v>5.118640745601539</v>
-      </c>
-      <c r="BV3" t="n">
-        <v>35814285.71428572</v>
-      </c>
-      <c r="BW3" t="n">
-        <v>37452.80463907915</v>
       </c>
     </row>
     <row r="4">
@@ -1475,70 +1475,70 @@
         <v>-0.07119021134593995</v>
       </c>
       <c r="BB4" t="n">
+        <v>-3.631906365239701</v>
+      </c>
+      <c r="BC4" t="n">
+        <v>-35936.1565974827</v>
+      </c>
+      <c r="BD4" t="n">
+        <v>-1.857142857142857</v>
+      </c>
+      <c r="BE4" t="n">
+        <v>-4.142857142857143</v>
+      </c>
+      <c r="BF4" t="n">
+        <v>-1.778276703612107</v>
+      </c>
+      <c r="BG4" t="n">
+        <v>-1.249571107904442</v>
+      </c>
+      <c r="BH4" t="n">
+        <v>-50067.16370049702</v>
+      </c>
+      <c r="BI4" t="n">
+        <v>-0.9121887090282392</v>
+      </c>
+      <c r="BJ4" t="n">
+        <v>-0.2925525092191776</v>
+      </c>
+      <c r="BK4" t="n">
+        <v>-0.8193438541735754</v>
+      </c>
+      <c r="BL4" t="n">
+        <v>-1.494677145180248</v>
+      </c>
+      <c r="BM4" t="n">
+        <v>-3.409066859066854</v>
+      </c>
+      <c r="BN4" t="n">
         <v>0.3904761904761891</v>
       </c>
-      <c r="BC4" t="n">
-        <v>-1.249571107904442</v>
-      </c>
-      <c r="BD4" t="n">
+      <c r="BO4" t="n">
         <v>-15990384.09892576</v>
       </c>
-      <c r="BE4" t="n">
-        <v>-0.2925525092191776</v>
-      </c>
-      <c r="BF4" t="n">
+      <c r="BP4" t="n">
+        <v>-47375000</v>
+      </c>
+      <c r="BQ4" t="n">
         <v>-1.34206460464199</v>
       </c>
-      <c r="BG4" t="n">
-        <v>-3.631906365239701</v>
-      </c>
-      <c r="BH4" t="n">
+      <c r="BR4" t="n">
         <v>-9899809.703647742</v>
       </c>
-      <c r="BI4" t="n">
+      <c r="BS4" t="n">
+        <v>-153.7142857142857</v>
+      </c>
+      <c r="BT4" t="n">
         <v>-221285.7142857143</v>
       </c>
-      <c r="BJ4" t="n">
-        <v>-1.494677145180248</v>
-      </c>
-      <c r="BK4" t="n">
-        <v>-153.7142857142857</v>
-      </c>
-      <c r="BL4" t="n">
+      <c r="BU4" t="n">
         <v>-3.558124899791565</v>
       </c>
-      <c r="BM4" t="n">
-        <v>-1.857142857142857</v>
-      </c>
-      <c r="BN4" t="n">
+      <c r="BV4" t="n">
+        <v>-0.2738095238095468</v>
+      </c>
+      <c r="BW4" t="n">
         <v>-145.4285714285714</v>
-      </c>
-      <c r="BO4" t="n">
-        <v>-3.409066859066854</v>
-      </c>
-      <c r="BP4" t="n">
-        <v>-0.8193438541735754</v>
-      </c>
-      <c r="BQ4" t="n">
-        <v>-4.142857142857143</v>
-      </c>
-      <c r="BR4" t="n">
-        <v>-0.2738095238095468</v>
-      </c>
-      <c r="BS4" t="n">
-        <v>-50067.16370049702</v>
-      </c>
-      <c r="BT4" t="n">
-        <v>-0.9121887090282392</v>
-      </c>
-      <c r="BU4" t="n">
-        <v>-1.778276703612107</v>
-      </c>
-      <c r="BV4" t="n">
-        <v>-47375000</v>
-      </c>
-      <c r="BW4" t="n">
-        <v>-35936.1565974827</v>
       </c>
     </row>
     <row r="5">
@@ -1722,70 +1722,70 @@
         <v>-0.1242532855436081</v>
       </c>
       <c r="BB5" t="n">
+        <v>1.920472582972565</v>
+      </c>
+      <c r="BC5" t="n">
+        <v>43151.187135523</v>
+      </c>
+      <c r="BD5" t="n">
+        <v>-0.4285714285714288</v>
+      </c>
+      <c r="BE5" t="n">
+        <v>2.428571428571429</v>
+      </c>
+      <c r="BF5" t="n">
+        <v>7.531659597412201</v>
+      </c>
+      <c r="BG5" t="n">
+        <v>1.654076479076479</v>
+      </c>
+      <c r="BH5" t="n">
+        <v>63381.40331890332</v>
+      </c>
+      <c r="BI5" t="n">
+        <v>-1.660328101851029</v>
+      </c>
+      <c r="BJ5" t="n">
+        <v>-0.1507395382395345</v>
+      </c>
+      <c r="BK5" t="n">
+        <v>1.038260705391769</v>
+      </c>
+      <c r="BL5" t="n">
+        <v>6.504241120649795</v>
+      </c>
+      <c r="BM5" t="n">
+        <v>7.757575757575765</v>
+      </c>
+      <c r="BN5" t="n">
         <v>-3.285714285714285</v>
       </c>
-      <c r="BC5" t="n">
-        <v>1.654076479076479</v>
-      </c>
-      <c r="BD5" t="n">
+      <c r="BO5" t="n">
         <v>32189200.93795094</v>
       </c>
-      <c r="BE5" t="n">
-        <v>-0.1507395382395345</v>
-      </c>
-      <c r="BF5" t="n">
+      <c r="BP5" t="n">
+        <v>52928571.42857143</v>
+      </c>
+      <c r="BQ5" t="n">
         <v>3.459761418437495</v>
       </c>
-      <c r="BG5" t="n">
-        <v>1.920472582972565</v>
-      </c>
-      <c r="BH5" t="n">
+      <c r="BR5" t="n">
         <v>21480469.62569704</v>
       </c>
-      <c r="BI5" t="n">
+      <c r="BS5" t="n">
+        <v>-6.142857142857139</v>
+      </c>
+      <c r="BT5" t="n">
         <v>150142.8571428571</v>
       </c>
-      <c r="BJ5" t="n">
-        <v>6.504241120649795</v>
-      </c>
-      <c r="BK5" t="n">
-        <v>-6.142857142857139</v>
-      </c>
-      <c r="BL5" t="n">
+      <c r="BU5" t="n">
         <v>6.42938311688313</v>
       </c>
-      <c r="BM5" t="n">
-        <v>-0.4285714285714288</v>
-      </c>
-      <c r="BN5" t="n">
+      <c r="BV5" t="n">
+        <v>0.904761904761898</v>
+      </c>
+      <c r="BW5" t="n">
         <v>-13</v>
-      </c>
-      <c r="BO5" t="n">
-        <v>7.757575757575765</v>
-      </c>
-      <c r="BP5" t="n">
-        <v>1.038260705391769</v>
-      </c>
-      <c r="BQ5" t="n">
-        <v>2.428571428571429</v>
-      </c>
-      <c r="BR5" t="n">
-        <v>0.904761904761898</v>
-      </c>
-      <c r="BS5" t="n">
-        <v>63381.40331890332</v>
-      </c>
-      <c r="BT5" t="n">
-        <v>-1.660328101851029</v>
-      </c>
-      <c r="BU5" t="n">
-        <v>7.531659597412201</v>
-      </c>
-      <c r="BV5" t="n">
-        <v>52928571.42857143</v>
-      </c>
-      <c r="BW5" t="n">
-        <v>43151.187135523</v>
       </c>
     </row>
     <row r="6">
@@ -1969,70 +1969,70 @@
         <v>0.2</v>
       </c>
       <c r="BB6" t="n">
+        <v>0.466329966329937</v>
+      </c>
+      <c r="BC6" t="n">
+        <v>21663.84941547984</v>
+      </c>
+      <c r="BD6" t="n">
+        <v>-0.5714285714285716</v>
+      </c>
+      <c r="BE6" t="n">
+        <v>-0.2857142857142856</v>
+      </c>
+      <c r="BF6" t="n">
+        <v>2.584874626178973</v>
+      </c>
+      <c r="BG6" t="n">
+        <v>0.7109988776655438</v>
+      </c>
+      <c r="BH6" t="n">
+        <v>20683.05274971943</v>
+      </c>
+      <c r="BI6" t="n">
+        <v>1.491909258213607</v>
+      </c>
+      <c r="BJ6" t="n">
+        <v>0.441301907968576</v>
+      </c>
+      <c r="BK6" t="n">
+        <v>0.7432662546792983</v>
+      </c>
+      <c r="BL6" t="n">
+        <v>4.471333155572296</v>
+      </c>
+      <c r="BM6" t="n">
+        <v>3.550729517396178</v>
+      </c>
+      <c r="BN6" t="n">
         <v>-3.011904761904766</v>
       </c>
-      <c r="BC6" t="n">
-        <v>0.7109988776655438</v>
-      </c>
-      <c r="BD6" t="n">
+      <c r="BO6" t="n">
         <v>21437800.22446689</v>
       </c>
-      <c r="BE6" t="n">
-        <v>0.441301907968576</v>
-      </c>
-      <c r="BF6" t="n">
+      <c r="BP6" t="n">
+        <v>32039285.71428572</v>
+      </c>
+      <c r="BQ6" t="n">
         <v>1.664902911098551</v>
       </c>
-      <c r="BG6" t="n">
-        <v>0.466329966329937</v>
-      </c>
-      <c r="BH6" t="n">
+      <c r="BR6" t="n">
         <v>17220138.87581823</v>
       </c>
-      <c r="BI6" t="n">
+      <c r="BS6" t="n">
+        <v>-34.42857142857144</v>
+      </c>
+      <c r="BT6" t="n">
         <v>-59285.71428571429</v>
       </c>
-      <c r="BJ6" t="n">
-        <v>4.471333155572296</v>
-      </c>
-      <c r="BK6" t="n">
-        <v>-34.42857142857144</v>
-      </c>
-      <c r="BL6" t="n">
+      <c r="BU6" t="n">
         <v>3.113468013468037</v>
       </c>
-      <c r="BM6" t="n">
-        <v>-0.5714285714285716</v>
-      </c>
-      <c r="BN6" t="n">
+      <c r="BV6" t="n">
+        <v>-9.809523809523796</v>
+      </c>
+      <c r="BW6" t="n">
         <v>-39.14285714285714</v>
-      </c>
-      <c r="BO6" t="n">
-        <v>3.550729517396178</v>
-      </c>
-      <c r="BP6" t="n">
-        <v>0.7432662546792983</v>
-      </c>
-      <c r="BQ6" t="n">
-        <v>-0.2857142857142856</v>
-      </c>
-      <c r="BR6" t="n">
-        <v>-9.809523809523796</v>
-      </c>
-      <c r="BS6" t="n">
-        <v>20683.05274971943</v>
-      </c>
-      <c r="BT6" t="n">
-        <v>1.491909258213607</v>
-      </c>
-      <c r="BU6" t="n">
-        <v>2.584874626178973</v>
-      </c>
-      <c r="BV6" t="n">
-        <v>32039285.71428572</v>
-      </c>
-      <c r="BW6" t="n">
-        <v>21663.84941547984</v>
       </c>
     </row>
     <row r="7">
@@ -2214,70 +2214,70 @@
         <v>-0.2142857142857143</v>
       </c>
       <c r="BB7" t="n">
+        <v>2.461531986531952</v>
+      </c>
+      <c r="BC7" t="n">
+        <v>-75642.47911531196</v>
+      </c>
+      <c r="BD7" t="n">
+        <v>-0.4285714285714284</v>
+      </c>
+      <c r="BE7" t="n">
+        <v>-2.714285714285714</v>
+      </c>
+      <c r="BF7" t="n">
+        <v>-2.434903692798429</v>
+      </c>
+      <c r="BG7" t="n">
+        <v>-1.681144781144781</v>
+      </c>
+      <c r="BH7" t="n">
+        <v>-116616.694725028</v>
+      </c>
+      <c r="BI7" t="n">
+        <v>-2.038827903262884</v>
+      </c>
+      <c r="BJ7" t="n">
+        <v>-1.552890011223347</v>
+      </c>
+      <c r="BK7" t="n">
+        <v>-1.226097887320798</v>
+      </c>
+      <c r="BL7" t="n">
+        <v>-4.906481083416068</v>
+      </c>
+      <c r="BM7" t="n">
+        <v>-8.133389450056129</v>
+      </c>
+      <c r="BN7" t="n">
         <v>7.226190476190482</v>
       </c>
-      <c r="BC7" t="n">
-        <v>-1.681144781144781</v>
-      </c>
-      <c r="BD7" t="n">
+      <c r="BO7" t="n">
         <v>-46131181.25701459</v>
       </c>
-      <c r="BE7" t="n">
-        <v>-1.552890011223347</v>
-      </c>
-      <c r="BF7" t="n">
+      <c r="BP7" t="n">
+        <v>-46985714.28571428</v>
+      </c>
+      <c r="BQ7" t="n">
         <v>1.415799534143218</v>
       </c>
-      <c r="BG7" t="n">
-        <v>2.461531986531952</v>
-      </c>
-      <c r="BH7" t="n">
+      <c r="BR7" t="n">
         <v>-28510247.28539434</v>
       </c>
-      <c r="BI7" t="n">
+      <c r="BS7" t="n">
+        <v>-52.14285714285714</v>
+      </c>
+      <c r="BT7" t="n">
         <v>-202714.2857142857</v>
       </c>
-      <c r="BJ7" t="n">
-        <v>-4.906481083416068</v>
-      </c>
-      <c r="BK7" t="n">
-        <v>-52.14285714285714</v>
-      </c>
-      <c r="BL7" t="n">
+      <c r="BU7" t="n">
         <v>-4.991386083052745</v>
       </c>
-      <c r="BM7" t="n">
-        <v>-0.4285714285714284</v>
-      </c>
-      <c r="BN7" t="n">
+      <c r="BV7" t="n">
+        <v>2.554761904761961</v>
+      </c>
+      <c r="BW7" t="n">
         <v>-39.42857142857142</v>
-      </c>
-      <c r="BO7" t="n">
-        <v>-8.133389450056129</v>
-      </c>
-      <c r="BP7" t="n">
-        <v>-1.226097887320798</v>
-      </c>
-      <c r="BQ7" t="n">
-        <v>-2.714285714285714</v>
-      </c>
-      <c r="BR7" t="n">
-        <v>2.554761904761961</v>
-      </c>
-      <c r="BS7" t="n">
-        <v>-116616.694725028</v>
-      </c>
-      <c r="BT7" t="n">
-        <v>-2.038827903262884</v>
-      </c>
-      <c r="BU7" t="n">
-        <v>-2.434903692798429</v>
-      </c>
-      <c r="BV7" t="n">
-        <v>-46985714.28571428</v>
-      </c>
-      <c r="BW7" t="n">
-        <v>-75642.47911531196</v>
       </c>
     </row>
     <row r="8">
@@ -2459,70 +2459,70 @@
         <v>0.03703703703703703</v>
       </c>
       <c r="BB8" t="n">
+        <v>2.908100849767521</v>
+      </c>
+      <c r="BC8" t="n">
+        <v>-4548.762185185959</v>
+      </c>
+      <c r="BD8" t="n">
+        <v>1.285714285714286</v>
+      </c>
+      <c r="BE8" t="n">
+        <v>-0.3809523809523809</v>
+      </c>
+      <c r="BF8" t="n">
+        <v>0.4161102612230252</v>
+      </c>
+      <c r="BG8" t="n">
+        <v>0.02219416386083073</v>
+      </c>
+      <c r="BH8" t="n">
+        <v>4306.902356902348</v>
+      </c>
+      <c r="BI8" t="n">
+        <v>-1.764638618162135</v>
+      </c>
+      <c r="BJ8" t="n">
+        <v>0.04992784992785104</v>
+      </c>
+      <c r="BK8" t="n">
+        <v>-0.2100185794679381</v>
+      </c>
+      <c r="BL8" t="n">
+        <v>-3.853046640417631</v>
+      </c>
+      <c r="BM8" t="n">
+        <v>-0.8562169312169203</v>
+      </c>
+      <c r="BN8" t="n">
         <v>0.7801587301587318</v>
       </c>
-      <c r="BC8" t="n">
-        <v>0.02219416386083073</v>
-      </c>
-      <c r="BD8" t="n">
+      <c r="BO8" t="n">
         <v>-1123549.38271605</v>
       </c>
-      <c r="BE8" t="n">
-        <v>0.04992784992785104</v>
-      </c>
-      <c r="BF8" t="n">
+      <c r="BP8" t="n">
+        <v>17047619.04761905</v>
+      </c>
+      <c r="BQ8" t="n">
         <v>1.058509221515948</v>
       </c>
-      <c r="BG8" t="n">
-        <v>2.908100849767521</v>
-      </c>
-      <c r="BH8" t="n">
+      <c r="BR8" t="n">
         <v>-3208857.414709636</v>
       </c>
-      <c r="BI8" t="n">
+      <c r="BS8" t="n">
+        <v>99.19047619047618</v>
+      </c>
+      <c r="BT8" t="n">
         <v>98380.95238095238</v>
       </c>
-      <c r="BJ8" t="n">
-        <v>-3.853046640417631</v>
-      </c>
-      <c r="BK8" t="n">
-        <v>99.19047619047618</v>
-      </c>
-      <c r="BL8" t="n">
+      <c r="BU8" t="n">
         <v>0.4179573512906813</v>
       </c>
-      <c r="BM8" t="n">
-        <v>1.285714285714286</v>
-      </c>
-      <c r="BN8" t="n">
+      <c r="BV8" t="n">
+        <v>1.553968253968236</v>
+      </c>
+      <c r="BW8" t="n">
         <v>100.1904761904762</v>
-      </c>
-      <c r="BO8" t="n">
-        <v>-0.8562169312169203</v>
-      </c>
-      <c r="BP8" t="n">
-        <v>-0.2100185794679381</v>
-      </c>
-      <c r="BQ8" t="n">
-        <v>-0.3809523809523809</v>
-      </c>
-      <c r="BR8" t="n">
-        <v>1.553968253968236</v>
-      </c>
-      <c r="BS8" t="n">
-        <v>4306.902356902348</v>
-      </c>
-      <c r="BT8" t="n">
-        <v>-1.764638618162135</v>
-      </c>
-      <c r="BU8" t="n">
-        <v>0.4161102612230252</v>
-      </c>
-      <c r="BV8" t="n">
-        <v>17047619.04761905</v>
-      </c>
-      <c r="BW8" t="n">
-        <v>-4548.762185185959</v>
       </c>
     </row>
     <row r="9">
@@ -2704,70 +2704,70 @@
         <v>0.1114058355437666</v>
       </c>
       <c r="BB9" t="n">
+        <v>-1.645987654321004</v>
+      </c>
+      <c r="BC9" t="n">
+        <v>-2960.308476089813</v>
+      </c>
+      <c r="BD9" t="n">
+        <v>1.428571428571428</v>
+      </c>
+      <c r="BE9" t="n">
+        <v>1.571428571428572</v>
+      </c>
+      <c r="BF9" t="n">
+        <v>-1.408705421315915</v>
+      </c>
+      <c r="BG9" t="n">
+        <v>-0.1072530864197534</v>
+      </c>
+      <c r="BH9" t="n">
+        <v>4000</v>
+      </c>
+      <c r="BI9" t="n">
+        <v>1.523671908588845</v>
+      </c>
+      <c r="BJ9" t="n">
+        <v>-1.86759259259259</v>
+      </c>
+      <c r="BK9" t="n">
+        <v>-0.1709516090952017</v>
+      </c>
+      <c r="BL9" t="n">
+        <v>-0.3468278613674443</v>
+      </c>
+      <c r="BM9" t="n">
+        <v>1.716049382716037</v>
+      </c>
+      <c r="BN9" t="n">
         <v>-2.795238095238098</v>
       </c>
-      <c r="BC9" t="n">
-        <v>-0.1072530864197534</v>
-      </c>
-      <c r="BD9" t="n">
+      <c r="BO9" t="n">
         <v>8436805.555555556</v>
       </c>
-      <c r="BE9" t="n">
-        <v>-1.86759259259259</v>
-      </c>
-      <c r="BF9" t="n">
+      <c r="BP9" t="n">
+        <v>30514285.71428572</v>
+      </c>
+      <c r="BQ9" t="n">
         <v>0.1124926709178453</v>
       </c>
-      <c r="BG9" t="n">
-        <v>-1.645987654321004</v>
-      </c>
-      <c r="BH9" t="n">
+      <c r="BR9" t="n">
         <v>380603.5183481816</v>
       </c>
-      <c r="BI9" t="n">
+      <c r="BS9" t="n">
+        <v>119.8571428571428</v>
+      </c>
+      <c r="BT9" t="n">
         <v>77571.42857142857</v>
       </c>
-      <c r="BJ9" t="n">
-        <v>-0.3468278613674443</v>
-      </c>
-      <c r="BK9" t="n">
-        <v>119.8571428571428</v>
-      </c>
-      <c r="BL9" t="n">
+      <c r="BU9" t="n">
         <v>2.462808641975315</v>
       </c>
-      <c r="BM9" t="n">
-        <v>1.428571428571428</v>
-      </c>
-      <c r="BN9" t="n">
+      <c r="BV9" t="n">
+        <v>-2.214285714285694</v>
+      </c>
+      <c r="BW9" t="n">
         <v>111</v>
-      </c>
-      <c r="BO9" t="n">
-        <v>1.716049382716037</v>
-      </c>
-      <c r="BP9" t="n">
-        <v>-0.1709516090952017</v>
-      </c>
-      <c r="BQ9" t="n">
-        <v>1.571428571428572</v>
-      </c>
-      <c r="BR9" t="n">
-        <v>-2.214285714285694</v>
-      </c>
-      <c r="BS9" t="n">
-        <v>4000</v>
-      </c>
-      <c r="BT9" t="n">
-        <v>1.523671908588845</v>
-      </c>
-      <c r="BU9" t="n">
-        <v>-1.408705421315915</v>
-      </c>
-      <c r="BV9" t="n">
-        <v>30514285.71428572</v>
-      </c>
-      <c r="BW9" t="n">
-        <v>-2960.308476089813</v>
       </c>
     </row>
     <row r="10">
@@ -2949,70 +2949,70 @@
         <v>0.1481481481481481</v>
       </c>
       <c r="BB10" t="n">
+        <v>-0.02088744588749591</v>
+      </c>
+      <c r="BC10" t="n">
+        <v>36742.99356689063</v>
+      </c>
+      <c r="BD10" t="n">
+        <v>-3.238095238095238</v>
+      </c>
+      <c r="BE10" t="n">
+        <v>-1.047619047619048</v>
+      </c>
+      <c r="BF10" t="n">
+        <v>1.648014363087881</v>
+      </c>
+      <c r="BG10" t="n">
+        <v>0.7605248917748917</v>
+      </c>
+      <c r="BH10" t="n">
+        <v>37765.52128427129</v>
+      </c>
+      <c r="BI10" t="n">
+        <v>2.167549933726402</v>
+      </c>
+      <c r="BJ10" t="n">
+        <v>-0.5143578643578621</v>
+      </c>
+      <c r="BK10" t="n">
+        <v>0.679610656908451</v>
+      </c>
+      <c r="BL10" t="n">
+        <v>2.801101869943778</v>
+      </c>
+      <c r="BM10" t="n">
+        <v>2.823430735930728</v>
+      </c>
+      <c r="BN10" t="n">
         <v>1.552380952380954</v>
       </c>
-      <c r="BC10" t="n">
-        <v>0.7605248917748917</v>
-      </c>
-      <c r="BD10" t="n">
+      <c r="BO10" t="n">
         <v>9723471.320346322</v>
       </c>
-      <c r="BE10" t="n">
-        <v>-0.5143578643578621</v>
-      </c>
-      <c r="BF10" t="n">
+      <c r="BP10" t="n">
+        <v>11400000</v>
+      </c>
+      <c r="BQ10" t="n">
         <v>-3.176464446501171</v>
       </c>
-      <c r="BG10" t="n">
-        <v>-0.02088744588749591</v>
-      </c>
-      <c r="BH10" t="n">
+      <c r="BR10" t="n">
         <v>6252939.205402439</v>
       </c>
-      <c r="BI10" t="n">
+      <c r="BS10" t="n">
+        <v>-253.2380952380952</v>
+      </c>
+      <c r="BT10" t="n">
         <v>-65190.4761904762</v>
       </c>
-      <c r="BJ10" t="n">
-        <v>2.801101869943778</v>
-      </c>
-      <c r="BK10" t="n">
-        <v>-253.2380952380952</v>
-      </c>
-      <c r="BL10" t="n">
+      <c r="BU10" t="n">
         <v>2.167978896103904</v>
       </c>
-      <c r="BM10" t="n">
-        <v>-3.238095238095238</v>
-      </c>
-      <c r="BN10" t="n">
+      <c r="BV10" t="n">
+        <v>-3.885714285714272</v>
+      </c>
+      <c r="BW10" t="n">
         <v>-225.2857142857143</v>
-      </c>
-      <c r="BO10" t="n">
-        <v>2.823430735930728</v>
-      </c>
-      <c r="BP10" t="n">
-        <v>0.679610656908451</v>
-      </c>
-      <c r="BQ10" t="n">
-        <v>-1.047619047619048</v>
-      </c>
-      <c r="BR10" t="n">
-        <v>-3.885714285714272</v>
-      </c>
-      <c r="BS10" t="n">
-        <v>37765.52128427129</v>
-      </c>
-      <c r="BT10" t="n">
-        <v>2.167549933726402</v>
-      </c>
-      <c r="BU10" t="n">
-        <v>1.648014363087881</v>
-      </c>
-      <c r="BV10" t="n">
-        <v>11400000</v>
-      </c>
-      <c r="BW10" t="n">
-        <v>36742.99356689063</v>
       </c>
     </row>
     <row r="11">
@@ -3194,70 +3194,70 @@
         <v>0.07487684729064041</v>
       </c>
       <c r="BB11" t="n">
+        <v>2.524305555555571</v>
+      </c>
+      <c r="BC11" t="n">
+        <v>11802.30447752376</v>
+      </c>
+      <c r="BD11" t="n">
+        <v>1</v>
+      </c>
+      <c r="BE11" t="n">
+        <v>2.142857142857143</v>
+      </c>
+      <c r="BF11" t="n">
+        <v>2.675240895800101</v>
+      </c>
+      <c r="BG11" t="n">
+        <v>0.1440972222222223</v>
+      </c>
+      <c r="BH11" t="n">
+        <v>8112.847222222226</v>
+      </c>
+      <c r="BI11" t="n">
+        <v>0.9361258786697384</v>
+      </c>
+      <c r="BJ11" t="n">
+        <v>0.2534722222222179</v>
+      </c>
+      <c r="BK11" t="n">
+        <v>0.3434862144840212</v>
+      </c>
+      <c r="BL11" t="n">
+        <v>3.575933309705249</v>
+      </c>
+      <c r="BM11" t="n">
+        <v>3.447916666666671</v>
+      </c>
+      <c r="BN11" t="n">
         <v>0.5952380952380985</v>
       </c>
-      <c r="BC11" t="n">
-        <v>0.1440972222222223</v>
-      </c>
-      <c r="BD11" t="n">
+      <c r="BO11" t="n">
         <v>6861241.319444444</v>
       </c>
-      <c r="BE11" t="n">
-        <v>0.2534722222222179</v>
-      </c>
-      <c r="BF11" t="n">
+      <c r="BP11" t="n">
+        <v>16628571.42857143</v>
+      </c>
+      <c r="BQ11" t="n">
         <v>-1.656410597200079</v>
       </c>
-      <c r="BG11" t="n">
-        <v>2.524305555555571</v>
-      </c>
-      <c r="BH11" t="n">
+      <c r="BR11" t="n">
         <v>6051108.600626144</v>
       </c>
-      <c r="BI11" t="n">
+      <c r="BS11" t="n">
+        <v>81.14285714285714</v>
+      </c>
+      <c r="BT11" t="n">
         <v>91714.28571428571</v>
       </c>
-      <c r="BJ11" t="n">
-        <v>3.575933309705249</v>
-      </c>
-      <c r="BK11" t="n">
-        <v>81.14285714285714</v>
-      </c>
-      <c r="BL11" t="n">
+      <c r="BU11" t="n">
         <v>3.383680555555557</v>
       </c>
-      <c r="BM11" t="n">
-        <v>1</v>
-      </c>
-      <c r="BN11" t="n">
+      <c r="BV11" t="n">
+        <v>3.90952380952379</v>
+      </c>
+      <c r="BW11" t="n">
         <v>77.28571428571428</v>
-      </c>
-      <c r="BO11" t="n">
-        <v>3.447916666666671</v>
-      </c>
-      <c r="BP11" t="n">
-        <v>0.3434862144840212</v>
-      </c>
-      <c r="BQ11" t="n">
-        <v>2.142857142857143</v>
-      </c>
-      <c r="BR11" t="n">
-        <v>3.90952380952379</v>
-      </c>
-      <c r="BS11" t="n">
-        <v>8112.847222222226</v>
-      </c>
-      <c r="BT11" t="n">
-        <v>0.9361258786697384</v>
-      </c>
-      <c r="BU11" t="n">
-        <v>2.675240895800101</v>
-      </c>
-      <c r="BV11" t="n">
-        <v>16628571.42857143</v>
-      </c>
-      <c r="BW11" t="n">
-        <v>11802.30447752376</v>
       </c>
     </row>
   </sheetData>

</xml_diff>